<commit_message>
Cas test RCM2023-3 dans MV
</commit_message>
<xml_diff>
--- a/Manuel Validation/Cas tests références.xlsx
+++ b/Manuel Validation/Cas tests références.xlsx
@@ -15,64 +15,71 @@
     <sheet name="Cas 2" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_A" localSheetId="0">'Cas 2'!$B$29</definedName>
-    <definedName name="_A0" localSheetId="0">'Cas 2'!$B$72</definedName>
+    <definedName name="_A" localSheetId="0">'Cas 2'!$B$32</definedName>
+    <definedName name="_A0" localSheetId="0">'Cas 2'!$B$75</definedName>
     <definedName name="_Ace" localSheetId="0">'Cas 2'!$E$4</definedName>
-    <definedName name="_Acr" localSheetId="0">'Cas 2'!$B$68</definedName>
+    <definedName name="_Acr" localSheetId="0">'Cas 2'!$B$71</definedName>
     <definedName name="_As_inf" localSheetId="0">'Cas 2'!$E$10</definedName>
-    <definedName name="_Av" localSheetId="0">'Cas 2'!$B$30</definedName>
+    <definedName name="_Av" localSheetId="0">'Cas 2'!$B$33</definedName>
     <definedName name="_b" localSheetId="0">'Cas 2'!$B$4</definedName>
-    <definedName name="_B0" localSheetId="0">'Cas 2'!$B$73</definedName>
-    <definedName name="_bb" localSheetId="0">'Cas 2'!$E$20</definedName>
+    <definedName name="_B0" localSheetId="0">'Cas 2'!$B$76</definedName>
+    <definedName name="_bb" localSheetId="0">'Cas 2'!$E$21</definedName>
     <definedName name="_bc" localSheetId="0">'Cas 2'!$E$3</definedName>
-    <definedName name="_bm" localSheetId="0">'Cas 2'!$E$21</definedName>
-    <definedName name="_bp" localSheetId="0">'Cas 2'!$B$67</definedName>
-    <definedName name="_bt" localSheetId="0">'Cas 2'!$E$19</definedName>
-    <definedName name="_cf" localSheetId="0">'Cas 2'!$B$10</definedName>
-    <definedName name="_cw" localSheetId="0">'Cas 2'!$B$11</definedName>
-    <definedName name="_d" localSheetId="0">'Cas 2'!$H$12</definedName>
+    <definedName name="_bm" localSheetId="0">'Cas 2'!$E$22</definedName>
+    <definedName name="_bp" localSheetId="0">'Cas 2'!$B$70</definedName>
+    <definedName name="_bt" localSheetId="0">'Cas 2'!$E$20</definedName>
+    <definedName name="_cf" localSheetId="0">'Cas 2'!$B$11</definedName>
+    <definedName name="_cw" localSheetId="0">'Cas 2'!$B$12</definedName>
+    <definedName name="_d" localSheetId="0">'Cas 2'!$H$13</definedName>
+    <definedName name="_dw" localSheetId="0">'Cas 2'!$B$9</definedName>
     <definedName name="_Ecm_dalle" localSheetId="0">'Cas 2'!$H$8</definedName>
-    <definedName name="_ep" localSheetId="0">'Cas 2'!$E$18</definedName>
-    <definedName name="_epsilon" localSheetId="0">'Cas 2'!$B$14</definedName>
+    <definedName name="_ep" localSheetId="0">'Cas 2'!$E$19</definedName>
+    <definedName name="_epsilon" localSheetId="0">'Cas 2'!$B$15</definedName>
     <definedName name="_fck_dalle" localSheetId="0">'Cas 2'!$H$5</definedName>
     <definedName name="_fck_enrobage" localSheetId="0">'Cas 2'!$E$6</definedName>
     <definedName name="_fcm_dalle" localSheetId="0">'Cas 2'!$H$6</definedName>
     <definedName name="_fcm_enrobage" localSheetId="0">'Cas 2'!$E$7</definedName>
     <definedName name="_fctm_dalle" localSheetId="0">'Cas 2'!$H$7</definedName>
     <definedName name="_fctm_enrobage" localSheetId="0">'Cas 2'!$E$8</definedName>
-    <definedName name="_fusc" localSheetId="0">'Cas 2'!$H$13</definedName>
-    <definedName name="_fy" localSheetId="0">'Cas 2'!$B$13</definedName>
-    <definedName name="_fyp" localSheetId="0">'Cas 2'!$E$23</definedName>
+    <definedName name="_fusc" localSheetId="0">'Cas 2'!$H$14</definedName>
+    <definedName name="_fy" localSheetId="0">'Cas 2'!$B$14</definedName>
+    <definedName name="_fyd">'Cas 2'!$E$12</definedName>
+    <definedName name="_fyp" localSheetId="0">'Cas 2'!$E$24</definedName>
     <definedName name="_h" localSheetId="0">'Cas 2'!$B$3</definedName>
-    <definedName name="_hp" localSheetId="0">'Cas 2'!$E$16</definedName>
-    <definedName name="_hpg" localSheetId="0">'Cas 2'!$E$17</definedName>
-    <definedName name="_hsc" localSheetId="0">'Cas 2'!$H$11</definedName>
+    <definedName name="_hp" localSheetId="0">'Cas 2'!$E$17</definedName>
+    <definedName name="_hpg" localSheetId="0">'Cas 2'!$E$18</definedName>
+    <definedName name="_hsc" localSheetId="0">'Cas 2'!$H$12</definedName>
     <definedName name="_hw" localSheetId="0">'Cas 2'!$B$8</definedName>
-    <definedName name="_Iy" localSheetId="0">'Cas 2'!$B$31</definedName>
-    <definedName name="_Iz" localSheetId="0">'Cas 2'!$B$32</definedName>
-    <definedName name="_kr">'Cas 2'!$B$69</definedName>
+    <definedName name="_Iy" localSheetId="0">'Cas 2'!$B$34</definedName>
+    <definedName name="_Iz" localSheetId="0">'Cas 2'!$B$35</definedName>
+    <definedName name="_kr">'Cas 2'!$B$72</definedName>
     <definedName name="_L" localSheetId="0">'Cas 2'!$B$2</definedName>
-    <definedName name="_Mel_y_Rd" localSheetId="0">'Cas 2'!$B$50</definedName>
-    <definedName name="_Mel_z_Rd" localSheetId="0">'Cas 2'!$B$51</definedName>
-    <definedName name="_Mpl_y_Rd" localSheetId="0">'Cas 2'!$B$52</definedName>
-    <definedName name="_Mpl_z_Rd" localSheetId="0">'Cas 2'!$B$53</definedName>
-    <definedName name="_n" localSheetId="0">'Cas 2'!$B$66</definedName>
-    <definedName name="_NtRd" localSheetId="0">'Cas 2'!$B$48</definedName>
+    <definedName name="_Mel_y_Rd" localSheetId="0">'Cas 2'!$B$53</definedName>
+    <definedName name="_Mel_z_Rd" localSheetId="0">'Cas 2'!$B$54</definedName>
+    <definedName name="_Mpl_y_Rd" localSheetId="0">'Cas 2'!$B$55</definedName>
+    <definedName name="_Mpl_z_Rd" localSheetId="0">'Cas 2'!$B$56</definedName>
+    <definedName name="_n" localSheetId="0">'Cas 2'!$B$69</definedName>
+    <definedName name="_NtRd" localSheetId="0">'Cas 2'!$B$51</definedName>
+    <definedName name="_qBac" localSheetId="0">'Cas 2'!$E$26</definedName>
+    <definedName name="_qDalle" localSheetId="0">'Cas 2'!$H$10</definedName>
+    <definedName name="_qEnrobage" localSheetId="0">'Cas 2'!$E$13</definedName>
+    <definedName name="_qProfile" localSheetId="0">'Cas 2'!$B$18</definedName>
     <definedName name="_r" localSheetId="0">'Cas 2'!$B$7</definedName>
-    <definedName name="_rho" localSheetId="0">'Cas 2'!$B$16</definedName>
+    <definedName name="_rho" localSheetId="0">'Cas 2'!$B$17</definedName>
     <definedName name="_tc" localSheetId="0">'Cas 2'!$H$4</definedName>
     <definedName name="_td" localSheetId="0">'Cas 2'!$H$3</definedName>
     <definedName name="_tf" localSheetId="0">'Cas 2'!$B$5</definedName>
-    <definedName name="_tp" localSheetId="0">'Cas 2'!$E$22</definedName>
+    <definedName name="_tp" localSheetId="0">'Cas 2'!$E$23</definedName>
     <definedName name="_tw" localSheetId="0">'Cas 2'!$B$6</definedName>
-    <definedName name="_VplRd" localSheetId="0">'Cas 2'!$B$49</definedName>
-    <definedName name="_Wel_y" localSheetId="0">'Cas 2'!$B$33</definedName>
-    <definedName name="_Wel_z" localSheetId="0">'Cas 2'!$B$34</definedName>
-    <definedName name="_Wpl_y" localSheetId="0">'Cas 2'!$B$35</definedName>
-    <definedName name="_Wpl_z" localSheetId="0">'Cas 2'!$B$36</definedName>
-    <definedName name="_za" localSheetId="0">'Cas 2'!$B$71</definedName>
-    <definedName name="_zcr" localSheetId="0">'Cas 2'!$B$70</definedName>
-    <definedName name="_zel" localSheetId="0">'Cas 2'!$B$74</definedName>
+    <definedName name="_VplRd" localSheetId="0">'Cas 2'!$B$52</definedName>
+    <definedName name="_Wel_y" localSheetId="0">'Cas 2'!$B$36</definedName>
+    <definedName name="_Wel_z" localSheetId="0">'Cas 2'!$B$37</definedName>
+    <definedName name="_Wpl_y" localSheetId="0">'Cas 2'!$B$38</definedName>
+    <definedName name="_Wpl_z" localSheetId="0">'Cas 2'!$B$39</definedName>
+    <definedName name="_za" localSheetId="0">'Cas 2'!$B$74</definedName>
+    <definedName name="_zcr" localSheetId="0">'Cas 2'!$B$73</definedName>
+    <definedName name="_zel" localSheetId="0">'Cas 2'!$B$77</definedName>
+    <definedName name="_zpl" localSheetId="0">'Cas 2'!$B$102</definedName>
     <definedName name="_zs_inf" localSheetId="0">'Cas 2'!$E$11</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -85,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="152">
   <si>
     <t>h (mm)</t>
   </si>
@@ -370,6 +377,177 @@
   </si>
   <si>
     <t>Ih,y (cm4)</t>
+  </si>
+  <si>
+    <t>n0</t>
+  </si>
+  <si>
+    <t>psiL</t>
+  </si>
+  <si>
+    <t>Multiplicateur de fluage</t>
+  </si>
+  <si>
+    <t>CP</t>
+  </si>
+  <si>
+    <t>Retrait</t>
+  </si>
+  <si>
+    <t>RH</t>
+  </si>
+  <si>
+    <t>phi RH</t>
+  </si>
+  <si>
+    <t>beta(fcm)</t>
+  </si>
+  <si>
+    <t>t0 (j)</t>
+  </si>
+  <si>
+    <t>t (j)</t>
+  </si>
+  <si>
+    <t>beta (t0)</t>
+  </si>
+  <si>
+    <t>phi0</t>
+  </si>
+  <si>
+    <t>beta H</t>
+  </si>
+  <si>
+    <t>beta c(t,t0)</t>
+  </si>
+  <si>
+    <t>phi(t,t0)</t>
+  </si>
+  <si>
+    <t>nL</t>
+  </si>
+  <si>
+    <t>Propriétés plastiques</t>
+  </si>
+  <si>
+    <t>Nw (kN)</t>
+  </si>
+  <si>
+    <t>dw (mm)</t>
+  </si>
+  <si>
+    <t>Ns (kN)</t>
+  </si>
+  <si>
+    <t>fyd (MPa)</t>
+  </si>
+  <si>
+    <t>Ncw (kN)</t>
+  </si>
+  <si>
+    <t>Ncr (kN)</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>zpl (mm)</t>
+  </si>
+  <si>
+    <t>zpl,min (mm)</t>
+  </si>
+  <si>
+    <t>zpl,max (mm)</t>
+  </si>
+  <si>
+    <t>hc (mm)</t>
+  </si>
+  <si>
+    <t>Mpl,Rd (kN.m)</t>
+  </si>
+  <si>
+    <t>qProfilé (kN/ml)</t>
+  </si>
+  <si>
+    <t>qEnrobage</t>
+  </si>
+  <si>
+    <t>b (m)</t>
+  </si>
+  <si>
+    <t>mu (kg/m2)</t>
+  </si>
+  <si>
+    <t>qBac (kN/ml)</t>
+  </si>
+  <si>
+    <t>qDalle (kN/m)</t>
+  </si>
+  <si>
+    <t>qPP (kN/ml)</t>
+  </si>
+  <si>
+    <t>M(G1) (kN.m)</t>
+  </si>
+  <si>
+    <t>V(G1) (kN)</t>
+  </si>
+  <si>
+    <t>Analyse</t>
+  </si>
+  <si>
+    <t>Vérification</t>
+  </si>
+  <si>
+    <t>V(Qc) (kN)</t>
+  </si>
+  <si>
+    <t>M (Qc) (kN.m)</t>
+  </si>
+  <si>
+    <t>V(ELS) (kN)</t>
+  </si>
+  <si>
+    <t>M(ELS) (kN.m)</t>
+  </si>
+  <si>
+    <t>V(ELU) (kN)</t>
+  </si>
+  <si>
+    <t>M (ELU) (kN.m)</t>
+  </si>
+  <si>
+    <t>Critere M</t>
+  </si>
+  <si>
+    <t>Critere V</t>
+  </si>
+  <si>
+    <t>f(G1) (mm)</t>
+  </si>
+  <si>
+    <t>f (Qc)</t>
+  </si>
+  <si>
+    <t>Calcul sur RDM7</t>
+  </si>
+  <si>
+    <t>f (ELS) (mm)</t>
+  </si>
+  <si>
+    <t>f (G+0,2Q) (mm)</t>
+  </si>
+  <si>
+    <t>f (Hz)</t>
+  </si>
+  <si>
+    <t>MbRd (kN.m)</t>
+  </si>
+  <si>
+    <t>Critere LT</t>
+  </si>
+  <si>
+    <t>Valeur issue de l'article RCM 2023 n°3</t>
   </si>
 </sst>
 </file>
@@ -381,7 +559,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="170" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -428,7 +606,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -528,12 +706,34 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -564,6 +764,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -576,10 +780,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -861,30 +1067,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="28"/>
+    <col min="3" max="3" width="11.42578125" style="24"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="25"/>
+      <c r="B1" s="29"/>
       <c r="C1"/>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="25"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="24" t="s">
+      <c r="E1" s="29"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="25"/>
+      <c r="H1" s="29"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -943,7 +1151,7 @@
       </c>
       <c r="E4">
         <f>_b*_h/100-_A-(_b-_bc)*_hw/100</f>
-        <v>892.5</v>
+        <v>892.7</v>
       </c>
       <c r="G4" t="s">
         <v>76</v>
@@ -966,7 +1174,7 @@
       </c>
       <c r="E5" s="23">
         <f>_Ace*100/_hw</f>
-        <v>190.7051282051282</v>
+        <v>190.74786324786325</v>
       </c>
       <c r="G5" t="s">
         <v>62</v>
@@ -1015,7 +1223,7 @@
       <c r="G7" t="s">
         <v>63</v>
       </c>
-      <c r="H7" s="30">
+      <c r="H7" s="26">
         <f>0.3*_fck_enrobage^(2/3)</f>
         <v>2.5649639200150443</v>
       </c>
@@ -1032,53 +1240,66 @@
       <c r="D8" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="30">
+      <c r="E8" s="26">
         <f>0.3*_fck_enrobage^(2/3)</f>
         <v>2.5649639200150443</v>
       </c>
       <c r="G8" t="s">
         <v>64</v>
       </c>
-      <c r="H8" s="30">
+      <c r="H8" s="26">
         <f>22*(_fcm_enrobage/10)^0.3*1000</f>
         <v>31475.806210019346</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="6"/>
+      <c r="A9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B9" s="6">
+        <f>_hw-2*_r</f>
+        <v>426</v>
+      </c>
       <c r="C9"/>
       <c r="D9" t="s">
         <v>64</v>
       </c>
-      <c r="E9" s="30">
+      <c r="E9" s="26">
         <f>22*(_fcm_enrobage/10)^0.3*1000</f>
         <v>31475.806210019346</v>
       </c>
+      <c r="G9" t="s">
+        <v>126</v>
+      </c>
+      <c r="H9">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="6">
-        <f>(_b-2*_r-_tw)/2</f>
-        <v>74.8</v>
-      </c>
+      <c r="B10" s="6"/>
       <c r="C10"/>
       <c r="D10" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="31">
+      <c r="E10" s="27">
         <f>PI()*(12^2+8^2)/4*2/100</f>
         <v>3.267256359733385</v>
       </c>
+      <c r="G10" t="s">
+        <v>129</v>
+      </c>
+      <c r="H10" s="26">
+        <f>(_tc+_hp*_bm/_ep)/1000*H9*2500*9.81/1000</f>
+        <v>6.4277418478260868</v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B11" s="6">
-        <f>_hw-2*_r</f>
-        <v>426</v>
+        <f>(_b-2*_r-_tw)/2</f>
+        <v>74.8</v>
       </c>
       <c r="C11"/>
       <c r="D11" t="s">
@@ -1089,871 +1310,1340 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="6">
+        <f>_hw-2*_r</f>
+        <v>426</v>
+      </c>
       <c r="C12"/>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>8</v>
-      </c>
-      <c r="B13" s="1">
-        <v>355</v>
-      </c>
+      <c r="D12" t="s">
+        <v>115</v>
+      </c>
+      <c r="E12" s="23">
+        <f>500/1.15</f>
+        <v>434.78260869565219</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C13"/>
+      <c r="D13" t="s">
+        <v>125</v>
+      </c>
+      <c r="E13" s="26">
+        <f>_Ace*10^(-4)*2500*9.81/1000</f>
+        <v>2.1893467500000003</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="1">
+        <v>355</v>
+      </c>
+      <c r="C14"/>
+    </row>
+    <row r="15" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="14">
+      <c r="B15" s="14">
         <f>SQRT(235/_fy)</f>
         <v>0.81361651346682706</v>
       </c>
-      <c r="C14"/>
-      <c r="D14" s="24" t="s">
+      <c r="C15"/>
+      <c r="D15" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="E14" s="25"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="6"/>
-      <c r="C15"/>
-      <c r="D15" t="s">
-        <v>67</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>68</v>
-      </c>
+      <c r="E15" s="29"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="1">
-        <v>7850</v>
-      </c>
+      <c r="B16" s="6"/>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>69</v>
-      </c>
-      <c r="E16" s="1">
-        <v>58</v>
+        <v>67</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B17" s="6"/>
+      <c r="A17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="1">
+        <v>7850</v>
+      </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E17" s="1">
         <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B18" s="6"/>
+      <c r="A18" t="s">
+        <v>124</v>
+      </c>
+      <c r="B18" s="35">
+        <f>_rho*_A*10^(-4)*9.81/1000</f>
+        <v>0.78009610500000004</v>
+      </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E18" s="1">
-        <v>207</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B19" s="6"/>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E19" s="1">
-        <v>101</v>
+        <v>207</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B20" s="6"/>
       <c r="C20"/>
       <c r="D20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E20" s="1">
-        <v>62</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B21" s="6"/>
       <c r="C21"/>
       <c r="D21" t="s">
-        <v>78</v>
-      </c>
-      <c r="E21">
-        <f>(E19+E20)/2</f>
-        <v>81.5</v>
+        <v>73</v>
+      </c>
+      <c r="E21" s="1">
+        <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B22" s="6"/>
       <c r="C22"/>
       <c r="D22" t="s">
-        <v>74</v>
-      </c>
-      <c r="E22" s="1">
-        <v>1</v>
+        <v>78</v>
+      </c>
+      <c r="E22">
+        <f>(E20+E21)/2</f>
+        <v>81.5</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B23" s="6"/>
       <c r="C23"/>
       <c r="D23" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E23" s="1">
-        <v>350</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B24" s="6"/>
       <c r="C24"/>
+      <c r="D24" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" s="1">
+        <v>350</v>
+      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="6"/>
+      <c r="C25"/>
+      <c r="D25" t="s">
+        <v>127</v>
+      </c>
+      <c r="E25" s="1">
+        <v>11.37</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="6"/>
+      <c r="C26"/>
+      <c r="D26" t="s">
+        <v>128</v>
+      </c>
+      <c r="E26" s="25">
+        <f>E25*H9*9.81/1000</f>
+        <v>0.27884924999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="6"/>
+      <c r="C27"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C25"/>
-    </row>
-    <row r="26" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C26"/>
-    </row>
-    <row r="27" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="24" t="s">
+      <c r="C28"/>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C29"/>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B27" s="25"/>
-      <c r="C27" s="28" t="s">
+      <c r="B30" s="29"/>
+      <c r="C30" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D30" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B31" s="8">
         <f>(2*(_h-2*_r)+2*_b+2*(_b-2*_r-_tw)+2*PI()*_r)/10</f>
         <v>174.11468914507714</v>
       </c>
-      <c r="D28" t="str">
-        <f>IF(C28&lt;&gt;"",(B28/C28-1)*100,"")</f>
+      <c r="D31" t="str">
+        <f>IF(C31&lt;&gt;"",(B31/C31-1)*100,"")</f>
         <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>5</v>
-      </c>
-      <c r="B29" s="4">
-        <v>101.5</v>
-      </c>
-      <c r="C29" s="28">
-        <v>101.1</v>
-      </c>
-      <c r="D29" s="30">
-        <f t="shared" ref="D29:D64" si="0">IF(C29&lt;&gt;"",(B29/C29-1)*100,"")</f>
-        <v>0.39564787339267937</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>6</v>
-      </c>
-      <c r="B30" s="5">
-        <f>B29-2*_b*_tf/100+2*(_tw+2*_r)*_tf/2/100</f>
-        <v>50.808</v>
-      </c>
-      <c r="C30" s="28">
-        <v>50.4</v>
-      </c>
-      <c r="D30" s="30">
-        <f t="shared" si="0"/>
-        <v>0.80952380952381553</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>9</v>
-      </c>
-      <c r="B31" s="4">
-        <v>43014.311000000002</v>
-      </c>
-      <c r="C31" s="28">
-        <v>42933</v>
-      </c>
-      <c r="D31" s="30">
-        <f t="shared" si="0"/>
-        <v>0.18939044557799711</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B32" s="4">
-        <v>1939.511</v>
-      </c>
-      <c r="C32" s="28">
-        <v>1936</v>
-      </c>
-      <c r="D32" s="30">
-        <f t="shared" si="0"/>
-        <v>0.18135330578512576</v>
+        <v>101.3</v>
+      </c>
+      <c r="C32" s="24">
+        <v>101.1</v>
+      </c>
+      <c r="D32" s="26">
+        <f t="shared" ref="D32:D67" si="0">IF(C32&lt;&gt;"",(B32/C32-1)*100,"")</f>
+        <v>0.19782393669633969</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B33" s="5">
-        <f>B31/(_h/2/10)</f>
-        <v>1730.9581891348089</v>
-      </c>
-      <c r="C33" s="28">
-        <v>1728</v>
-      </c>
-      <c r="D33" s="30">
-        <f t="shared" si="0"/>
-        <v>0.17119150085700419</v>
+        <f>B32-2*_b*_tf/100+2*(_tw+2*_r)*_tf/2/100</f>
+        <v>50.607999999999997</v>
+      </c>
+      <c r="C33" s="24">
+        <v>50.4</v>
+      </c>
+      <c r="D33" s="26">
+        <f t="shared" si="0"/>
+        <v>0.41269841269842011</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>13</v>
-      </c>
-      <c r="B34" s="5">
-        <f>B32/(_b/2/10)</f>
-        <v>193.9511</v>
-      </c>
-      <c r="C34" s="28">
-        <v>193.6</v>
-      </c>
-      <c r="D34" s="30">
-        <f t="shared" si="0"/>
-        <v>0.18135330578512576</v>
+        <v>9</v>
+      </c>
+      <c r="B34" s="4">
+        <v>43014.311000000002</v>
+      </c>
+      <c r="C34" s="24">
+        <v>42933</v>
+      </c>
+      <c r="D34" s="26">
+        <f t="shared" si="0"/>
+        <v>0.18939044557799711</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B35" s="4">
-        <v>1949.546</v>
-      </c>
-      <c r="C35" s="28">
-        <v>1946</v>
-      </c>
-      <c r="D35" s="30">
-        <f t="shared" si="0"/>
-        <v>0.18221993833504868</v>
+        <v>1939.511</v>
+      </c>
+      <c r="C35" s="24">
+        <v>1936</v>
+      </c>
+      <c r="D35" s="26">
+        <f t="shared" si="0"/>
+        <v>0.18135330578512576</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>15</v>
-      </c>
-      <c r="B36" s="4">
-        <v>301.74400000000003</v>
-      </c>
-      <c r="C36" s="28">
-        <v>298.3</v>
-      </c>
-      <c r="D36" s="30">
-        <f t="shared" si="0"/>
-        <v>1.1545424069728583</v>
+        <v>12</v>
+      </c>
+      <c r="B36" s="5">
+        <f>B34/(_h/2/10)</f>
+        <v>1730.9581891348089</v>
+      </c>
+      <c r="C36" s="24">
+        <v>1728</v>
+      </c>
+      <c r="D36" s="26">
+        <f t="shared" si="0"/>
+        <v>0.17119150085700419</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B37" s="9"/>
-      <c r="D37" s="30" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="A37" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="5">
+        <f>B35/(_b/2/10)</f>
+        <v>193.9511</v>
+      </c>
+      <c r="C37" s="24">
+        <v>193.6</v>
+      </c>
+      <c r="D37" s="26">
+        <f t="shared" si="0"/>
+        <v>0.18135330578512576</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>27</v>
-      </c>
-      <c r="B38" s="9">
-        <f>_rho*_A/10000</f>
-        <v>79.677499999999995</v>
-      </c>
-      <c r="C38" s="28">
-        <v>74.900000000000006</v>
-      </c>
-      <c r="D38" s="30">
-        <f t="shared" si="0"/>
-        <v>6.3785046728971784</v>
+        <v>14</v>
+      </c>
+      <c r="B38" s="4">
+        <v>1949.546</v>
+      </c>
+      <c r="C38" s="24">
+        <v>1946</v>
+      </c>
+      <c r="D38" s="26">
+        <f t="shared" si="0"/>
+        <v>0.18221993833504868</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>29</v>
-      </c>
-      <c r="B39" s="9">
-        <f>B38*_L</f>
-        <v>995.96874999999989</v>
-      </c>
-      <c r="C39" s="28">
-        <v>992</v>
-      </c>
-      <c r="D39" s="30">
-        <f t="shared" si="0"/>
-        <v>0.40007560483870108</v>
+        <v>15</v>
+      </c>
+      <c r="B39" s="4">
+        <v>301.74400000000003</v>
+      </c>
+      <c r="C39" s="24">
+        <v>298.3</v>
+      </c>
+      <c r="D39" s="26">
+        <f t="shared" si="0"/>
+        <v>1.1545424069728583</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B40" s="9"/>
-      <c r="D40" s="30" t="str">
+      <c r="D40" s="26" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>30</v>
-      </c>
-      <c r="B41" s="11">
-        <f>B28*_L*100</f>
-        <v>217643.36143134642</v>
-      </c>
-      <c r="C41" s="28">
-        <v>217643</v>
-      </c>
-      <c r="D41" s="30">
-        <f t="shared" si="0"/>
-        <v>1.6606614796632613E-4</v>
+        <v>27</v>
+      </c>
+      <c r="B41" s="9">
+        <f>_rho*_A/10000</f>
+        <v>79.520499999999998</v>
+      </c>
+      <c r="C41" s="24">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="D41" s="26">
+        <f t="shared" si="0"/>
+        <v>6.1688918558077344</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>31</v>
-      </c>
-      <c r="B42" s="11">
-        <f>(B28-_b/10)*_L*100</f>
-        <v>192643.36143134642</v>
-      </c>
-      <c r="C42" s="28">
-        <v>192643</v>
-      </c>
-      <c r="D42" s="30">
-        <f t="shared" si="0"/>
-        <v>1.8761717084370133E-4</v>
+        <v>29</v>
+      </c>
+      <c r="B42" s="9">
+        <f>B41*_L</f>
+        <v>994.00625000000002</v>
+      </c>
+      <c r="C42" s="24">
+        <v>992</v>
+      </c>
+      <c r="D42" s="26">
+        <f t="shared" si="0"/>
+        <v>0.20224294354838079</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B43" s="9"/>
-      <c r="D43" s="30" t="str">
+      <c r="D43" s="26" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>25</v>
-      </c>
-      <c r="B44" s="9">
-        <f>B28/_A*100</f>
-        <v>171.54156566017451</v>
-      </c>
-      <c r="C44" s="28">
-        <v>172.2</v>
-      </c>
-      <c r="D44" s="30">
-        <f t="shared" si="0"/>
-        <v>-0.38236605100201437</v>
+        <v>30</v>
+      </c>
+      <c r="B44" s="11">
+        <f>B31*_L*100</f>
+        <v>217643.36143134642</v>
+      </c>
+      <c r="C44" s="24">
+        <v>217643</v>
+      </c>
+      <c r="D44" s="26">
+        <f t="shared" si="0"/>
+        <v>1.6606614796632613E-4</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>26</v>
-      </c>
-      <c r="B45" s="9">
-        <f>(B28-_b/10)/_A*100</f>
-        <v>151.83713216263757</v>
-      </c>
-      <c r="C45" s="28">
-        <v>152.4</v>
-      </c>
-      <c r="D45" s="30">
-        <f t="shared" si="0"/>
-        <v>-0.36933585128768875</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D46" s="30" t="str">
+        <v>31</v>
+      </c>
+      <c r="B45" s="11">
+        <f>(B31-_b/10)*_L*100</f>
+        <v>192643.36143134642</v>
+      </c>
+      <c r="C45" s="24">
+        <v>192643</v>
+      </c>
+      <c r="D45" s="26">
+        <f t="shared" si="0"/>
+        <v>1.8761717084370133E-4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B46" s="9"/>
+      <c r="D46" s="26" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="B47" s="25"/>
-      <c r="D47" s="30" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>25</v>
+      </c>
+      <c r="B47" s="9">
+        <f>B31/_A*100</f>
+        <v>171.88024594775629</v>
+      </c>
+      <c r="C47" s="24">
+        <v>172.2</v>
+      </c>
+      <c r="D47" s="26">
+        <f t="shared" si="0"/>
+        <v>-0.18568760292897446</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>26</v>
+      </c>
+      <c r="B48" s="9">
+        <f>(B31-_b/10)/_A*100</f>
+        <v>152.13690932386689</v>
+      </c>
+      <c r="C48" s="24">
+        <v>152.4</v>
+      </c>
+      <c r="D48" s="26">
+        <f t="shared" si="0"/>
+        <v>-0.17263167725269923</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D49" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="B50" s="29"/>
+      <c r="D50" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>17</v>
       </c>
-      <c r="B48" s="13">
+      <c r="B51" s="13">
         <f>_A*100*_fy/1000</f>
-        <v>3603.25</v>
-      </c>
-      <c r="C48" s="28">
+        <v>3596.15</v>
+      </c>
+      <c r="C51" s="24">
         <v>3589</v>
       </c>
-      <c r="D48" s="30">
-        <f t="shared" si="0"/>
-        <v>0.39704653106715782</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+      <c r="D51" s="26">
+        <f t="shared" si="0"/>
+        <v>0.19921983839510382</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>22</v>
       </c>
-      <c r="B49" s="13">
+      <c r="B52" s="13">
         <f>_Av*100*_fy/(1000*SQRT(3))</f>
-        <v>1041.357442933021</v>
-      </c>
-      <c r="C49" s="28">
+        <v>1037.2582560217745</v>
+      </c>
+      <c r="C52" s="24">
         <v>1033</v>
       </c>
-      <c r="D49" s="30">
-        <f t="shared" si="0"/>
-        <v>0.8090457824802666</v>
-      </c>
-      <c r="E49" s="26" t="s">
+      <c r="D52" s="26">
+        <f t="shared" si="0"/>
+        <v>0.41222226735473377</v>
+      </c>
+      <c r="E52" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="F49" s="27"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+      <c r="F52" s="31"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>18</v>
       </c>
-      <c r="B50" s="13">
+      <c r="B53" s="13">
         <f>_Wel_y*1000*_fy*10^(-6)</f>
         <v>614.49015714285713</v>
       </c>
-      <c r="C50" s="28">
+      <c r="C53" s="24">
         <v>613</v>
       </c>
-      <c r="D50" s="30">
+      <c r="D53" s="26">
         <f t="shared" si="0"/>
         <v>0.2430925192262956</v>
       </c>
-      <c r="E50" s="15" t="s">
+      <c r="E53" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="F50" s="17">
+      <c r="F53" s="17">
         <f>9*_epsilon</f>
         <v>7.3225486212014435</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>19</v>
       </c>
-      <c r="B51" s="13">
+      <c r="B54" s="13">
         <f>_Wel_z*1000*_fy*10^(-6)</f>
         <v>68.852640499999993</v>
       </c>
-      <c r="D51" s="30" t="str">
+      <c r="D54" s="26" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="E51" s="15" t="s">
+      <c r="E54" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="F51" s="17">
+      <c r="F54" s="17">
         <f>10*_epsilon</f>
         <v>8.1361651346682713</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
         <v>20</v>
       </c>
-      <c r="B52" s="13">
+      <c r="B55" s="13">
         <f>_Wpl_y*1000*_fy*10^(-6)</f>
         <v>692.08882999999992</v>
       </c>
-      <c r="C52" s="28">
+      <c r="C55" s="24">
         <v>691</v>
       </c>
-      <c r="D52" s="30">
+      <c r="D55" s="26">
         <f t="shared" si="0"/>
         <v>0.15757308248913748</v>
       </c>
-      <c r="E52" s="16" t="s">
+      <c r="E55" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="F52" s="18">
+      <c r="F55" s="18">
         <f>14*_epsilon</f>
         <v>11.390631188535579</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="13">
+      <c r="B56" s="13">
         <f>_Wpl_z*1000*_fy*10^(-6)</f>
         <v>107.11912</v>
       </c>
-      <c r="D53" s="30" t="str">
+      <c r="D56" s="26" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B54" s="13"/>
-      <c r="D54" s="3" t="str">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B57" s="13"/>
+      <c r="D57" s="3" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="E54" s="21" t="s">
+      <c r="E57" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="F54" s="22"/>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="F57" s="22"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
         <v>39</v>
       </c>
-      <c r="B55" s="12">
+      <c r="B58" s="12">
         <f>_cf/_tf</f>
         <v>5.1586206896551721</v>
       </c>
-      <c r="D55" s="3" t="str">
+      <c r="D58" s="3" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="E55" s="15" t="s">
+      <c r="E58" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="F55" s="19">
+      <c r="F58" s="19">
         <f>33*_epsilon</f>
         <v>26.849344944405292</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>40</v>
       </c>
-      <c r="B56" s="12">
+      <c r="B59" s="12">
         <f>_cw/_tw</f>
         <v>50.714285714285715</v>
       </c>
-      <c r="D56" s="3" t="str">
+      <c r="D59" s="3" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="E56" s="15" t="s">
+      <c r="E59" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="F56" s="19">
+      <c r="F59" s="19">
         <f>38*_epsilon</f>
         <v>30.917427511739429</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D57" s="3" t="str">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D60" s="3" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="E57" s="16" t="s">
+      <c r="E60" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="F57" s="20">
+      <c r="F60" s="20">
         <f>42*_epsilon</f>
         <v>34.171893565606737</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>34</v>
       </c>
-      <c r="B58">
-        <f>IF(B55&lt;=F50,1,IF(B55&lt;=F51,2,IF(B55&lt;=F52,3,4)))</f>
+      <c r="B61">
+        <f>IF(B58&lt;=F53,1,IF(B58&lt;=F54,2,IF(B58&lt;=F55,3,4)))</f>
         <v>1</v>
       </c>
-      <c r="D58" s="3" t="str">
+      <c r="D61" s="3" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
         <v>35</v>
       </c>
-      <c r="B59">
-        <f>IF(B56&lt;=F55,1,IF(B56&lt;=F56,2,IF(B56&lt;=F57,3,4)))</f>
+      <c r="B62">
+        <f>IF(B59&lt;=F58,1,IF(B59&lt;=F59,2,IF(B59&lt;=F60,3,4)))</f>
         <v>4</v>
       </c>
-      <c r="D59" s="3" t="str">
+      <c r="D62" s="3" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="E59" s="21" t="s">
+      <c r="E62" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="F59" s="22"/>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+      <c r="F62" s="22"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
         <v>36</v>
       </c>
-      <c r="B60">
-        <f>IF(B56&lt;=F60,1,IF(B56&lt;=F61,2,IF(B56&lt;=F62,3,4)))</f>
+      <c r="B63">
+        <f>IF(B59&lt;=F63,1,IF(B59&lt;=F64,2,IF(B59&lt;=F65,3,4)))</f>
         <v>1</v>
       </c>
-      <c r="D60" s="3" t="str">
+      <c r="D63" s="3" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="E60" s="15" t="s">
+      <c r="E63" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="F60" s="19">
+      <c r="F63" s="19">
         <f>72*_epsilon</f>
         <v>58.580388969611548</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D61" s="3" t="str">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D64" s="3" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="E61" s="15" t="s">
+      <c r="E64" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="F61" s="19">
+      <c r="F64" s="19">
         <f>83*_epsilon</f>
         <v>67.530170617746649</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>52</v>
       </c>
-      <c r="B62" s="3">
+      <c r="B65" s="3">
         <f>_hw/_tw</f>
         <v>55.714285714285715</v>
       </c>
-      <c r="D62" s="3" t="str">
+      <c r="D65" s="3" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="E62" s="16" t="s">
+      <c r="E65" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="F62" s="20">
+      <c r="F65" s="20">
         <f>124*_epsilon</f>
         <v>100.88844766988656</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
         <v>51</v>
       </c>
-      <c r="B63" s="23">
+      <c r="B66" s="23">
         <f>124*_epsilon</f>
         <v>100.88844766988656</v>
       </c>
-      <c r="D63" s="3" t="str">
+      <c r="D66" s="3" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D64" s="3" t="str">
+    <row r="67" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D67" s="3" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="24" t="s">
+    <row r="68" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="B65" s="25"/>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+      <c r="B68" s="29"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
         <v>80</v>
       </c>
-      <c r="B66">
+      <c r="B69">
         <v>6.67</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>85</v>
       </c>
-      <c r="B67">
+      <c r="B70">
         <f>_bc-_tw</f>
         <v>191.6</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>83</v>
       </c>
-      <c r="B68" s="30">
+      <c r="B71" s="26">
         <f>(4-PI())*_r^2/(2*_n)</f>
         <v>28.377634165434873</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>84</v>
       </c>
-      <c r="B69" s="29">
+      <c r="B72" s="25">
         <f>(10-3*PI())/(12-3*PI())</f>
         <v>0.22336793894575216</v>
       </c>
-      <c r="E69">
+      <c r="E72">
         <f>(53002/52921-1)*100</f>
         <v>0.15305833223107079</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>86</v>
       </c>
-      <c r="B70">
+      <c r="B73">
         <f>_tf+_kr*_r</f>
         <v>19.190726717860795</v>
       </c>
-      <c r="E70">
+      <c r="E73">
         <f>(47200/47128-1)*100</f>
         <v>0.15277542013241163</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>87</v>
       </c>
-      <c r="B71">
+      <c r="B74">
         <f>_h/2</f>
         <v>248.5</v>
       </c>
-      <c r="E71">
+      <c r="E74">
         <f>(47083/47005-1)*100</f>
         <v>0.16593979363896949</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>88</v>
       </c>
-      <c r="B72" s="23">
+      <c r="B75" s="23">
         <f>_A*100+_As_inf*100-_Acr-_bp*_tf/_n</f>
-        <v>10031.826262677469</v>
-      </c>
-      <c r="C72" s="28">
+        <v>10011.826262677469</v>
+      </c>
+      <c r="C75" s="24">
         <v>9998</v>
       </c>
-      <c r="D72">
-        <f>(B72/C72-1)*100</f>
-        <v>0.33833029283325544</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+      <c r="D75">
+        <f>(B75/C75-1)*100</f>
+        <v>0.13829028483165473</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>89</v>
       </c>
-      <c r="B73" s="23">
+      <c r="B76" s="23">
         <f>_A*100*_za+_As_inf*100*_zs_inf-_Acr*_zcr-_bp*_tf^2/(2*_n)</f>
-        <v>2656752.2111678715</v>
-      </c>
-      <c r="C73" s="28">
+        <v>2651782.2111678715</v>
+      </c>
+      <c r="C76" s="24">
         <v>2646805</v>
       </c>
-      <c r="D73">
-        <f>(B73/C73-1)*100</f>
-        <v>0.37581956992946974</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+      <c r="D76">
+        <f>(B76/C76-1)*100</f>
+        <v>0.18804600897577295</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>90</v>
       </c>
-      <c r="B74" s="3">
+      <c r="B77" s="3">
         <f>_n*_A0/_bp*(-1+SQRT(1+2*_bp*_B0/(_n*_A0^2)))</f>
-        <v>204.78830751093571</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+        <v>204.73330249305826</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>91</v>
       </c>
-      <c r="B75">
+      <c r="B78">
         <f>_tf+_r</f>
         <v>35.5</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>92</v>
       </c>
-      <c r="B76">
+      <c r="B79">
         <f>_zs_inf</f>
         <v>422.5</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>93</v>
       </c>
-      <c r="B77" t="b">
-        <f>IF(B75&lt;=_zel,IF(_zel&lt;=B76,TRUE,FALSE),FALSE)</f>
+      <c r="B80" t="b">
+        <f>IF(B78&lt;=_zel,IF(_zel&lt;=B79,TRUE,FALSE),FALSE)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>94</v>
       </c>
-      <c r="B78">
+      <c r="B81">
         <f>(_Iy*10^4+_A*100*(_za-_zel)^2+_As_inf*100*(_zs_inf-_zel)^2+_bp*(_zel-_tf)^3/(3*_n)-_Acr*(_zcr-_zel)^2)*10^(-4)</f>
-        <v>53002.140380188146</v>
-      </c>
-      <c r="C78" s="28">
+        <v>52998.314147422454</v>
+      </c>
+      <c r="C81" s="24">
         <f>52814</f>
         <v>52814</v>
       </c>
-      <c r="D78">
-        <f>(B78/C78-1)*100</f>
-        <v>0.35623202216863437</v>
+      <c r="D81">
+        <f>(B81/C81-1)*100</f>
+        <v>0.34898729015497842</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>95</v>
+      </c>
+      <c r="B82" s="26">
+        <f>210000/_Ecm_dalle</f>
+        <v>6.6717909812633494</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>96</v>
+      </c>
+      <c r="B83" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E83" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="F83" s="22"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>100</v>
+      </c>
+      <c r="B84" s="1">
+        <f>50/100</f>
+        <v>0.5</v>
+      </c>
+      <c r="E84" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="F84" s="33">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>101</v>
+      </c>
+      <c r="B85" s="25">
+        <f>IF(E6&lt;=35,1+(1-B84)/(0.1*E5^(1/3)),FALSE)</f>
+        <v>1.8685939040970632</v>
+      </c>
+      <c r="E85" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="F85" s="34">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>102</v>
+      </c>
+      <c r="B86" s="25">
+        <f>16.8/SQRT(_fcm_enrobage)</f>
+        <v>2.9245046200557239</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>103</v>
+      </c>
+      <c r="B87">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>104</v>
+      </c>
+      <c r="B88">
+        <v>18250</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>105</v>
+      </c>
+      <c r="B89" s="25">
+        <f>1/(0.1+B87^0.2)</f>
+        <v>0.42792578098028256</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>106</v>
+      </c>
+      <c r="B90" s="26">
+        <f>B85*B86*B89</f>
+        <v>2.3384909388400645</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>107</v>
+      </c>
+      <c r="B91" s="3">
+        <f>IF(_fck_enrobage&lt;=25,MIN(1.5*(1+(0.012*B84*100)^18+250),1500),FALSE)</f>
+        <v>376.50015233993503</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>108</v>
+      </c>
+      <c r="B92" s="26">
+        <f>((B88-B87)/(B91+B88-B87))^0.3</f>
+        <v>0.9938741085684526</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>109</v>
+      </c>
+      <c r="B93" s="25">
+        <f>B90*B92</f>
+        <v>2.3241655972350728</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>110</v>
+      </c>
+      <c r="B94" s="26">
+        <f>B82*(1+B83*B93)</f>
+        <v>23.728772758918403</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="96" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="B96" s="29"/>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>112</v>
+      </c>
+      <c r="B97">
+        <f>_dw*_tw*_fy/1000</f>
+        <v>1270.3320000000001</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>114</v>
+      </c>
+      <c r="B98" s="23">
+        <f>_As_inf*100*_fyd/1000</f>
+        <v>142.05462433623416</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>116</v>
+      </c>
+      <c r="B99" s="23">
+        <f>0.85*_dw*_bp*_fck_enrobage/(1.5*1000)</f>
+        <v>1156.3059999999996</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>117</v>
+      </c>
+      <c r="B100" s="3">
+        <f>0.85*(_r*_bp-(4-PI())*_r^2/2)*_fck_enrobage/(1.5*1000)</f>
+        <v>54.31955005165112</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>118</v>
+      </c>
+      <c r="B101" s="26">
+        <f>(B97+B98-B100)/(2*B97+B99)</f>
+        <v>0.36734598178632322</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>119</v>
+      </c>
+      <c r="B102" s="23">
+        <f>_tf+_r+B101*_dw</f>
+        <v>191.98938824097368</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>120</v>
+      </c>
+      <c r="B103">
+        <f>_tf+_r</f>
+        <v>35.5</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>121</v>
+      </c>
+      <c r="B104">
+        <f>_zs_inf</f>
+        <v>422.5</v>
+      </c>
+      <c r="D104" s="3"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>93</v>
+      </c>
+      <c r="B105" t="b">
+        <f>IF(B103&lt;=_zpl,IF(_zpl&lt;=B104,TRUE,FALSE),FALSE)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>122</v>
+      </c>
+      <c r="B106" s="23">
+        <f>_zpl-_tf-_r</f>
+        <v>156.48938824097368</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>123</v>
+      </c>
+      <c r="B107" s="3">
+        <f>((_Wpl_y*10^3-(_h/2-_zpl)^2*_tw)*_fy+B98*1000*(_zs_inf-_h/2)+0.85*B106*_bp*_fck_enrobage/1.5*(_h/2-_tf-_r-B106/2)+B100*1000*(_h/2-_tf-_r/2))*10^(-6)</f>
+        <v>776.66314007116341</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="109" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="28" t="s">
+        <v>133</v>
+      </c>
+      <c r="B109" s="29"/>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>130</v>
+      </c>
+      <c r="B110" s="26">
+        <f>_qProfile+_qEnrobage+_qBac+_qDalle</f>
+        <v>9.6760339528260868</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>132</v>
+      </c>
+      <c r="B111" s="3">
+        <f>B110*_L/2</f>
+        <v>60.475212205163039</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>131</v>
+      </c>
+      <c r="B112" s="3">
+        <f>B110*_L^2/8</f>
+        <v>188.98503814113451</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>135</v>
+      </c>
+      <c r="B113" s="3">
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>136</v>
+      </c>
+      <c r="B114" s="3">
+        <v>45.3</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>137</v>
+      </c>
+      <c r="B115" s="3">
+        <f>B111+B113</f>
+        <v>73.775212205163044</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>138</v>
+      </c>
+      <c r="B116" s="3">
+        <f t="shared" ref="B116" si="1">B112+B114</f>
+        <v>234.28503814113452</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>139</v>
+      </c>
+      <c r="B117" s="3">
+        <f>1.35*B111+1.5*B113</f>
+        <v>101.59153647697011</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>140</v>
+      </c>
+      <c r="B118" s="3">
+        <f>1.35*B112+1.5*B114</f>
+        <v>323.07980149053162</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="120" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A120" s="28" t="s">
+        <v>134</v>
+      </c>
+      <c r="B120" s="29"/>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>141</v>
+      </c>
+      <c r="B121" s="26">
+        <f>B118/B107</f>
+        <v>0.41598446587915677</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>142</v>
+      </c>
+      <c r="B122" s="26">
+        <f>B117/_VplRd</f>
+        <v>9.794237441561271E-2</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>149</v>
+      </c>
+      <c r="B123" s="36">
+        <v>492.5</v>
+      </c>
+      <c r="C123" s="24" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>150</v>
+      </c>
+      <c r="B124" s="26">
+        <f>B118/B123</f>
+        <v>0.65599959693508958</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>143</v>
+      </c>
+      <c r="B125" s="3">
+        <f>5*B110*(_L*1000)^4/(384*210000*47199*10^(4))</f>
+        <v>31.033025872841279</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>144</v>
+      </c>
+      <c r="B126" s="37">
+        <v>6.476</v>
+      </c>
+      <c r="C126" s="24" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>146</v>
+      </c>
+      <c r="B127" s="3">
+        <f>B125+B126</f>
+        <v>37.509025872841278</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>147</v>
+      </c>
+      <c r="B128">
+        <f>B125+0.2*B126</f>
+        <v>32.32822587284128</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>148</v>
+      </c>
+      <c r="B129">
+        <f>PI()/2*SQRT(210*52998*10/(B110*1000/9.81*_L*_L^4))</f>
+        <v>0.95514662218841706</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="11">
+    <mergeCell ref="A96:B96"/>
+    <mergeCell ref="A109:B109"/>
+    <mergeCell ref="A120:B120"/>
     <mergeCell ref="G1:H1"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="A68:B68"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="E52:F52"/>
     <mergeCell ref="D1:E1"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E15">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E16">
       <formula1>"Aucun,Perpendiculaire,Longitudinal"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fin cas test 3
</commit_message>
<xml_diff>
--- a/Manuel Validation/Cas tests références.xlsx
+++ b/Manuel Validation/Cas tests références.xlsx
@@ -104,10 +104,13 @@
     <definedName name="_n" localSheetId="0">'Cas 2'!$B$69</definedName>
     <definedName name="_n_dalle" localSheetId="1">'Cas 3'!$B$70</definedName>
     <definedName name="_n_enrobage" localSheetId="1">'Cas 3'!#REF!</definedName>
-    <definedName name="_Nf" localSheetId="1">'Cas 3'!$B$93</definedName>
+    <definedName name="_Na" localSheetId="1">'Cas 3'!$H$23</definedName>
+    <definedName name="_Ncp" localSheetId="1">'Cas 3'!$B$104</definedName>
+    <definedName name="_Nf" localSheetId="1">'Cas 3'!$B$102</definedName>
     <definedName name="_nr" localSheetId="1">'Cas 3'!$H$16</definedName>
+    <definedName name="_Ns_inf" localSheetId="1">'Cas 3'!$H$24</definedName>
     <definedName name="_NtRd" localSheetId="0">'Cas 2'!$B$51</definedName>
-    <definedName name="_Nw" localSheetId="1">'Cas 3'!$B$94</definedName>
+    <definedName name="_Nw" localSheetId="1">'Cas 3'!$B$103</definedName>
     <definedName name="_qBac" localSheetId="0">'Cas 2'!$E$26</definedName>
     <definedName name="_qBac" localSheetId="1">'Cas 3'!$E$26</definedName>
     <definedName name="_qDalle" localSheetId="0">'Cas 2'!$H$10</definedName>
@@ -140,14 +143,15 @@
     <definedName name="_Wpl_z" localSheetId="0">'Cas 2'!$B$39</definedName>
     <definedName name="_Wpl_z" localSheetId="1">'Cas 3'!$B$40</definedName>
     <definedName name="_za" localSheetId="0">'Cas 2'!$B$74</definedName>
-    <definedName name="_za" localSheetId="1">'Cas 3'!$B$71</definedName>
+    <definedName name="_za" localSheetId="1">'Cas 3'!$B$73</definedName>
     <definedName name="_zcr" localSheetId="0">'Cas 2'!$B$73</definedName>
     <definedName name="_zcr" localSheetId="1">'Cas 3'!#REF!</definedName>
     <definedName name="_zel" localSheetId="0">'Cas 2'!$B$77</definedName>
-    <definedName name="_zel" localSheetId="1">'Cas 3'!$B$73</definedName>
+    <definedName name="_zel" localSheetId="1">'Cas 3'!$B$79</definedName>
     <definedName name="_zpl" localSheetId="0">'Cas 2'!$B$102</definedName>
-    <definedName name="_zpl" localSheetId="1">'Cas 3'!$B$96</definedName>
-    <definedName name="_zs" localSheetId="1">'Cas 3'!$B$72</definedName>
+    <definedName name="_zpl_a" localSheetId="1">'Cas 3'!$B$107</definedName>
+    <definedName name="_zpl_c" localSheetId="1">'Cas 3'!$B$105</definedName>
+    <definedName name="_zs" localSheetId="1">'Cas 3'!$B$74</definedName>
     <definedName name="_zs_inf" localSheetId="0">'Cas 2'!$E$11</definedName>
     <definedName name="_zs_inf" localSheetId="1">'Cas 3'!$E$11</definedName>
   </definedNames>
@@ -161,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="218">
   <si>
     <t>h (mm)</t>
   </si>
@@ -722,20 +726,114 @@
   </si>
   <si>
     <t>Ncp (kN)</t>
+  </si>
+  <si>
+    <t>n enrobage</t>
+  </si>
+  <si>
+    <t>Calcul coefficient équivalence LT</t>
+  </si>
+  <si>
+    <t>ANE dans la dalle</t>
+  </si>
+  <si>
+    <t>ANE dans section</t>
+  </si>
+  <si>
+    <t>Hypothèse</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>de (mm)</t>
+  </si>
+  <si>
+    <t>C (mm2)</t>
+  </si>
+  <si>
+    <t>zce (mm)</t>
+  </si>
+  <si>
+    <t>zpl,a (mm)</t>
+  </si>
+  <si>
+    <t>zpl,c (mm)</t>
+  </si>
+  <si>
+    <t>Moment dalle (kN.m)</t>
+  </si>
+  <si>
+    <t>Moment semelle sup (kN.m)</t>
+  </si>
+  <si>
+    <t>Moment âme (kN.m)</t>
+  </si>
+  <si>
+    <t>Moment semelle inf (kN.m)</t>
+  </si>
+  <si>
+    <t>Moment armatures inf (kN.m)</t>
+  </si>
+  <si>
+    <t>V(G2) (kN)</t>
+  </si>
+  <si>
+    <t>M(G2) (kN.m)</t>
+  </si>
+  <si>
+    <t>V(Q1) (kN)</t>
+  </si>
+  <si>
+    <t>M(Q1) (kN.m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimensionnement armatures transversales </t>
+  </si>
+  <si>
+    <t>ved (MPa)</t>
+  </si>
+  <si>
+    <t>DFx/Dx (kN/m)</t>
+  </si>
+  <si>
+    <t>theta (°)</t>
+  </si>
+  <si>
+    <t>ved,lim (MPa)</t>
+  </si>
+  <si>
+    <t>nu</t>
+  </si>
+  <si>
+    <t>gamma sf</t>
+  </si>
+  <si>
+    <t>Asf/sf (cm2/m)</t>
+  </si>
+  <si>
+    <t>f(G2) (mm)</t>
+  </si>
+  <si>
+    <t>f(Q1) (mm)</t>
+  </si>
+  <si>
+    <t>f (SHC) (mm)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -765,6 +863,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -780,7 +891,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -902,12 +1013,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -960,8 +1110,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1289,8 +1460,8 @@
         <v>60</v>
       </c>
       <c r="H2" s="23">
-        <f>2*_tc*(1+_hp*_bm/(_ep*_tc))</f>
-        <v>209.67149758454107</v>
+        <f>IF(E16="Perpendiculaire",2*_tc,FALSE)</f>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -2489,8 +2660,8 @@
         <v>107</v>
       </c>
       <c r="B91" s="3">
-        <f>IF(_fck_enrobage&lt;=25,MIN(1.5*(1+(0.012*B84*100)^18+250),1500),FALSE)</f>
-        <v>376.50015233993503</v>
+        <f>IF(_fcm_enrobage&lt;=35,MIN(B81*1.5*(1+(0.012*B80)^18)+250,1500),FALSE)</f>
+        <v>1500</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -2499,7 +2670,7 @@
       </c>
       <c r="B92" s="26">
         <f>((B88-B87)/(B91+B88-B87))^0.3</f>
-        <v>0.9938741085684526</v>
+        <v>0.97651355707570364</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -2508,7 +2679,7 @@
       </c>
       <c r="B93" s="25">
         <f>B90*B92</f>
-        <v>2.3241655972350728</v>
+        <v>2.283568104876013</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -2517,7 +2688,7 @@
       </c>
       <c r="B94" s="26">
         <f>B82*(1+B83*B93)</f>
-        <v>23.728772758918403</v>
+        <v>23.430828977197017</v>
       </c>
     </row>
     <row r="95" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -2831,12 +3002,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I123"/>
+  <dimension ref="A1:I154"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="24"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" style="24" customWidth="1"/>
     <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
@@ -2876,8 +3047,8 @@
         <v>60</v>
       </c>
       <c r="H2" s="23">
-        <f>2*_tc*(1+_hp*_bm/(_ep*_tc))</f>
-        <v>209.67149758454107</v>
+        <f>IF(E16="Perpendiculaire",2*_tc,FALSE)</f>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -2937,7 +3108,7 @@
       <c r="D5" t="s">
         <v>60</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5" s="3">
         <f>_Ace*100/_hw</f>
         <v>190.74786324786325</v>
       </c>
@@ -4017,493 +4188,795 @@
       <c r="A70" t="s">
         <v>183</v>
       </c>
-      <c r="B70">
-        <v>6.77</v>
+      <c r="B70" s="32">
+        <v>25.2</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>187</v>
+      </c>
+      <c r="B71" s="32">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>191</v>
+      </c>
+      <c r="B72" s="47" t="s">
+        <v>189</v>
+      </c>
+      <c r="C72" s="48" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>87</v>
       </c>
-      <c r="B71">
+      <c r="B73" s="39">
         <f>_td+_h/2</f>
         <v>388.5</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+      <c r="C73" s="46">
+        <f>_za</f>
+        <v>388.5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>184</v>
       </c>
-      <c r="B72">
+      <c r="B74" s="39">
         <f>_td+_zs_inf</f>
         <v>562.5</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+      <c r="C74" s="46">
+        <f>_zs</f>
+        <v>562.5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>88</v>
+      </c>
+      <c r="B75" s="42" t="s">
+        <v>192</v>
+      </c>
+      <c r="C75" s="44">
+        <f>_A*100+_As_inf*100+_beff_mi_travee*1000*_tc/_n_dalle</f>
+        <v>18591.646270893973</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>193</v>
+      </c>
+      <c r="B76" s="42" t="s">
+        <v>192</v>
+      </c>
+      <c r="C76" s="45">
+        <f>_Ace*100/(B71*_hw)</f>
+        <v>7.7225855565936534</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>194</v>
+      </c>
+      <c r="B77" s="42" t="s">
+        <v>192</v>
+      </c>
+      <c r="C77" s="44">
+        <f>_A*100*(_h/2-_tf)+_As_inf*100*(_zs_inf-_tf)+_beff_mi_travee*1000*_tc/_n_dalle*(_tc/2-_tf-_td)</f>
+        <v>1580410.56741363</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>195</v>
+      </c>
+      <c r="B78" s="43" t="s">
+        <v>192</v>
+      </c>
+      <c r="C78" s="44">
+        <f>C75/C76*(-1+SQRT(1+2*C77*C76/C75^2))</f>
+        <v>83.556465257011979</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>90</v>
       </c>
-      <c r="B73" s="3">
+      <c r="B79" s="51">
         <f>(_beff_mi_travee*1000*_tc^2/(2*_n_dalle)+_A*100*_za+_As_inf*100*_zs)/(_beff_mi_travee*1000*_tc/_n_dalle+_A*100+_As_inf*100)</f>
-        <v>131.594015157716</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+        <v>239.50648863397487</v>
+      </c>
+      <c r="C79" s="52">
+        <f>_td+_tf+C78</f>
+        <v>238.05646525701198</v>
+      </c>
+      <c r="D79">
+        <f>_zel-_td</f>
+        <v>99.506488633974868</v>
+      </c>
+      <c r="E79" s="3">
+        <f>C79-_td</f>
+        <v>98.056465257011979</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>91</v>
       </c>
-      <c r="B74">
+      <c r="B80" s="39">
         <f>_tc</f>
         <v>82</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+      <c r="C80" s="46">
+        <f>_tc+_td</f>
+        <v>222</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>92</v>
       </c>
-      <c r="B75">
+      <c r="B81" s="39">
         <f>_td+_tf</f>
         <v>154.5</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+      <c r="C81" s="46">
+        <f>C80+_h</f>
+        <v>719</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
         <v>93</v>
       </c>
-      <c r="B76" t="b">
-        <f>IF(B74&lt;=_zel,IF(_zel&lt;=B75,TRUE,FALSE),FALSE)</f>
+      <c r="B82" s="39" t="b">
+        <f>IF(B80&lt;=_zel,IF(_zel&lt;=B81,TRUE,FALSE),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="C82" s="39" t="b">
+        <f>IF(C80&lt;=C79,IF(C79&lt;=C81,TRUE,FALSE),FALSE)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>94</v>
       </c>
-      <c r="B77" s="5">
+      <c r="B83" s="53">
         <f>(_Iy*10^4+_A*100*(_za-_zel)^2+_As_inf*100*(_zs-_zel)^2+_beff_mi_travee*1000*_tc/_n_dalle*(_tc^2/12+(_tc/2-_zel)^2))*10^(-4)</f>
-        <v>142488.53513587199</v>
-      </c>
-      <c r="C77" s="24">
-        <f>52814</f>
-        <v>52814</v>
-      </c>
-      <c r="D77">
-        <f>(B77/C77-1)*100</f>
-        <v>169.79311382563714</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+        <v>101421.8641875779</v>
+      </c>
+      <c r="C83" s="54">
+        <f>(_Iy*10^4+_A*100*(_za-C79)^2+_As_inf*100*(_zs-C79)^2+_beff_mi_travee*1000*_tc/_n_dalle*(_tc^2/12+(_tc/2-C79)^2)+(_bc-_tw)*C78^3/(3*B71))*10^(-4)</f>
+        <v>101576.61353768932</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B84" s="41"/>
+      <c r="C84" s="40"/>
+    </row>
+    <row r="85" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="49" t="s">
+        <v>188</v>
+      </c>
+      <c r="B85" s="50"/>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>95</v>
       </c>
-      <c r="B78" s="26">
+      <c r="B86" s="26">
         <f>210000/_Ecm_dalle</f>
         <v>6.6717909812633494</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>96</v>
       </c>
-      <c r="B79" s="1">
+      <c r="B87" s="1">
         <v>1.1000000000000001</v>
       </c>
-      <c r="E79" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="F79" s="22"/>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>100</v>
       </c>
-      <c r="B80" s="1">
+      <c r="B88" s="1">
         <f>50/100</f>
         <v>0.5</v>
       </c>
-      <c r="E80" s="28" t="s">
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>60</v>
+      </c>
+      <c r="B89" s="32">
+        <f>H2</f>
+        <v>164</v>
+      </c>
+      <c r="D89" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="E89" s="22"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>101</v>
+      </c>
+      <c r="B90" s="25">
+        <f>IF(E6&lt;=35,1+(1-B88)/(0.1*B89^(1/3)),FALSE)</f>
+        <v>1.9134582902287138</v>
+      </c>
+      <c r="D90" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="F80" s="29">
+      <c r="E90" s="29">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>101</v>
-      </c>
-      <c r="B81" s="25">
-        <f>IF(E6&lt;=35,1+(1-B80)/(0.1*E5^(1/3)),FALSE)</f>
-        <v>1.8685939040970632</v>
-      </c>
-      <c r="E81" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="F81" s="30">
-        <v>0.55000000000000004</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>102</v>
       </c>
-      <c r="B82" s="25">
+      <c r="B91" s="38">
         <f>16.8/SQRT(_fcm_enrobage)</f>
         <v>2.9245046200557239</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+      <c r="D91" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="E91" s="30">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>103</v>
       </c>
-      <c r="B83">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+      <c r="B92" s="1">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>104</v>
       </c>
-      <c r="B84">
+      <c r="B93">
         <v>18250</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>105</v>
       </c>
-      <c r="B85" s="25">
-        <f>1/(0.1+B83^0.2)</f>
-        <v>0.42792578098028256</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+      <c r="B94" s="25">
+        <f>1/(0.1+B92^0.2)</f>
+        <v>0.48844954537902541</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>106</v>
       </c>
-      <c r="B86" s="26">
-        <f>B81*B82*B85</f>
-        <v>2.3384909388400645</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+      <c r="B95" s="26">
+        <f>B90*B91*B94</f>
+        <v>2.7333234126112149</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>107</v>
       </c>
-      <c r="B87" s="3">
-        <f>IF(_fck_enrobage&lt;=25,MIN(1.5*(1+(0.012*B80*100)^18+250),1500),FALSE)</f>
-        <v>376.50015233993503</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+      <c r="B96" s="3">
+        <f>IF(_fcm_enrobage&lt;=35,MIN(B89*1.5*(1+(0.012*B88)^18)+250,1500),FALSE)</f>
+        <v>496</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>108</v>
       </c>
-      <c r="B88" s="26">
-        <f>((B84-B83)/(B87+B84-B83))^0.3</f>
-        <v>0.9938741085684526</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+      <c r="B97" s="26">
+        <f>((B93-B92)/(B96+B93-B92))^0.3</f>
+        <v>0.99197557722517693</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>109</v>
       </c>
-      <c r="B89" s="25">
-        <f>B86*B88</f>
-        <v>2.3241655972350728</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+      <c r="B98" s="25">
+        <f>B95*B97</f>
+        <v>2.7113900699681004</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>110</v>
       </c>
-      <c r="B90" s="26">
-        <f>B78*(1+B79*B89)</f>
-        <v>23.728772758918403</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="92" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="34" t="s">
+      <c r="B99" s="26">
+        <f>B86*(1+B87*B98)</f>
+        <v>26.570601578313543</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="101" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="34" t="s">
         <v>111</v>
       </c>
-      <c r="B92" s="35"/>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A93" s="7" t="s">
+      <c r="B101" s="35"/>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="B93" s="38">
+      <c r="B102" s="55">
         <f>_tf*_b*_fy/1000</f>
         <v>1029.5</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
         <v>112</v>
       </c>
-      <c r="B94">
-        <f>_A*100*_fy/1000-2*B93</f>
+      <c r="B103">
+        <f>_A*100*_fy/1000-2*B102</f>
         <v>1537.15</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
         <v>186</v>
       </c>
-      <c r="B95">
+      <c r="B104" s="23">
         <f>_eta*0.85*_beff_mi_travee*1000*_tc*_fck_dalle/(1000*1.5)</f>
         <v>2259.5775141604267</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>119</v>
-      </c>
-      <c r="B96" s="23">
-        <f>B95/(0.85*_beff_mi_travee*1000*_fck_dalle/1000/1.5)</f>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>197</v>
+      </c>
+      <c r="B105" s="23">
+        <f>B104/(0.85*_beff_mi_travee*1000*_fck_dalle/1000/1.5)</f>
         <v>63.799835693941468</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>118</v>
+      </c>
+      <c r="B106" s="26">
+        <f>(_Na+_Ns_inf-_Ncp)/(2*_Nf)</f>
+        <v>0.71812875676338395</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>196</v>
+      </c>
+      <c r="B107" s="23">
+        <f>_td+B106*_tf</f>
+        <v>150.41286697306907</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>120</v>
       </c>
-      <c r="B97">
-        <f>_tf+_r</f>
-        <v>35.5</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+      <c r="B108">
+        <f>_td</f>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
         <v>121</v>
       </c>
-      <c r="B98">
-        <f>_zs_inf</f>
-        <v>422.5</v>
-      </c>
-      <c r="D98" s="3"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
+      <c r="B109">
+        <f>_td+_tf</f>
+        <v>154.5</v>
+      </c>
+      <c r="D109" s="3"/>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
         <v>93</v>
       </c>
-      <c r="B99" t="b">
-        <f>IF(B97&lt;=_zpl,IF(_zpl&lt;=B98,TRUE,FALSE),FALSE)</f>
+      <c r="B110" t="b">
+        <f>IF(B108&lt;=_zpl_a,IF(_zpl_a&lt;=B109,TRUE,FALSE),FALSE)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>122</v>
-      </c>
-      <c r="B100" s="23">
-        <f>_zpl-_tf-_r</f>
-        <v>28.299835693941468</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>198</v>
+      </c>
+      <c r="B111" s="23">
+        <f>_Ncp*(_zpl_a-_zpl_c/2)/1000</f>
+        <v>267.78919498217044</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>199</v>
+      </c>
+      <c r="B112" s="3">
+        <f>(B106^2+(1-B106)^2)*_Nf*_tf/2/1000</f>
+        <v>4.4422021517425065</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>200</v>
+      </c>
+      <c r="B113" s="23">
+        <f>_Nw*(_h/2+_td-_zpl_a)/1000</f>
+        <v>365.97563653234687</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>201</v>
+      </c>
+      <c r="B114" s="3">
+        <f>_Nf*(_h-_tf/2+_td-_zpl_a)/1000</f>
+        <v>493.47757845122544</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>202</v>
+      </c>
+      <c r="B115" s="3">
+        <f>_Ns_inf*(_zs_inf+_td-_zpl_a)/1000</f>
+        <v>58.538882875936423</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
         <v>123</v>
       </c>
-      <c r="B101" s="3" t="e">
-        <f>((_Wpl_y*10^3-(_h/2-_zpl)^2*_tw)*_fy+#REF!*1000*(_zs_inf-_h/2)+0.85*B100*_bp*_fck_enrobage/1.5*(_h/2-_tf-_r-B100/2)+#REF!*1000*(_h/2-_tf-_r/2))*10^(-6)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="103" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A103" s="34" t="s">
+      <c r="B116" s="3">
+        <f>SUM(B111:B115)</f>
+        <v>1190.2234949934218</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="118" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="34" t="s">
         <v>133</v>
       </c>
-      <c r="B103" s="35"/>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
+      <c r="B118" s="35"/>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
         <v>130</v>
       </c>
-      <c r="B104" s="26">
+      <c r="B119" s="26">
         <f>_qProfile+_qEnrobage+_qBac+_qDalle</f>
         <v>9.6760339528260868</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
         <v>132</v>
       </c>
-      <c r="B105" s="3">
-        <f>B104*_L/2</f>
+      <c r="B120" s="3">
+        <f>B119*_L/2</f>
         <v>60.475212205163039</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
         <v>131</v>
       </c>
-      <c r="B106" s="3">
-        <f>B104*_L^2/8</f>
+      <c r="B121" s="3">
+        <f>B119*_L^2/8</f>
         <v>188.98503814113451</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>203</v>
+      </c>
+      <c r="B122" s="3">
+        <f>2.5*_L/2</f>
+        <v>15.625</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>204</v>
+      </c>
+      <c r="B123" s="3">
+        <f>2.5*_L^2/8</f>
+        <v>48.828125</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>205</v>
+      </c>
+      <c r="B124" s="3">
+        <f>6.25*_L/2</f>
+        <v>39.0625</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>206</v>
+      </c>
+      <c r="B125" s="3">
+        <f>6.25*_L^2/8</f>
+        <v>122.0703125</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
         <v>135</v>
       </c>
-      <c r="B107" s="3">
+      <c r="B126" s="3">
         <v>13.3</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
         <v>136</v>
       </c>
-      <c r="B108" s="3">
+      <c r="B127" s="3">
         <v>45.3</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
         <v>137</v>
       </c>
-      <c r="B109" s="3">
-        <f>B105+B107</f>
-        <v>73.775212205163044</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
+      <c r="B128" s="3">
+        <f>B120+B122+B124</f>
+        <v>115.16271220516305</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
         <v>138</v>
       </c>
-      <c r="B110" s="3">
-        <f t="shared" ref="B110" si="1">B106+B108</f>
-        <v>234.28503814113452</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
+      <c r="B129" s="3">
+        <f>B121+B123+B125</f>
+        <v>359.88347564113451</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
         <v>139</v>
       </c>
-      <c r="B111" s="3">
-        <f>1.35*B105+1.5*B107</f>
-        <v>101.59153647697011</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
+      <c r="B130" s="3">
+        <f>1.35*(B120+B122)+1.5*B124</f>
+        <v>161.32903647697012</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
         <v>140</v>
       </c>
-      <c r="B112" s="3">
-        <f>1.35*B106+1.5*B108</f>
-        <v>323.07980149053162</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="114" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="34" t="s">
+      <c r="B131" s="3">
+        <f>1.35*(B121+B123)+1.5*B125</f>
+        <v>504.15323899053163</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="133" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A133" s="34" t="s">
         <v>134</v>
       </c>
-      <c r="B114" s="35"/>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
+      <c r="B133" s="35"/>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
         <v>141</v>
       </c>
-      <c r="B115" s="26" t="e">
-        <f>B112/B101</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
+      <c r="B134" s="26">
+        <f>B131/B116</f>
+        <v>0.42357863133370427</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
         <v>142</v>
       </c>
-      <c r="B116" s="26">
-        <f>B111/_VplRd</f>
-        <v>9.794237441561271E-2</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
+      <c r="B135" s="26">
+        <f>B130/_VplRd</f>
+        <v>0.15553410690190103</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
         <v>149</v>
       </c>
-      <c r="B117" s="32">
+      <c r="B136" s="32">
         <v>492.5</v>
       </c>
-      <c r="C117" s="24" t="s">
+      <c r="C136" s="24" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
         <v>150</v>
       </c>
-      <c r="B118" s="26">
-        <f>B112/B117</f>
-        <v>0.65599959693508958</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
+      <c r="B137" s="26">
+        <f>B131/B136</f>
+        <v>1.0236613989655465</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
         <v>143</v>
       </c>
-      <c r="B119" s="3">
-        <f>5*B104*(_L*1000)^4/(384*210000*47199*10^(4))</f>
+      <c r="B138" s="3">
+        <f>5*B119*(_L*1000)^4/(384*210000*47199*10^(4))</f>
         <v>31.033025872841279</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>215</v>
+      </c>
+      <c r="B139" s="26">
+        <f>5*2.5*(_L*1000)^4/(384*210000*99895*10^(4))</f>
+        <v>3.7883997101966984</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>216</v>
+      </c>
+      <c r="B140" s="26">
+        <f>5*6.25*(_L*1000)^4/(384*210000*142875*10^(4))</f>
+        <v>6.6219105695555411</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
         <v>144</v>
       </c>
-      <c r="B120" s="33">
+      <c r="B141" s="33">
         <v>6.476</v>
       </c>
-      <c r="C120" s="24" t="s">
+      <c r="C141" s="24" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>217</v>
+      </c>
+      <c r="B142" s="33">
+        <f>112.5*_L^2/(8*210000*101577)*10^8</f>
+        <v>10.300727175302621</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
         <v>146</v>
       </c>
-      <c r="B121" s="3">
-        <f>B119+B120</f>
+      <c r="B143" s="3">
+        <f>B138+B141</f>
         <v>37.509025872841278</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
         <v>147</v>
       </c>
-      <c r="B122">
-        <f>B119+0.2*B120</f>
-        <v>32.32822587284128</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
+      <c r="B144">
+        <f>B138+B139+0.2*B141</f>
+        <v>36.11662558303798</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
         <v>148</v>
       </c>
-      <c r="B123">
-        <f>PI()/2*SQRT(210*52998*10/(B104*1000/9.81*_L*_L^4))</f>
-        <v>0.95514662218841706</v>
+      <c r="B145">
+        <f>PI()/2*SQRT(210*142677*10/(B119*1000/9.81*_L*_L^4))</f>
+        <v>1.5671742538677766</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="147" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A147" s="34" t="s">
+        <v>207</v>
+      </c>
+      <c r="B147" s="35"/>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>209</v>
+      </c>
+      <c r="B148" s="3">
+        <f>_nr*H22/(2*_ep/1000)</f>
+        <v>180.76620113283414</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>208</v>
+      </c>
+      <c r="B149" s="26">
+        <f>B148/1000/(_tc/1000)</f>
+        <v>2.2044658674735871</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>210</v>
+      </c>
+      <c r="B150" s="33">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>212</v>
+      </c>
+      <c r="B151" s="14">
+        <f>0.6*(1-_fck_dalle/250)</f>
+        <v>0.54</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>211</v>
+      </c>
+      <c r="B152" s="26">
+        <f>B151*_fck_dalle/1.5*SIN(RADIANS(B150))*COS(RADIANS(B150))</f>
+        <v>3.6405764746872631</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>213</v>
+      </c>
+      <c r="B153" s="26">
+        <f>B149/B152</f>
+        <v>0.60552659250564367</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>214</v>
+      </c>
+      <c r="B154" s="26">
+        <f>B149*_tc*TAN(RADIANS(B150))/(500/1.15)*10</f>
+        <v>2.1184145373689756</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="E53:F53"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A92:B92"/>
-    <mergeCell ref="A103:B103"/>
-    <mergeCell ref="A114:B114"/>
+  <mergeCells count="15">
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="A85:B85"/>
+    <mergeCell ref="A147:B147"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="D15:E15"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="E53:F53"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="A101:B101"/>
+    <mergeCell ref="A118:B118"/>
+    <mergeCell ref="A133:B133"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E16">

</xml_diff>

<commit_message>
Cas test poutre acier continue
</commit_message>
<xml_diff>
--- a/Manuel Validation/Cas tests références.xlsx
+++ b/Manuel Validation/Cas tests références.xlsx
@@ -9,17 +9,20 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15300" windowHeight="4260" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15300" windowHeight="4260" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Cas 2" sheetId="1" r:id="rId1"/>
     <sheet name="Cas 3" sheetId="2" r:id="rId2"/>
+    <sheet name="Cas 5" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_A" localSheetId="0">'Cas 2'!$B$32</definedName>
     <definedName name="_A" localSheetId="1">'Cas 3'!$B$33</definedName>
+    <definedName name="_A" localSheetId="2">'Cas 5'!$B$11</definedName>
     <definedName name="_A0" localSheetId="0">'Cas 2'!$B$75</definedName>
     <definedName name="_A0" localSheetId="1">'Cas 3'!#REF!</definedName>
+    <definedName name="_Ac" localSheetId="2">'Cas 5'!$H$5</definedName>
     <definedName name="_Ace" localSheetId="0">'Cas 2'!$E$4</definedName>
     <definedName name="_Ace" localSheetId="1">'Cas 3'!$E$4</definedName>
     <definedName name="_Acr" localSheetId="0">'Cas 2'!$B$71</definedName>
@@ -28,8 +31,12 @@
     <definedName name="_As_inf" localSheetId="1">'Cas 3'!$E$10</definedName>
     <definedName name="_Av" localSheetId="0">'Cas 2'!$B$33</definedName>
     <definedName name="_Av" localSheetId="1">'Cas 3'!$B$34</definedName>
+    <definedName name="_Av" localSheetId="2">'Cas 5'!$B$12</definedName>
     <definedName name="_b" localSheetId="0">'Cas 2'!$B$4</definedName>
     <definedName name="_b" localSheetId="1">'Cas 3'!$B$15</definedName>
+    <definedName name="_b" localSheetId="2">'Cas 5'!$E$3</definedName>
+    <definedName name="_b_Droite" localSheetId="2">'Cas 5'!$B$7</definedName>
+    <definedName name="_b_Gauche" localSheetId="2">'Cas 5'!$B$6</definedName>
     <definedName name="_B0" localSheetId="0">'Cas 2'!$B$76</definedName>
     <definedName name="_B0" localSheetId="1">'Cas 3'!#REF!</definedName>
     <definedName name="_bb" localSheetId="0">'Cas 2'!$E$21</definedName>
@@ -50,8 +57,10 @@
     <definedName name="_bt" localSheetId="0">'Cas 2'!$E$20</definedName>
     <definedName name="_cf" localSheetId="0">'Cas 2'!$B$11</definedName>
     <definedName name="_cf" localSheetId="1">'Cas 3'!$B$22</definedName>
+    <definedName name="_cf" localSheetId="2">'Cas 5'!$E$12</definedName>
     <definedName name="_cw" localSheetId="0">'Cas 2'!$B$12</definedName>
     <definedName name="_cw" localSheetId="1">'Cas 3'!$B$23</definedName>
+    <definedName name="_cw" localSheetId="2">'Cas 5'!$E$13</definedName>
     <definedName name="_d" localSheetId="0">'Cas 2'!$H$13</definedName>
     <definedName name="_dsc" localSheetId="1">'Cas 3'!$H$14</definedName>
     <definedName name="_dw" localSheetId="0">'Cas 2'!$B$9</definedName>
@@ -62,6 +71,7 @@
     <definedName name="_ep" localSheetId="1">'Cas 3'!$E$19</definedName>
     <definedName name="_epsilon" localSheetId="0">'Cas 2'!$B$15</definedName>
     <definedName name="_epsilon" localSheetId="1">'Cas 3'!$B$26</definedName>
+    <definedName name="_epsilon" localSheetId="2">'Cas 5'!$E$16</definedName>
     <definedName name="_eta" localSheetId="1">'Cas 3'!$H$28</definedName>
     <definedName name="_fck_dalle" localSheetId="0">'Cas 2'!$H$5</definedName>
     <definedName name="_fck_dalle" localSheetId="1">'Cas 3'!$H$5</definedName>
@@ -76,11 +86,13 @@
     <definedName name="_fusc" localSheetId="1">'Cas 3'!$H$15</definedName>
     <definedName name="_fy" localSheetId="0">'Cas 2'!$B$14</definedName>
     <definedName name="_fy" localSheetId="1">'Cas 3'!$B$25</definedName>
+    <definedName name="_fy" localSheetId="2">'Cas 5'!$E$15</definedName>
     <definedName name="_fyd" localSheetId="0">'Cas 2'!$E$12</definedName>
     <definedName name="_fyd" localSheetId="1">'Cas 3'!$E$12</definedName>
     <definedName name="_fyp" localSheetId="0">'Cas 2'!$E$24</definedName>
     <definedName name="_h" localSheetId="0">'Cas 2'!$B$3</definedName>
     <definedName name="_h" localSheetId="1">'Cas 3'!$B$14</definedName>
+    <definedName name="_h" localSheetId="2">'Cas 5'!$E$2</definedName>
     <definedName name="_hp" localSheetId="0">'Cas 2'!$E$17</definedName>
     <definedName name="_hp" localSheetId="1">'Cas 3'!$E$17</definedName>
     <definedName name="_hpg" localSheetId="0">'Cas 2'!$E$18</definedName>
@@ -88,15 +100,22 @@
     <definedName name="_hsc" localSheetId="1">'Cas 3'!$H$13</definedName>
     <definedName name="_hw" localSheetId="0">'Cas 2'!$B$8</definedName>
     <definedName name="_hw" localSheetId="1">'Cas 3'!$B$19</definedName>
+    <definedName name="_hw" localSheetId="2">'Cas 5'!$E$9</definedName>
     <definedName name="_Iy" localSheetId="0">'Cas 2'!$B$34</definedName>
     <definedName name="_Iy" localSheetId="1">'Cas 3'!$B$35</definedName>
+    <definedName name="_Iy" localSheetId="2">'Cas 5'!$B$13</definedName>
     <definedName name="_Iz" localSheetId="0">'Cas 2'!$B$35</definedName>
+    <definedName name="_Iz" localSheetId="2">'Cas 5'!$B$14</definedName>
     <definedName name="_kr" localSheetId="0">'Cas 2'!$B$72</definedName>
     <definedName name="_kr" localSheetId="1">'Cas 3'!#REF!</definedName>
     <definedName name="_kt" localSheetId="1">'Cas 3'!$H$21</definedName>
     <definedName name="_kt_max" localSheetId="1">'Cas 3'!$H$20</definedName>
     <definedName name="_L" localSheetId="0">'Cas 2'!$B$2</definedName>
     <definedName name="_L" localSheetId="1">'Cas 3'!$B$2</definedName>
+    <definedName name="_L_ConsoleD" localSheetId="2">'Cas 5'!$B$4</definedName>
+    <definedName name="_L_ConsoleG" localSheetId="2">'Cas 5'!$B$2</definedName>
+    <definedName name="_L_tot" localSheetId="2">'Cas 5'!$B$5</definedName>
+    <definedName name="_L_Travee" localSheetId="2">'Cas 5'!$B$3</definedName>
     <definedName name="_Mel_y_Rd" localSheetId="0">'Cas 2'!$B$53</definedName>
     <definedName name="_Mel_z_Rd" localSheetId="0">'Cas 2'!$B$54</definedName>
     <definedName name="_Mpl_y_Rd" localSheetId="0">'Cas 2'!$B$55</definedName>
@@ -121,27 +140,39 @@
     <definedName name="_qProfile" localSheetId="1">'Cas 3'!$B$29</definedName>
     <definedName name="_r" localSheetId="0">'Cas 2'!$B$7</definedName>
     <definedName name="_r" localSheetId="1">'Cas 3'!$B$18</definedName>
+    <definedName name="_r" localSheetId="2">'Cas 5'!$E$8</definedName>
     <definedName name="_rho" localSheetId="0">'Cas 2'!$B$17</definedName>
     <definedName name="_rho" localSheetId="1">'Cas 3'!$B$28</definedName>
+    <definedName name="_rhoA" localSheetId="2">'Cas 5'!$E$18</definedName>
+    <definedName name="_rhoC" localSheetId="2">'Cas 5'!$H$6</definedName>
     <definedName name="_tc" localSheetId="0">'Cas 2'!$H$4</definedName>
     <definedName name="_tc" localSheetId="1">'Cas 3'!$H$4</definedName>
     <definedName name="_td" localSheetId="0">'Cas 2'!$H$3</definedName>
     <definedName name="_td" localSheetId="1">'Cas 3'!$H$3</definedName>
+    <definedName name="_td" localSheetId="2">'Cas 5'!$H$2</definedName>
     <definedName name="_tf" localSheetId="0">'Cas 2'!$B$5</definedName>
     <definedName name="_tf" localSheetId="1">'Cas 3'!$B$16</definedName>
+    <definedName name="_tf" localSheetId="2">'Cas 5'!$E$4</definedName>
+    <definedName name="_th" localSheetId="2">'Cas 5'!$H$3</definedName>
+    <definedName name="_theta" localSheetId="2">'Cas 5'!$H$4</definedName>
     <definedName name="_tp" localSheetId="0">'Cas 2'!$E$23</definedName>
     <definedName name="_tw" localSheetId="0">'Cas 2'!$B$6</definedName>
     <definedName name="_tw" localSheetId="1">'Cas 3'!$B$17</definedName>
+    <definedName name="_tw" localSheetId="2">'Cas 5'!$E$5</definedName>
     <definedName name="_VplRd" localSheetId="0">'Cas 2'!$B$52</definedName>
     <definedName name="_VplRd" localSheetId="1">'Cas 3'!$B$53</definedName>
     <definedName name="_Wel_y" localSheetId="0">'Cas 2'!$B$36</definedName>
     <definedName name="_Wel_y" localSheetId="1">'Cas 3'!$B$37</definedName>
+    <definedName name="_Wel_y" localSheetId="2">'Cas 5'!$B$15</definedName>
     <definedName name="_Wel_z" localSheetId="0">'Cas 2'!$B$37</definedName>
     <definedName name="_Wel_z" localSheetId="1">'Cas 3'!$B$38</definedName>
+    <definedName name="_Wel_z" localSheetId="2">'Cas 5'!$B$16</definedName>
     <definedName name="_Wpl_y" localSheetId="0">'Cas 2'!$B$38</definedName>
     <definedName name="_Wpl_y" localSheetId="1">'Cas 3'!$B$39</definedName>
+    <definedName name="_Wpl_y" localSheetId="2">'Cas 5'!$B$17</definedName>
     <definedName name="_Wpl_z" localSheetId="0">'Cas 2'!$B$39</definedName>
     <definedName name="_Wpl_z" localSheetId="1">'Cas 3'!$B$40</definedName>
+    <definedName name="_Wpl_z" localSheetId="2">'Cas 5'!$B$18</definedName>
     <definedName name="_za" localSheetId="0">'Cas 2'!$B$74</definedName>
     <definedName name="_za" localSheetId="1">'Cas 3'!$B$73</definedName>
     <definedName name="_zcr" localSheetId="0">'Cas 2'!$B$73</definedName>
@@ -165,7 +196,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="237">
   <si>
     <t>h (mm)</t>
   </si>
@@ -819,6 +850,63 @@
   </si>
   <si>
     <t>f (SHC) (mm)</t>
+  </si>
+  <si>
+    <t>L_ConsoleG (m)</t>
+  </si>
+  <si>
+    <t>L_travée (m)</t>
+  </si>
+  <si>
+    <t>L_ConsoleD (m)</t>
+  </si>
+  <si>
+    <t>Données profil acier</t>
+  </si>
+  <si>
+    <t>L tot (m)</t>
+  </si>
+  <si>
+    <t>bGauche (m)</t>
+  </si>
+  <si>
+    <t>bDroite (m)</t>
+  </si>
+  <si>
+    <t>th (mm)</t>
+  </si>
+  <si>
+    <t>Ac (mm2)</t>
+  </si>
+  <si>
+    <t>rho c (kg/m3)</t>
+  </si>
+  <si>
+    <t>V(G) (kN)</t>
+  </si>
+  <si>
+    <t>M(G) (kN.m)</t>
+  </si>
+  <si>
+    <t>V(Q1#1) (kN)</t>
+  </si>
+  <si>
+    <t>résultats obtenus sur RDM7</t>
+  </si>
+  <si>
+    <t>M(Q1#1) (kN.m)</t>
+  </si>
+  <si>
+    <t>V(Q1#2) (kN)</t>
+  </si>
+  <si>
+    <t>M(Q1#2) (kN.m)</t>
+  </si>
+  <si>
+    <t>V(Q1#3) (kN)</t>
+  </si>
+  <si>
+    <t>M(Q1#3) (kN.m)</t>
   </si>
 </sst>
 </file>
@@ -1098,6 +1186,24 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1110,29 +1216,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1427,20 +1515,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="35"/>
+      <c r="B1" s="51"/>
       <c r="C1"/>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="50" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="35"/>
+      <c r="E1" s="51"/>
       <c r="F1" s="24"/>
-      <c r="G1" s="34" t="s">
+      <c r="G1" s="50" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="35"/>
+      <c r="H1" s="51"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -1702,10 +1790,10 @@
         <v>0.81361651346682706</v>
       </c>
       <c r="C15"/>
-      <c r="D15" s="34" t="s">
+      <c r="D15" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="35"/>
+      <c r="E15" s="51"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B16" s="6"/>
@@ -1844,10 +1932,10 @@
       <c r="C29"/>
     </row>
     <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="34" t="s">
+      <c r="A30" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="35"/>
+      <c r="B30" s="51"/>
       <c r="C30" s="24" t="s">
         <v>53</v>
       </c>
@@ -2115,10 +2203,10 @@
       </c>
     </row>
     <row r="50" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="34" t="s">
+      <c r="A50" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="B50" s="35"/>
+      <c r="B50" s="51"/>
       <c r="D50" s="26" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2155,10 +2243,10 @@
         <f t="shared" si="0"/>
         <v>0.41222226735473377</v>
       </c>
-      <c r="E52" s="36" t="s">
+      <c r="E52" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="F52" s="37"/>
+      <c r="F52" s="53"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -2406,10 +2494,10 @@
       </c>
     </row>
     <row r="68" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="34" t="s">
+      <c r="A68" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="B68" s="35"/>
+      <c r="B68" s="51"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
@@ -2693,10 +2781,10 @@
     </row>
     <row r="95" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="96" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="34" t="s">
+      <c r="A96" s="50" t="s">
         <v>111</v>
       </c>
-      <c r="B96" s="35"/>
+      <c r="B96" s="51"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
@@ -2800,10 +2888,10 @@
     </row>
     <row r="108" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="109" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="34" t="s">
+      <c r="A109" s="50" t="s">
         <v>133</v>
       </c>
-      <c r="B109" s="35"/>
+      <c r="B109" s="51"/>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
@@ -2886,10 +2974,10 @@
     </row>
     <row r="119" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="120" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="34" t="s">
+      <c r="A120" s="50" t="s">
         <v>134</v>
       </c>
-      <c r="B120" s="35"/>
+      <c r="B120" s="51"/>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
@@ -3014,20 +3102,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="50" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="35"/>
+      <c r="B1" s="51"/>
       <c r="C1"/>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="50" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="35"/>
+      <c r="E1" s="51"/>
       <c r="F1" s="24"/>
-      <c r="G1" s="34" t="s">
+      <c r="G1" s="50" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="35"/>
+      <c r="H1" s="51"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -3262,16 +3350,16 @@
         <f>500/1.15</f>
         <v>434.78260869565219</v>
       </c>
-      <c r="G12" s="34" t="s">
+      <c r="G12" s="50" t="s">
         <v>162</v>
       </c>
-      <c r="H12" s="35"/>
+      <c r="H12" s="51"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="34" t="s">
+      <c r="A13" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="35"/>
+      <c r="B13" s="51"/>
       <c r="C13"/>
       <c r="D13" t="s">
         <v>125</v>
@@ -3310,10 +3398,10 @@
         <v>200</v>
       </c>
       <c r="C15"/>
-      <c r="D15" s="34" t="s">
+      <c r="D15" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="35"/>
+      <c r="E15" s="51"/>
       <c r="G15" t="s">
         <v>166</v>
       </c>
@@ -3617,10 +3705,10 @@
       <c r="C30"/>
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="34" t="s">
+      <c r="A31" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="35"/>
+      <c r="B31" s="51"/>
       <c r="C31" s="24" t="s">
         <v>53</v>
       </c>
@@ -3888,10 +3976,10 @@
       </c>
     </row>
     <row r="51" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="34" t="s">
+      <c r="A51" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="B51" s="35"/>
+      <c r="B51" s="51"/>
       <c r="D51" s="26" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3928,10 +4016,10 @@
         <f t="shared" si="0"/>
         <v>0.41222226735473377</v>
       </c>
-      <c r="E53" s="36" t="s">
+      <c r="E53" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="F53" s="37"/>
+      <c r="F53" s="53"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
@@ -4179,10 +4267,10 @@
       </c>
     </row>
     <row r="69" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="34" t="s">
+      <c r="A69" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="B69" s="35"/>
+      <c r="B69" s="51"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
@@ -4204,10 +4292,10 @@
       <c r="A72" t="s">
         <v>191</v>
       </c>
-      <c r="B72" s="47" t="s">
+      <c r="B72" s="43" t="s">
         <v>189</v>
       </c>
-      <c r="C72" s="48" t="s">
+      <c r="C72" s="44" t="s">
         <v>190</v>
       </c>
     </row>
@@ -4215,11 +4303,11 @@
       <c r="A73" t="s">
         <v>87</v>
       </c>
-      <c r="B73" s="39">
+      <c r="B73" s="35">
         <f>_td+_h/2</f>
         <v>388.5</v>
       </c>
-      <c r="C73" s="46">
+      <c r="C73" s="42">
         <f>_za</f>
         <v>388.5</v>
       </c>
@@ -4228,11 +4316,11 @@
       <c r="A74" t="s">
         <v>184</v>
       </c>
-      <c r="B74" s="39">
+      <c r="B74" s="35">
         <f>_td+_zs_inf</f>
         <v>562.5</v>
       </c>
-      <c r="C74" s="46">
+      <c r="C74" s="42">
         <f>_zs</f>
         <v>562.5</v>
       </c>
@@ -4241,10 +4329,10 @@
       <c r="A75" t="s">
         <v>88</v>
       </c>
-      <c r="B75" s="42" t="s">
+      <c r="B75" s="38" t="s">
         <v>192</v>
       </c>
-      <c r="C75" s="44">
+      <c r="C75" s="40">
         <f>_A*100+_As_inf*100+_beff_mi_travee*1000*_tc/_n_dalle</f>
         <v>18591.646270893973</v>
       </c>
@@ -4253,10 +4341,10 @@
       <c r="A76" t="s">
         <v>193</v>
       </c>
-      <c r="B76" s="42" t="s">
+      <c r="B76" s="38" t="s">
         <v>192</v>
       </c>
-      <c r="C76" s="45">
+      <c r="C76" s="41">
         <f>_Ace*100/(B71*_hw)</f>
         <v>7.7225855565936534</v>
       </c>
@@ -4265,10 +4353,10 @@
       <c r="A77" t="s">
         <v>194</v>
       </c>
-      <c r="B77" s="42" t="s">
+      <c r="B77" s="38" t="s">
         <v>192</v>
       </c>
-      <c r="C77" s="44">
+      <c r="C77" s="40">
         <f>_A*100*(_h/2-_tf)+_As_inf*100*(_zs_inf-_tf)+_beff_mi_travee*1000*_tc/_n_dalle*(_tc/2-_tf-_td)</f>
         <v>1580410.56741363</v>
       </c>
@@ -4277,10 +4365,10 @@
       <c r="A78" t="s">
         <v>195</v>
       </c>
-      <c r="B78" s="43" t="s">
+      <c r="B78" s="39" t="s">
         <v>192</v>
       </c>
-      <c r="C78" s="44">
+      <c r="C78" s="40">
         <f>C75/C76*(-1+SQRT(1+2*C77*C76/C75^2))</f>
         <v>83.556465257011979</v>
       </c>
@@ -4289,11 +4377,11 @@
       <c r="A79" t="s">
         <v>90</v>
       </c>
-      <c r="B79" s="51">
+      <c r="B79" s="45">
         <f>(_beff_mi_travee*1000*_tc^2/(2*_n_dalle)+_A*100*_za+_As_inf*100*_zs)/(_beff_mi_travee*1000*_tc/_n_dalle+_A*100+_As_inf*100)</f>
         <v>239.50648863397487</v>
       </c>
-      <c r="C79" s="52">
+      <c r="C79" s="46">
         <f>_td+_tf+C78</f>
         <v>238.05646525701198</v>
       </c>
@@ -4310,11 +4398,11 @@
       <c r="A80" t="s">
         <v>91</v>
       </c>
-      <c r="B80" s="39">
+      <c r="B80" s="35">
         <f>_tc</f>
         <v>82</v>
       </c>
-      <c r="C80" s="46">
+      <c r="C80" s="42">
         <f>_tc+_td</f>
         <v>222</v>
       </c>
@@ -4323,11 +4411,11 @@
       <c r="A81" t="s">
         <v>92</v>
       </c>
-      <c r="B81" s="39">
+      <c r="B81" s="35">
         <f>_td+_tf</f>
         <v>154.5</v>
       </c>
-      <c r="C81" s="46">
+      <c r="C81" s="42">
         <f>C80+_h</f>
         <v>719</v>
       </c>
@@ -4336,11 +4424,11 @@
       <c r="A82" t="s">
         <v>93</v>
       </c>
-      <c r="B82" s="39" t="b">
+      <c r="B82" s="35" t="b">
         <f>IF(B80&lt;=_zel,IF(_zel&lt;=B81,TRUE,FALSE),FALSE)</f>
         <v>0</v>
       </c>
-      <c r="C82" s="39" t="b">
+      <c r="C82" s="35" t="b">
         <f>IF(C80&lt;=C79,IF(C79&lt;=C81,TRUE,FALSE),FALSE)</f>
         <v>1</v>
       </c>
@@ -4349,24 +4437,24 @@
       <c r="A83" t="s">
         <v>94</v>
       </c>
-      <c r="B83" s="53">
+      <c r="B83" s="47">
         <f>(_Iy*10^4+_A*100*(_za-_zel)^2+_As_inf*100*(_zs-_zel)^2+_beff_mi_travee*1000*_tc/_n_dalle*(_tc^2/12+(_tc/2-_zel)^2))*10^(-4)</f>
         <v>101421.8641875779</v>
       </c>
-      <c r="C83" s="54">
+      <c r="C83" s="48">
         <f>(_Iy*10^4+_A*100*(_za-C79)^2+_As_inf*100*(_zs-C79)^2+_beff_mi_travee*1000*_tc/_n_dalle*(_tc^2/12+(_tc/2-C79)^2)+(_bc-_tw)*C78^3/(3*B71))*10^(-4)</f>
         <v>101576.61353768932</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B84" s="41"/>
-      <c r="C84" s="40"/>
+      <c r="B84" s="37"/>
+      <c r="C84" s="36"/>
     </row>
     <row r="85" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="49" t="s">
+      <c r="A85" s="54" t="s">
         <v>188</v>
       </c>
-      <c r="B85" s="50"/>
+      <c r="B85" s="55"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
@@ -4426,7 +4514,7 @@
       <c r="A91" t="s">
         <v>102</v>
       </c>
-      <c r="B91" s="38">
+      <c r="B91" s="34">
         <f>16.8/SQRT(_fcm_enrobage)</f>
         <v>2.9245046200557239</v>
       </c>
@@ -4509,16 +4597,16 @@
     </row>
     <row r="100" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="101" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="34" t="s">
+      <c r="A101" s="50" t="s">
         <v>111</v>
       </c>
-      <c r="B101" s="35"/>
+      <c r="B101" s="51"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="B102" s="55">
+      <c r="B102" s="49">
         <f>_tf*_b*_fy/1000</f>
         <v>1029.5</v>
       </c>
@@ -4652,10 +4740,10 @@
     </row>
     <row r="117" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="118" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="34" t="s">
+      <c r="A118" s="50" t="s">
         <v>133</v>
       </c>
-      <c r="B118" s="35"/>
+      <c r="B118" s="51"/>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
@@ -4774,10 +4862,10 @@
     </row>
     <row r="132" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="133" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A133" s="34" t="s">
+      <c r="A133" s="50" t="s">
         <v>134</v>
       </c>
-      <c r="B133" s="35"/>
+      <c r="B133" s="51"/>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
@@ -4893,10 +4981,10 @@
     </row>
     <row r="146" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="147" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="34" t="s">
+      <c r="A147" s="50" t="s">
         <v>207</v>
       </c>
-      <c r="B147" s="35"/>
+      <c r="B147" s="51"/>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
@@ -4962,16 +5050,16 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="D15:E15"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A51:B51"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="A85:B85"/>
     <mergeCell ref="A147:B147"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="D15:E15"/>
     <mergeCell ref="E53:F53"/>
     <mergeCell ref="A69:B69"/>
     <mergeCell ref="A101:B101"/>
@@ -4986,4 +5074,628 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H56"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="50" t="s">
+        <v>152</v>
+      </c>
+      <c r="B1" s="51"/>
+      <c r="D1" s="50" t="s">
+        <v>221</v>
+      </c>
+      <c r="E1" s="51"/>
+      <c r="G1" s="50" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="51"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="B2" s="10">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <v>497</v>
+      </c>
+      <c r="G2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B3" s="1">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1">
+        <v>200</v>
+      </c>
+      <c r="G3" t="s">
+        <v>225</v>
+      </c>
+      <c r="H3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>220</v>
+      </c>
+      <c r="B4" s="1">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="1">
+        <v>14.5</v>
+      </c>
+      <c r="G4" t="s">
+        <v>210</v>
+      </c>
+      <c r="H4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>222</v>
+      </c>
+      <c r="B5" s="1">
+        <f>_L_ConsoleG+_L_Travee+_L_ConsoleD</f>
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="1">
+        <v>8.4</v>
+      </c>
+      <c r="G5" t="s">
+        <v>226</v>
+      </c>
+      <c r="H5" s="23">
+        <f>(_b_Gauche+_b_Droite)*1000/2*_td+_th*_b+_th^2*TAN(RADIANS(_theta))</f>
+        <v>248923.76043070341</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>223</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="G6" t="s">
+        <v>227</v>
+      </c>
+      <c r="H6">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>224</v>
+      </c>
+      <c r="B7" s="1">
+        <v>2</v>
+      </c>
+      <c r="E7" s="1"/>
+      <c r="G7" t="s">
+        <v>129</v>
+      </c>
+      <c r="H7" s="25">
+        <f>_rhoC*_Ac*10^(-6)*9.81/1000</f>
+        <v>6.1048552245630008</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" s="1">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="50" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="51"/>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="6">
+        <f>_h-2*_tf</f>
+        <v>468</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="8">
+        <v>174.11468914507714</v>
+      </c>
+      <c r="D10" t="s">
+        <v>113</v>
+      </c>
+      <c r="E10" s="6">
+        <f>_hw-2*_r</f>
+        <v>426</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="4">
+        <v>101.3</v>
+      </c>
+      <c r="E11" s="6"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="5">
+        <v>50.607999999999997</v>
+      </c>
+      <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="6">
+        <f>(_b-2*_r-_tw)/2</f>
+        <v>74.8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4">
+        <v>43014.311000000002</v>
+      </c>
+      <c r="D13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" s="6">
+        <f>_hw-2*_r</f>
+        <v>426</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="4">
+        <v>1939.511</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="5">
+        <v>1730.9581891348089</v>
+      </c>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="1">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="5">
+        <v>193.9511</v>
+      </c>
+      <c r="D16" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" s="14">
+        <f>SQRT(235/_fy)</f>
+        <v>0.81361651346682706</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="4">
+        <v>1949.546</v>
+      </c>
+      <c r="E17" s="6"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="4">
+        <v>301.74400000000003</v>
+      </c>
+      <c r="D18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="1">
+        <v>7850</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>124</v>
+      </c>
+      <c r="E19" s="31">
+        <f>_rhoA*_A*10^(-4)*9.81/1000</f>
+        <v>0.78009610500000004</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="9">
+        <f>_rhoA*_A/10000</f>
+        <v>79.520499999999998</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="9">
+        <f>B20*_L_tot</f>
+        <v>1272.328</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="9"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="11">
+        <f>B10*_L_tot*100</f>
+        <v>278583.50263212342</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="11">
+        <f>(B10-_b/10)*_L_tot*100</f>
+        <v>246583.50263212342</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="9"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="9">
+        <f>B10/_A*100</f>
+        <v>171.88024594775629</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="9">
+        <f>(B10-_b/10)/_A*100</f>
+        <v>152.13690932386689</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="50" t="s">
+        <v>16</v>
+      </c>
+      <c r="B29" s="51"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>17</v>
+      </c>
+      <c r="B30" s="23">
+        <f>_A*100*_fy/1000</f>
+        <v>3596.15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31" s="23">
+        <f>_Av*100*_fy/(1000*SQRT(3))</f>
+        <v>1037.2582560217745</v>
+      </c>
+      <c r="D31" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="E31" s="53"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" s="23">
+        <f>_Wel_y*1000*_fy*10^(-6)</f>
+        <v>614.49015714285713</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="E32" s="17">
+        <f>9*_epsilon</f>
+        <v>7.3225486212014435</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" s="23">
+        <f>_Wel_z*1000*_fy*10^(-6)</f>
+        <v>68.852640499999993</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="E33" s="17">
+        <f>10*_epsilon</f>
+        <v>8.1361651346682713</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" s="23">
+        <f>_Wpl_y*1000*_fy*10^(-6)</f>
+        <v>692.08882999999992</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="E34" s="18">
+        <f>14*_epsilon</f>
+        <v>11.390631188535579</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>21</v>
+      </c>
+      <c r="B35" s="23">
+        <f>_Wpl_z*1000*_fy*10^(-6)</f>
+        <v>107.11912</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D36" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="E36" s="22"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="3">
+        <f>_cf/_tf</f>
+        <v>5.1586206896551721</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E37" s="19">
+        <f>33*_epsilon</f>
+        <v>26.849344944405292</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="3">
+        <f>_cw/_tw</f>
+        <v>50.714285714285715</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="E38" s="19">
+        <f>38*_epsilon</f>
+        <v>30.917427511739429</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D39" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="E39" s="20">
+        <f>42*_epsilon</f>
+        <v>34.171893565606737</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>34</v>
+      </c>
+      <c r="B40">
+        <f>IF(B37&lt;=E32,1,IF(B37&lt;=E33,2,IF(B37&lt;=E34,3,4)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>35</v>
+      </c>
+      <c r="B41">
+        <f>IF(B38&lt;=E37,1,IF(B38&lt;=E38,2,IF(B38&lt;=E39,3,4)))</f>
+        <v>4</v>
+      </c>
+      <c r="D41" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E41" s="22"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>36</v>
+      </c>
+      <c r="B42">
+        <f>IF(B38&lt;=E42,1,IF(B38&lt;=E43,2,IF(B38&lt;=E44,3,4)))</f>
+        <v>1</v>
+      </c>
+      <c r="D42" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E42" s="19">
+        <f>72*_epsilon</f>
+        <v>58.580388969611548</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D43" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E43" s="19">
+        <f>83*_epsilon</f>
+        <v>67.530170617746649</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>52</v>
+      </c>
+      <c r="B44" s="3">
+        <f>_hw/_tw</f>
+        <v>55.714285714285715</v>
+      </c>
+      <c r="D44" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="E44" s="20">
+        <f>124*_epsilon</f>
+        <v>100.88844766988656</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>51</v>
+      </c>
+      <c r="B45" s="3">
+        <f>124*_epsilon</f>
+        <v>100.88844766988656</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="B47" s="51"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>130</v>
+      </c>
+      <c r="B48" s="25">
+        <f>H7+E19</f>
+        <v>6.8849513295630009</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>228</v>
+      </c>
+      <c r="B49" s="3">
+        <f>B48*(_L_ConsoleG+_L_Travee/2)</f>
+        <v>55.079610636504007</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>229</v>
+      </c>
+      <c r="D50" s="24" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>236</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A29:B29"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
MAJ cas test 6
</commit_message>
<xml_diff>
--- a/Manuel Validation/Cas tests références.xlsx
+++ b/Manuel Validation/Cas tests références.xlsx
@@ -9,47 +9,65 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15300" windowHeight="4260"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15300" windowHeight="4260" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Cas 2" sheetId="1" r:id="rId1"/>
     <sheet name="Cas 3" sheetId="2" r:id="rId2"/>
     <sheet name="Cas 4" sheetId="4" r:id="rId3"/>
     <sheet name="Cas 5" sheetId="3" r:id="rId4"/>
+    <sheet name="Cas 6" sheetId="6" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_A" localSheetId="0">'Cas 2'!$B$32</definedName>
     <definedName name="_A" localSheetId="1">'Cas 3'!$B$33</definedName>
     <definedName name="_A" localSheetId="3">'Cas 5'!$B$11</definedName>
+    <definedName name="_A" localSheetId="4">'Cas 6'!$B$15</definedName>
     <definedName name="_A0" localSheetId="0">'Cas 2'!$B$75</definedName>
     <definedName name="_A0" localSheetId="1">'Cas 3'!#REF!</definedName>
     <definedName name="_Ac" localSheetId="3">'Cas 5'!$H$5</definedName>
+    <definedName name="_Ac_brute" localSheetId="4">'Cas 6'!$H$5</definedName>
     <definedName name="_Ace" localSheetId="0">'Cas 2'!$E$4</definedName>
     <definedName name="_Ace" localSheetId="1">'Cas 3'!$E$4</definedName>
+    <definedName name="_Ace" localSheetId="4">'Cas 6'!$E$4</definedName>
     <definedName name="_Acr" localSheetId="0">'Cas 2'!$B$71</definedName>
     <definedName name="_Acr" localSheetId="1">'Cas 3'!#REF!</definedName>
+    <definedName name="_Ah" localSheetId="4">'Cas 6'!$B$94</definedName>
     <definedName name="_As_inf" localSheetId="0">'Cas 2'!$E$10</definedName>
     <definedName name="_As_inf" localSheetId="1">'Cas 3'!$E$10</definedName>
+    <definedName name="_As_inf" localSheetId="4">'Cas 6'!$E$10</definedName>
     <definedName name="_Av" localSheetId="0">'Cas 2'!$B$33</definedName>
     <definedName name="_Av" localSheetId="1">'Cas 3'!$B$34</definedName>
     <definedName name="_Av" localSheetId="3">'Cas 5'!$B$12</definedName>
+    <definedName name="_Av" localSheetId="4">'Cas 6'!$B$16</definedName>
     <definedName name="_b" localSheetId="0">'Cas 2'!$B$4</definedName>
     <definedName name="_b" localSheetId="1">'Cas 3'!$B$15</definedName>
     <definedName name="_b" localSheetId="3">'Cas 5'!$E$3</definedName>
     <definedName name="_b_Droite" localSheetId="3">'Cas 5'!$B$7</definedName>
+    <definedName name="_b_Droite" localSheetId="4">'Cas 6'!$B$4</definedName>
     <definedName name="_b_Gauche" localSheetId="3">'Cas 5'!$B$6</definedName>
+    <definedName name="_b_Gauche" localSheetId="4">'Cas 6'!$B$3</definedName>
     <definedName name="_B0" localSheetId="0">'Cas 2'!$B$76</definedName>
     <definedName name="_B0" localSheetId="1">'Cas 3'!#REF!</definedName>
     <definedName name="_bb" localSheetId="0">'Cas 2'!$E$21</definedName>
     <definedName name="_bc" localSheetId="0">'Cas 2'!$E$3</definedName>
     <definedName name="_bc" localSheetId="1">'Cas 3'!$E$3</definedName>
+    <definedName name="_bc" localSheetId="4">'Cas 6'!$E$3</definedName>
     <definedName name="_bdroite" localSheetId="1">'Cas 3'!$B$4</definedName>
     <definedName name="_be1" localSheetId="1">'Cas 3'!$B$6</definedName>
+    <definedName name="_be1" localSheetId="4">'Cas 6'!$B$3</definedName>
     <definedName name="_be2" localSheetId="1">'Cas 3'!$B$7</definedName>
+    <definedName name="_be2" localSheetId="4">'Cas 6'!$B$4</definedName>
+    <definedName name="_beff" localSheetId="4">'Cas 6'!$B$90</definedName>
     <definedName name="_beff_appui" localSheetId="1">'Cas 3'!$B$11</definedName>
     <definedName name="_beff_mi_travee" localSheetId="1">'Cas 3'!$B$10</definedName>
+    <definedName name="_beff_mi_travee" localSheetId="4">'Cas 6'!$B$10</definedName>
     <definedName name="_beta1" localSheetId="1">'Cas 3'!$B$8</definedName>
+    <definedName name="_beta1" localSheetId="4">'Cas 6'!$B$8</definedName>
     <definedName name="_beta2" localSheetId="1">'Cas 3'!$B$9</definedName>
+    <definedName name="_beta2" localSheetId="4">'Cas 6'!$B$9</definedName>
+    <definedName name="_bfi">'Cas 6'!$E$5</definedName>
+    <definedName name="_bfs" localSheetId="4">'Cas 6'!$E$3</definedName>
     <definedName name="_bgauche" localSheetId="1">'Cas 3'!$B$3</definedName>
     <definedName name="_bm" localSheetId="0">'Cas 2'!$E$22</definedName>
     <definedName name="_bm" localSheetId="1">'Cas 3'!$E$22</definedName>
@@ -59,79 +77,102 @@
     <definedName name="_cf" localSheetId="0">'Cas 2'!$B$11</definedName>
     <definedName name="_cf" localSheetId="1">'Cas 3'!$B$22</definedName>
     <definedName name="_cf" localSheetId="3">'Cas 5'!$E$12</definedName>
+    <definedName name="_cf_sup" localSheetId="4">'Cas 6'!$E$12</definedName>
     <definedName name="_cw" localSheetId="0">'Cas 2'!$B$12</definedName>
     <definedName name="_cw" localSheetId="1">'Cas 3'!$B$23</definedName>
     <definedName name="_cw" localSheetId="3">'Cas 5'!$E$13</definedName>
+    <definedName name="_cw" localSheetId="4">'Cas 6'!$E$13</definedName>
     <definedName name="_d" localSheetId="0">'Cas 2'!$H$13</definedName>
     <definedName name="_dsc" localSheetId="1">'Cas 3'!$H$14</definedName>
+    <definedName name="_dsc" localSheetId="4">'Cas 6'!$H$16</definedName>
     <definedName name="_dw" localSheetId="0">'Cas 2'!$B$9</definedName>
     <definedName name="_dw" localSheetId="1">'Cas 3'!$B$20</definedName>
     <definedName name="_Ecm_dalle" localSheetId="0">'Cas 2'!$H$8</definedName>
     <definedName name="_Ecm_dalle" localSheetId="1">'Cas 3'!$H$8</definedName>
+    <definedName name="_Ecm_dalle" localSheetId="4">'Cas 6'!$H$10</definedName>
     <definedName name="_ep" localSheetId="0">'Cas 2'!$E$19</definedName>
     <definedName name="_ep" localSheetId="1">'Cas 3'!$E$19</definedName>
     <definedName name="_epsilon" localSheetId="0">'Cas 2'!$B$15</definedName>
     <definedName name="_epsilon" localSheetId="1">'Cas 3'!$B$26</definedName>
     <definedName name="_epsilon" localSheetId="3">'Cas 5'!$E$16</definedName>
+    <definedName name="_epsilon" localSheetId="4">'Cas 6'!$E$16</definedName>
     <definedName name="_eta" localSheetId="1">'Cas 3'!$H$28</definedName>
     <definedName name="_fck_dalle" localSheetId="0">'Cas 2'!$H$5</definedName>
     <definedName name="_fck_dalle" localSheetId="1">'Cas 3'!$H$5</definedName>
+    <definedName name="_fck_dalle" localSheetId="4">'Cas 6'!$H$7</definedName>
     <definedName name="_fck_enrobage" localSheetId="0">'Cas 2'!$E$6</definedName>
     <definedName name="_fck_enrobage" localSheetId="1">'Cas 3'!$E$6</definedName>
     <definedName name="_fcm_dalle" localSheetId="0">'Cas 2'!$H$6</definedName>
+    <definedName name="_fcm_dalle" localSheetId="4">'Cas 6'!$H$8</definedName>
     <definedName name="_fcm_enrobage" localSheetId="0">'Cas 2'!$E$7</definedName>
     <definedName name="_fcm_enrobage" localSheetId="1">'Cas 3'!$E$7</definedName>
     <definedName name="_fctm_dalle" localSheetId="0">'Cas 2'!$H$7</definedName>
+    <definedName name="_fctm_dalle" localSheetId="4">'Cas 6'!$H$9</definedName>
     <definedName name="_fctm_enrobage" localSheetId="0">'Cas 2'!$E$8</definedName>
     <definedName name="_fusc" localSheetId="0">'Cas 2'!$H$14</definedName>
     <definedName name="_fusc" localSheetId="1">'Cas 3'!$H$15</definedName>
+    <definedName name="_fusc" localSheetId="4">'Cas 6'!$H$17</definedName>
     <definedName name="_fy" localSheetId="0">'Cas 2'!$B$14</definedName>
     <definedName name="_fy" localSheetId="1">'Cas 3'!$B$25</definedName>
     <definedName name="_fy" localSheetId="3">'Cas 5'!$E$15</definedName>
+    <definedName name="_fy" localSheetId="4">'Cas 6'!$E$15</definedName>
     <definedName name="_fyd" localSheetId="0">'Cas 2'!$E$12</definedName>
     <definedName name="_fyd" localSheetId="1">'Cas 3'!$E$12</definedName>
     <definedName name="_fyp" localSheetId="0">'Cas 2'!$E$24</definedName>
     <definedName name="_h" localSheetId="0">'Cas 2'!$B$3</definedName>
     <definedName name="_h" localSheetId="1">'Cas 3'!$B$14</definedName>
     <definedName name="_h" localSheetId="3">'Cas 5'!$E$2</definedName>
+    <definedName name="_h" localSheetId="4">'Cas 6'!$E$2</definedName>
+    <definedName name="_h0_dalle" localSheetId="4">'Cas 6'!$H$2</definedName>
     <definedName name="_hp" localSheetId="0">'Cas 2'!$E$17</definedName>
     <definedName name="_hp" localSheetId="1">'Cas 3'!$E$17</definedName>
     <definedName name="_hpg" localSheetId="0">'Cas 2'!$E$18</definedName>
     <definedName name="_hsc" localSheetId="0">'Cas 2'!$H$12</definedName>
     <definedName name="_hsc" localSheetId="1">'Cas 3'!$H$13</definedName>
+    <definedName name="_hsc" localSheetId="4">'Cas 6'!$H$15</definedName>
     <definedName name="_hw" localSheetId="0">'Cas 2'!$B$8</definedName>
     <definedName name="_hw" localSheetId="1">'Cas 3'!$B$19</definedName>
     <definedName name="_hw" localSheetId="3">'Cas 5'!$E$9</definedName>
+    <definedName name="_hw" localSheetId="4">'Cas 6'!$E$8</definedName>
     <definedName name="_Iy" localSheetId="0">'Cas 2'!$B$34</definedName>
     <definedName name="_Iy" localSheetId="1">'Cas 3'!$B$35</definedName>
     <definedName name="_Iy" localSheetId="3">'Cas 5'!$B$13</definedName>
+    <definedName name="_Iy" localSheetId="4">'Cas 6'!$B$17</definedName>
     <definedName name="_Iz" localSheetId="0">'Cas 2'!$B$35</definedName>
     <definedName name="_Iz" localSheetId="3">'Cas 5'!$B$14</definedName>
+    <definedName name="_Iz" localSheetId="4">'Cas 6'!$B$18</definedName>
     <definedName name="_kr" localSheetId="0">'Cas 2'!$B$72</definedName>
     <definedName name="_kr" localSheetId="1">'Cas 3'!#REF!</definedName>
     <definedName name="_kt" localSheetId="1">'Cas 3'!$H$21</definedName>
     <definedName name="_kt_max" localSheetId="1">'Cas 3'!$H$20</definedName>
     <definedName name="_L" localSheetId="0">'Cas 2'!$B$2</definedName>
     <definedName name="_L" localSheetId="1">'Cas 3'!$B$2</definedName>
+    <definedName name="_L" localSheetId="4">'Cas 6'!$B$2</definedName>
     <definedName name="_L_ConsoleD" localSheetId="3">'Cas 5'!$B$4</definedName>
     <definedName name="_L_ConsoleG" localSheetId="3">'Cas 5'!$B$2</definedName>
     <definedName name="_L_tot" localSheetId="3">'Cas 5'!$B$5</definedName>
     <definedName name="_L_Travee" localSheetId="3">'Cas 5'!$B$3</definedName>
+    <definedName name="_L_Travee" localSheetId="4">'Cas 6'!$B$2</definedName>
     <definedName name="_Mel_y_Rd" localSheetId="0">'Cas 2'!$B$53</definedName>
     <definedName name="_Mel_z_Rd" localSheetId="0">'Cas 2'!$B$54</definedName>
     <definedName name="_Mpl_Rd" localSheetId="3">'Cas 5'!$B$69</definedName>
+    <definedName name="_Mpl_Rd" localSheetId="4">'Cas 6'!$B$103</definedName>
     <definedName name="_Mpl_y_Rd" localSheetId="0">'Cas 2'!$B$55</definedName>
     <definedName name="_Mpl_z_Rd" localSheetId="0">'Cas 2'!$B$56</definedName>
     <definedName name="_n" localSheetId="0">'Cas 2'!$B$69</definedName>
     <definedName name="_n_dalle" localSheetId="1">'Cas 3'!$B$70</definedName>
+    <definedName name="_n_dalle" localSheetId="4">'Cas 6'!$B$89</definedName>
     <definedName name="_n_enrobage" localSheetId="1">'Cas 3'!#REF!</definedName>
     <definedName name="_Na" localSheetId="1">'Cas 3'!$H$23</definedName>
+    <definedName name="_Na" localSheetId="4">'Cas 6'!$H$24</definedName>
     <definedName name="_Ncp" localSheetId="1">'Cas 3'!$B$104</definedName>
     <definedName name="_Nf" localSheetId="1">'Cas 3'!$B$102</definedName>
     <definedName name="_nr" localSheetId="1">'Cas 3'!$H$16</definedName>
+    <definedName name="_nr" localSheetId="4">'Cas 6'!$H$18</definedName>
     <definedName name="_Ns_inf" localSheetId="1">'Cas 3'!$H$24</definedName>
     <definedName name="_NtRd" localSheetId="0">'Cas 2'!$B$51</definedName>
     <definedName name="_Nw" localSheetId="1">'Cas 3'!$B$103</definedName>
+    <definedName name="_PRd" localSheetId="4">'Cas 6'!$H$23</definedName>
     <definedName name="_qBac" localSheetId="0">'Cas 2'!$E$26</definedName>
     <definedName name="_qBac" localSheetId="1">'Cas 3'!$E$26</definedName>
     <definedName name="_qDalle" localSheetId="0">'Cas 2'!$H$10</definedName>
@@ -143,51 +184,70 @@
     <definedName name="_r" localSheetId="0">'Cas 2'!$B$7</definedName>
     <definedName name="_r" localSheetId="1">'Cas 3'!$B$18</definedName>
     <definedName name="_r" localSheetId="3">'Cas 5'!$E$8</definedName>
+    <definedName name="_r" localSheetId="4">'Cas 6'!$E$10</definedName>
     <definedName name="_rho" localSheetId="0">'Cas 2'!$B$17</definedName>
     <definedName name="_rho" localSheetId="1">'Cas 3'!$B$28</definedName>
     <definedName name="_rhoA" localSheetId="3">'Cas 5'!$E$18</definedName>
+    <definedName name="_rhoA" localSheetId="4">'Cas 6'!$E$18</definedName>
     <definedName name="_rhoC" localSheetId="3">'Cas 5'!$H$6</definedName>
+    <definedName name="_rhoC" localSheetId="4">'Cas 6'!$H$6</definedName>
+    <definedName name="_sx" localSheetId="4">'Cas 6'!$H$19</definedName>
     <definedName name="_tc" localSheetId="0">'Cas 2'!$H$4</definedName>
     <definedName name="_tc" localSheetId="1">'Cas 3'!$H$4</definedName>
     <definedName name="_td" localSheetId="0">'Cas 2'!$H$3</definedName>
     <definedName name="_td" localSheetId="1">'Cas 3'!$H$3</definedName>
     <definedName name="_td" localSheetId="3">'Cas 5'!$H$2</definedName>
+    <definedName name="_td" localSheetId="4">'Cas 6'!$H$3</definedName>
     <definedName name="_tf" localSheetId="0">'Cas 2'!$B$5</definedName>
     <definedName name="_tf" localSheetId="1">'Cas 3'!$B$16</definedName>
     <definedName name="_tf" localSheetId="3">'Cas 5'!$E$4</definedName>
+    <definedName name="_tf" localSheetId="4">'Cas 6'!$B$16</definedName>
+    <definedName name="_tfi" localSheetId="4">'Cas 6'!$E$6</definedName>
+    <definedName name="_tfs" localSheetId="4">'Cas 6'!$E$4</definedName>
     <definedName name="_th" localSheetId="3">'Cas 5'!$H$3</definedName>
     <definedName name="_theta" localSheetId="3">'Cas 5'!$H$4</definedName>
+    <definedName name="_tj" localSheetId="4">'Cas 6'!$H$4</definedName>
     <definedName name="_tp" localSheetId="0">'Cas 2'!$E$23</definedName>
     <definedName name="_tw" localSheetId="0">'Cas 2'!$B$6</definedName>
     <definedName name="_tw" localSheetId="1">'Cas 3'!$B$17</definedName>
     <definedName name="_tw" localSheetId="3">'Cas 5'!$E$5</definedName>
+    <definedName name="_tw" localSheetId="4">'Cas 6'!$E$7</definedName>
     <definedName name="_VplRd" localSheetId="0">'Cas 2'!$B$52</definedName>
     <definedName name="_VplRd" localSheetId="1">'Cas 3'!$B$53</definedName>
     <definedName name="_VplRd" localSheetId="3">'Cas 5'!$B$52</definedName>
+    <definedName name="_VplRd" localSheetId="4">'Cas 6'!$B$56</definedName>
     <definedName name="_Wel_y" localSheetId="0">'Cas 2'!$B$36</definedName>
     <definedName name="_Wel_y" localSheetId="1">'Cas 3'!$B$37</definedName>
     <definedName name="_Wel_y" localSheetId="3">'Cas 5'!$B$15</definedName>
+    <definedName name="_Wel_y" localSheetId="4">'Cas 6'!$B$19</definedName>
     <definedName name="_Wel_z" localSheetId="0">'Cas 2'!$B$37</definedName>
     <definedName name="_Wel_z" localSheetId="1">'Cas 3'!$B$38</definedName>
     <definedName name="_Wel_z" localSheetId="3">'Cas 5'!$B$16</definedName>
+    <definedName name="_Wel_z" localSheetId="4">'Cas 6'!$B$20</definedName>
     <definedName name="_Wpl_y" localSheetId="0">'Cas 2'!$B$38</definedName>
     <definedName name="_Wpl_y" localSheetId="1">'Cas 3'!$B$39</definedName>
     <definedName name="_Wpl_y" localSheetId="3">'Cas 5'!$B$17</definedName>
+    <definedName name="_Wpl_y" localSheetId="4">'Cas 6'!$B$21</definedName>
     <definedName name="_Wpl_z" localSheetId="0">'Cas 2'!$B$39</definedName>
     <definedName name="_Wpl_z" localSheetId="1">'Cas 3'!$B$40</definedName>
     <definedName name="_Wpl_z" localSheetId="3">'Cas 5'!$B$18</definedName>
+    <definedName name="_Wpl_z" localSheetId="4">'Cas 6'!$B$22</definedName>
     <definedName name="_za" localSheetId="0">'Cas 2'!$B$74</definedName>
     <definedName name="_za" localSheetId="1">'Cas 3'!$B$73</definedName>
     <definedName name="_zcr" localSheetId="0">'Cas 2'!$B$73</definedName>
     <definedName name="_zcr" localSheetId="1">'Cas 3'!#REF!</definedName>
     <definedName name="_zel" localSheetId="0">'Cas 2'!$B$77</definedName>
     <definedName name="_zel" localSheetId="1">'Cas 3'!$B$79</definedName>
+    <definedName name="_zel" localSheetId="4">'Cas 6'!$B$79</definedName>
+    <definedName name="_zp" localSheetId="4">'Cas 6'!$B$93</definedName>
     <definedName name="_zpl" localSheetId="0">'Cas 2'!$B$102</definedName>
     <definedName name="_zpl_a" localSheetId="1">'Cas 3'!$B$107</definedName>
     <definedName name="_zpl_c" localSheetId="1">'Cas 3'!$B$105</definedName>
     <definedName name="_zs" localSheetId="1">'Cas 3'!$B$74</definedName>
+    <definedName name="_zs" localSheetId="4">'Cas 6'!$B$74</definedName>
     <definedName name="_zs_inf" localSheetId="0">'Cas 2'!$E$11</definedName>
     <definedName name="_zs_inf" localSheetId="1">'Cas 3'!$E$11</definedName>
+    <definedName name="_zs_inf" localSheetId="4">'Cas 6'!$E$11</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -199,7 +259,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="674" uniqueCount="272">
   <si>
     <t>h (mm)</t>
   </si>
@@ -976,6 +1036,45 @@
   </si>
   <si>
     <t>Sans objet, l'ensemble des résultats sont dans l'article RCM 2022 n°3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PropSection section seule </t>
+  </si>
+  <si>
+    <t>tj (mm)</t>
+  </si>
+  <si>
+    <t>Ac, brute (mm2)</t>
+  </si>
+  <si>
+    <t>sx (mm)</t>
+  </si>
+  <si>
+    <t>bfs (mm)</t>
+  </si>
+  <si>
+    <t>tfs (mm)</t>
+  </si>
+  <si>
+    <t>bfi (mm)</t>
+  </si>
+  <si>
+    <t>tfi (mm)</t>
+  </si>
+  <si>
+    <t>cf ,sup</t>
+  </si>
+  <si>
+    <t>Classe semelle sup</t>
+  </si>
+  <si>
+    <t>beff (m)</t>
+  </si>
+  <si>
+    <t>Ah (mm2)</t>
+  </si>
+  <si>
+    <t>zp (mm)</t>
   </si>
 </sst>
 </file>
@@ -1244,7 +1343,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1341,6 +1440,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -6292,4 +6404,1541 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I116"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="70" t="s">
+        <v>152</v>
+      </c>
+      <c r="B1" s="71"/>
+      <c r="D1" s="70" t="s">
+        <v>221</v>
+      </c>
+      <c r="E1" s="71"/>
+      <c r="G1" s="70" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="71"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B2" s="1">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <v>300</v>
+      </c>
+      <c r="G2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H2" s="23">
+        <f>1/(1/_td-_bfs/(2*(_b_Gauche+_b_Droite)*1000*_td))</f>
+        <v>123.71134020618557</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>223</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>263</v>
+      </c>
+      <c r="E3" s="1">
+        <v>120</v>
+      </c>
+      <c r="G3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>264</v>
+      </c>
+      <c r="E4" s="1">
+        <v>6</v>
+      </c>
+      <c r="G4" t="s">
+        <v>260</v>
+      </c>
+      <c r="H4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5">
+        <f>_L/8</f>
+        <v>1.25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>265</v>
+      </c>
+      <c r="E5" s="1">
+        <v>150</v>
+      </c>
+      <c r="G5" t="s">
+        <v>261</v>
+      </c>
+      <c r="H5" s="23">
+        <f>(_b_Gauche+_b_Droite)*1000*(_td-_tj)</f>
+        <v>220000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B6">
+        <f>MIN(_b_Gauche,B5)</f>
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>266</v>
+      </c>
+      <c r="E6" s="1">
+        <v>10.7</v>
+      </c>
+      <c r="G6" t="s">
+        <v>227</v>
+      </c>
+      <c r="H6">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B7">
+        <f>MIN(_b_Droite,B5)</f>
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="1">
+        <v>7.1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" s="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B8">
+        <f>MIN(1,0.55+0.025*_L/_be1)</f>
+        <v>0.8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="6">
+        <f>_h-_tfs-_tfi</f>
+        <v>283.3</v>
+      </c>
+      <c r="G8" t="s">
+        <v>61</v>
+      </c>
+      <c r="H8">
+        <f>_fck_dalle+8</f>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B9">
+        <f>MIN(1,0.55+0.025*_L/_be2)</f>
+        <v>0.8</v>
+      </c>
+      <c r="D9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E9" s="6">
+        <f>_hw-2*_r</f>
+        <v>283.3</v>
+      </c>
+      <c r="G9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" s="26">
+        <f>0.3*_fck_dalle^(2/3)</f>
+        <v>2.5649639200150443</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B10" s="26">
+        <f>_be1+_be2</f>
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0</v>
+      </c>
+      <c r="G10" t="s">
+        <v>64</v>
+      </c>
+      <c r="H10" s="13">
+        <f>22*(_fcm_dalle/10)^0.3*1000</f>
+        <v>31475.806210019346</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>161</v>
+      </c>
+      <c r="B11" s="26">
+        <f>_be1*_beta1+_be2*_beta2</f>
+        <v>1.6</v>
+      </c>
+      <c r="E11" s="6"/>
+      <c r="G11" t="s">
+        <v>129</v>
+      </c>
+      <c r="H11" s="25">
+        <f>_rhoC*_Ac_brute*10^(-6)*9.81/1000</f>
+        <v>5.3955000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>267</v>
+      </c>
+      <c r="E12" s="6">
+        <f>(_bfs-2*_r-_tw)/2</f>
+        <v>56.45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="70" t="s">
+        <v>259</v>
+      </c>
+      <c r="B13" s="71"/>
+      <c r="D13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" s="6">
+        <f>_hw-2*_r</f>
+        <v>283.3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="79">
+        <f>(2*(_h-2*_r)+_bfs+_bfi+(_bfs-2*_r-_tw)+(_bfi-2*_r-_tw)+2*PI()*_r)/10</f>
+        <v>112.58</v>
+      </c>
+      <c r="G14" s="70" t="s">
+        <v>162</v>
+      </c>
+      <c r="H14" s="71"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="9">
+        <f>(_bfs*_tfs+_bfi*_tfi+(_h-_tfs-_tfi)*_tw+4*(1-PI()/4)*_r^2)/100</f>
+        <v>43.3643</v>
+      </c>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="1">
+        <v>355</v>
+      </c>
+      <c r="G15" t="s">
+        <v>163</v>
+      </c>
+      <c r="H15" s="10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="64">
+        <f>((_h-_tfs-_tfi)*_tw)/100</f>
+        <v>20.1143</v>
+      </c>
+      <c r="D16" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" s="14">
+        <f>SQRT(235/_fy)</f>
+        <v>0.81361651346682706</v>
+      </c>
+      <c r="G16" t="s">
+        <v>164</v>
+      </c>
+      <c r="H16" s="10">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="4">
+        <v>5921.277</v>
+      </c>
+      <c r="E17" s="6"/>
+      <c r="G17" t="s">
+        <v>166</v>
+      </c>
+      <c r="H17" s="10">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="4">
+        <v>332.58</v>
+      </c>
+      <c r="D18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="1">
+        <v>7850</v>
+      </c>
+      <c r="G18" t="s">
+        <v>171</v>
+      </c>
+      <c r="H18" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="4">
+        <f>_Iy/(_h/10/2)</f>
+        <v>394.7518</v>
+      </c>
+      <c r="D19" t="s">
+        <v>124</v>
+      </c>
+      <c r="E19" s="31">
+        <f>_rhoA*_A*10^(-4)*9.81/1000</f>
+        <v>0.33394196965500006</v>
+      </c>
+      <c r="G19" t="s">
+        <v>262</v>
+      </c>
+      <c r="H19" s="10">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="4">
+        <v>51.758000000000003</v>
+      </c>
+      <c r="G20" t="s">
+        <v>165</v>
+      </c>
+      <c r="H20" s="3">
+        <f>0.8*_fusc*PI()*_dsc^2/4/(1000*1.25)</f>
+        <v>81.656276252105897</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="4">
+        <v>454.96199999999999</v>
+      </c>
+      <c r="G21" t="s">
+        <v>167</v>
+      </c>
+      <c r="H21" s="3">
+        <f>IF(_hsc/_dsc&gt;=4,1,FALSE)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="4">
+        <v>85.24</v>
+      </c>
+      <c r="G22" t="s">
+        <v>168</v>
+      </c>
+      <c r="H22" s="3">
+        <f>0.29*H21*_dsc^2*SQRT(_fck_dalle*_Ecm_dalle)/(1000*1.25)</f>
+        <v>74.293979654469197</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G23" t="s">
+        <v>172</v>
+      </c>
+      <c r="H23" s="26">
+        <f>MIN(H20,H22)</f>
+        <v>74.293979654469197</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="9">
+        <f>_rhoA*_A/10000</f>
+        <v>34.040975500000002</v>
+      </c>
+      <c r="G24" t="s">
+        <v>173</v>
+      </c>
+      <c r="H24" s="23">
+        <f>_A*100*_fy/1000</f>
+        <v>1539.4326500000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="9">
+        <f>B24*_L</f>
+        <v>340.40975500000002</v>
+      </c>
+      <c r="G25" t="s">
+        <v>174</v>
+      </c>
+      <c r="H25" s="23">
+        <f>0.85*_beff_mi_travee*1000*(_td-_tj)*_fck_dalle/1.5/1000</f>
+        <v>3116.6666666666665</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B26" s="9"/>
+      <c r="G26" t="s">
+        <v>179</v>
+      </c>
+      <c r="H26" s="23">
+        <f>MIN(H25,H24)</f>
+        <v>1539.4326500000002</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="11">
+        <f>B14*_L*100</f>
+        <v>112580</v>
+      </c>
+      <c r="G27" t="s">
+        <v>180</v>
+      </c>
+      <c r="H27" s="3">
+        <f>_nr*(_L*1000/2)/_sx*_PRd</f>
+        <v>1955.1047277491894</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="11">
+        <f>(B14-_bfs/10)*_L*100</f>
+        <v>100580</v>
+      </c>
+      <c r="G28" t="s">
+        <v>181</v>
+      </c>
+      <c r="H28" s="26">
+        <f>MIN(H27/H26,1)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B29" s="9"/>
+      <c r="G29" t="s">
+        <v>182</v>
+      </c>
+      <c r="H29">
+        <f>MAX(1-(355/_fy)*(0.75-0.03*_L),0.4)</f>
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="9">
+        <f>B14/_A*100</f>
+        <v>259.61447550173762</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" s="9">
+        <f>(B14-_bfs/10)/_A*100</f>
+        <v>231.9419430268677</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="33" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="70" t="s">
+        <v>16</v>
+      </c>
+      <c r="B33" s="71"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>17</v>
+      </c>
+      <c r="B34" s="23">
+        <f>_A*100*_fy/1000</f>
+        <v>1539.4326500000002</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>22</v>
+      </c>
+      <c r="B35" s="23">
+        <f>_Av*100*_fy/(1000*SQRT(3))</f>
+        <v>412.26137644441161</v>
+      </c>
+      <c r="D35" s="72" t="s">
+        <v>34</v>
+      </c>
+      <c r="E35" s="73"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>18</v>
+      </c>
+      <c r="B36" s="23">
+        <f>_Wel_y*1000*_fy*10^(-6)</f>
+        <v>140.136889</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="E36" s="17">
+        <f>9*_epsilon</f>
+        <v>7.3225486212014435</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37" s="23">
+        <f>_Wel_z*1000*_fy*10^(-6)</f>
+        <v>18.374089999999999</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="E37" s="17">
+        <f>10*_epsilon</f>
+        <v>8.1361651346682713</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" s="23">
+        <f>_Wpl_y*1000*_fy*10^(-6)</f>
+        <v>161.51150999999999</v>
+      </c>
+      <c r="D38" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="E38" s="18">
+        <f>14*_epsilon</f>
+        <v>11.390631188535579</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>21</v>
+      </c>
+      <c r="B39" s="23">
+        <f>_Wpl_z*1000*_fy*10^(-6)</f>
+        <v>30.260199999999998</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D40" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="E40" s="22"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>39</v>
+      </c>
+      <c r="B41" s="3">
+        <f>_cf_sup/_tfs</f>
+        <v>9.4083333333333332</v>
+      </c>
+      <c r="D41" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E41" s="19">
+        <f>33*_epsilon</f>
+        <v>26.849344944405292</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" s="3">
+        <f>_cw/_tw</f>
+        <v>39.901408450704231</v>
+      </c>
+      <c r="D42" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="E42" s="19">
+        <f>38*_epsilon</f>
+        <v>30.917427511739429</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D43" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="E43" s="20">
+        <f>42*_epsilon</f>
+        <v>34.171893565606737</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>268</v>
+      </c>
+      <c r="B44">
+        <f>IF(B41&lt;=E36,1,IF(B41&lt;=E37,2,IF(B41&lt;=E38,3,4)))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>35</v>
+      </c>
+      <c r="B45">
+        <f>IF(B42&lt;=E41,1,IF(B42&lt;=E42,2,IF(B42&lt;=E43,3,4)))</f>
+        <v>4</v>
+      </c>
+      <c r="D45" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E45" s="22"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>36</v>
+      </c>
+      <c r="B46">
+        <f>IF(B42&lt;=E46,1,IF(B42&lt;=E47,2,IF(B42&lt;=E48,3,4)))</f>
+        <v>1</v>
+      </c>
+      <c r="D46" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E46" s="19">
+        <f>72*_epsilon</f>
+        <v>58.580388969611548</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D47" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E47" s="19">
+        <f>83*_epsilon</f>
+        <v>67.530170617746649</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>52</v>
+      </c>
+      <c r="B48" s="3">
+        <f>_hw/_tw</f>
+        <v>39.901408450704231</v>
+      </c>
+      <c r="D48" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="E48" s="20">
+        <f>124*_epsilon</f>
+        <v>100.88844766988656</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="3">
+        <f>124*_epsilon</f>
+        <v>100.88844766988656</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="51" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="70" t="s">
+        <v>133</v>
+      </c>
+      <c r="B51" s="71"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>130</v>
+      </c>
+      <c r="B52" s="25">
+        <f>H11+E19</f>
+        <v>5.7294419696550003</v>
+      </c>
+      <c r="C52" s="26">
+        <f>B52*1.35</f>
+        <v>7.7347466590342506</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="28" t="s">
+        <v>228</v>
+      </c>
+      <c r="B53" s="53">
+        <v>34.424999999999997</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="16" t="s">
+        <v>229</v>
+      </c>
+      <c r="B54" s="52" t="s">
+        <v>236</v>
+      </c>
+      <c r="D54" s="24" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="28" t="s">
+        <v>230</v>
+      </c>
+      <c r="B55" s="50">
+        <v>13.47</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="B56" s="51">
+        <v>14.74</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="B57" s="51">
+        <v>-19.5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="B58" s="51">
+        <v>11.67</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="15" t="s">
+        <v>233</v>
+      </c>
+      <c r="B59" s="51">
+        <v>25.17</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="B60" s="51">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="B61" s="52">
+        <v>-19.5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="28" t="s">
+        <v>237</v>
+      </c>
+      <c r="B62" s="50">
+        <v>66.650000000000006</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="B63" s="51">
+        <v>96.16</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="B64" s="51">
+        <v>-71.05</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="15" t="s">
+        <v>238</v>
+      </c>
+      <c r="B65" s="51">
+        <v>63.95</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="B66" s="51">
+        <v>111.9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="B67" s="51">
+        <v>-41.81</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="15" t="s">
+        <v>239</v>
+      </c>
+      <c r="B68" s="51">
+        <v>49.15</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="54" t="s">
+        <v>246</v>
+      </c>
+      <c r="B69" s="51">
+        <v>58.96</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="16" t="s">
+        <v>247</v>
+      </c>
+      <c r="B70" s="52">
+        <v>-71.06</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="54"/>
+      <c r="B71" s="76"/>
+    </row>
+    <row r="72" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="77" t="s">
+        <v>188</v>
+      </c>
+      <c r="B72" s="78"/>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>95</v>
+      </c>
+      <c r="B73" s="26">
+        <f>210000/_Ecm_dalle</f>
+        <v>6.6717909812633494</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>96</v>
+      </c>
+      <c r="B74" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>100</v>
+      </c>
+      <c r="B75" s="1">
+        <f>50/100</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>60</v>
+      </c>
+      <c r="B76" s="32">
+        <f>_h0_dalle</f>
+        <v>123.71134020618557</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>101</v>
+      </c>
+      <c r="B77" s="25">
+        <f>IF(_fck_dalle&lt;=35,1+(1-B75)/(0.1*B76^(1/3)),FALSE)</f>
+        <v>2.0034602351846282</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>102</v>
+      </c>
+      <c r="B78" s="34">
+        <f>16.8/SQRT(_fcm_dalle)</f>
+        <v>2.9245046200557239</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>103</v>
+      </c>
+      <c r="B79" s="1">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>104</v>
+      </c>
+      <c r="B80">
+        <v>18250</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>105</v>
+      </c>
+      <c r="B81" s="25">
+        <f>1/(0.1+B79^0.2)</f>
+        <v>0.48844954537902541</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>106</v>
+      </c>
+      <c r="B82" s="26">
+        <f>B77*B78*B81</f>
+        <v>2.8618887566193885</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>107</v>
+      </c>
+      <c r="B83" s="3">
+        <f>IF(_fcm_dalle&lt;=35,MIN(B76*1.5*(1+(0.012*B75)^18)+250,1500),FALSE)</f>
+        <v>435.56701030927832</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>108</v>
+      </c>
+      <c r="B84" s="26">
+        <f>((B80-B79)/(B83+B80-B79))^0.3</f>
+        <v>0.99293840715187665</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>109</v>
+      </c>
+      <c r="B85" s="25">
+        <f>B82*B84</f>
+        <v>2.8416792634435204</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>110</v>
+      </c>
+      <c r="B86" s="26">
+        <f>B73*(1+B74*B85)</f>
+        <v>27.526790070897466</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="54"/>
+      <c r="B87" s="76"/>
+    </row>
+    <row r="88" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="70" t="s">
+        <v>79</v>
+      </c>
+      <c r="B88" s="71"/>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>183</v>
+      </c>
+      <c r="B89" s="32">
+        <v>25.2</v>
+      </c>
+      <c r="C89" s="24"/>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>269</v>
+      </c>
+      <c r="B90" s="32">
+        <f>_beff_mi_travee</f>
+        <v>2</v>
+      </c>
+      <c r="C90" s="24"/>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B91" s="14"/>
+      <c r="C91" s="24"/>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>191</v>
+      </c>
+      <c r="B92" s="43" t="s">
+        <v>189</v>
+      </c>
+      <c r="C92" s="44" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>271</v>
+      </c>
+      <c r="B93" s="35">
+        <f>_td+_h/2</f>
+        <v>270</v>
+      </c>
+      <c r="C93" s="42">
+        <f>B93</f>
+        <v>270</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>270</v>
+      </c>
+      <c r="B94" s="80">
+        <f>_A*100+_beff*1000*(_td-_tj)/B89</f>
+        <v>13066.58873015873</v>
+      </c>
+      <c r="C94" s="40">
+        <f>B94</f>
+        <v>13066.58873015873</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>90</v>
+      </c>
+      <c r="B95" s="45">
+        <f>(B89*_A*100/(_beff*1000))*(-1+SQRT(1+2*_zp/(B89*_A*100/(_beff*1000))))</f>
+        <v>125.61217341909804</v>
+      </c>
+      <c r="C95" s="46">
+        <f>_zp*_A*100/_Ah+_beff*1000*(_td-_tj)^2/(2*B89*_Ah)</f>
+        <v>126.35239879771393</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>91</v>
+      </c>
+      <c r="B96" s="35">
+        <f>_tj</f>
+        <v>10</v>
+      </c>
+      <c r="C96" s="42">
+        <f>-_h</f>
+        <v>-300</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>92</v>
+      </c>
+      <c r="B97" s="35">
+        <f>_td</f>
+        <v>120</v>
+      </c>
+      <c r="C97" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>93</v>
+      </c>
+      <c r="B98" s="35" t="b">
+        <f>IF(B96&lt;=_zel,IF(_zel&lt;=B97,TRUE,FALSE),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="C98" s="35" t="b">
+        <f>IF(C96&lt;=C95,IF(C95&lt;=C97,TRUE,FALSE),FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>94</v>
+      </c>
+      <c r="B99" s="47">
+        <f>(_Iy*10^4+_A*100*(_zp-C95)^2+_beff*1000*B95^3/(3*B89))*10^(-4)</f>
+        <v>20112.625407572665</v>
+      </c>
+      <c r="C99" s="48">
+        <f>(_Iy*10^4+_A*100*(_zp-C95)^2+_beff*1000*(_td-_tj)/(3*B89)*((_td-_tj)^2+3*C95*(C95-(_td-_tj))))*10^(-4)</f>
+        <v>20194.300001846041</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B100" s="81"/>
+      <c r="C100" s="82"/>
+    </row>
+    <row r="101" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="102" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="70" t="s">
+        <v>134</v>
+      </c>
+      <c r="B102" s="71"/>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>123</v>
+      </c>
+      <c r="B103" s="23">
+        <f>_Wpl_y*1000*_fy*10^(-6)</f>
+        <v>161.51150999999999</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>248</v>
+      </c>
+      <c r="B104" s="23">
+        <f>_Av*100*_fy/(1000*SQRT(3))</f>
+        <v>412.26137644441161</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B105" s="23"/>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106" s="21"/>
+      <c r="B106" s="62" t="s">
+        <v>249</v>
+      </c>
+      <c r="C106" s="63" t="s">
+        <v>250</v>
+      </c>
+      <c r="D106" s="22" t="s">
+        <v>251</v>
+      </c>
+      <c r="F106" s="21"/>
+      <c r="G106" s="65" t="s">
+        <v>249</v>
+      </c>
+      <c r="H106" s="66" t="s">
+        <v>250</v>
+      </c>
+      <c r="I106" s="29" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A107" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="B107" s="59">
+        <f>MAX(B63,ABS(B64))/_Mpl_Rd</f>
+        <v>0.59537552462979271</v>
+      </c>
+      <c r="C107" s="55">
+        <f>MAX(B66,ABS(B67))/_Mpl_Rd</f>
+        <v>0.69282987943088403</v>
+      </c>
+      <c r="D107" s="17">
+        <f>MAX(B69,ABS(B70))/_Mpl_Rd</f>
+        <v>0.43996864372080979</v>
+      </c>
+      <c r="F107" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="G107" s="67">
+        <f>B107</f>
+        <v>0.59537552462979271</v>
+      </c>
+      <c r="H107" s="68">
+        <f t="shared" ref="H107:I108" si="0">C107</f>
+        <v>0.69282987943088403</v>
+      </c>
+      <c r="I107" s="69">
+        <f t="shared" si="0"/>
+        <v>0.43996864372080979</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A108" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="B108" s="59">
+        <f>B62/B104</f>
+        <v>0.16166928023873936</v>
+      </c>
+      <c r="C108" s="55">
+        <f>B65/B104</f>
+        <v>0.15512003707828032</v>
+      </c>
+      <c r="D108" s="17">
+        <f>B68/B104</f>
+        <v>0.11922048197650471</v>
+      </c>
+      <c r="F108" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="G108" s="59">
+        <f>B108</f>
+        <v>0.16166928023873936</v>
+      </c>
+      <c r="H108" s="55">
+        <f t="shared" si="0"/>
+        <v>0.15512003707828032</v>
+      </c>
+      <c r="I108" s="17">
+        <f t="shared" si="0"/>
+        <v>0.11922048197650471</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A109" s="15" t="s">
+        <v>255</v>
+      </c>
+      <c r="B109" s="60">
+        <f>1/B107</f>
+        <v>1.6796122088186354</v>
+      </c>
+      <c r="C109" s="56">
+        <f t="shared" ref="C109:D109" si="1">1/C107</f>
+        <v>1.4433557640750667</v>
+      </c>
+      <c r="D109" s="57">
+        <f t="shared" si="1"/>
+        <v>2.2728892485223753</v>
+      </c>
+      <c r="F109" s="15" t="s">
+        <v>257</v>
+      </c>
+      <c r="G109" s="60">
+        <v>521.97</v>
+      </c>
+      <c r="H109" s="56">
+        <v>546.22</v>
+      </c>
+      <c r="I109" s="57">
+        <v>496.55</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A110" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="B110" s="60">
+        <v>5.4870000000000001</v>
+      </c>
+      <c r="C110" s="56">
+        <v>4.9240000000000004</v>
+      </c>
+      <c r="D110" s="57">
+        <v>6.9660000000000002</v>
+      </c>
+      <c r="F110" s="15" t="s">
+        <v>252</v>
+      </c>
+      <c r="G110" s="59">
+        <f>SQRT(_Mpl_Rd/G109)</f>
+        <v>0.55626145483781619</v>
+      </c>
+      <c r="H110" s="55">
+        <f>SQRT(_Mpl_Rd/H109)</f>
+        <v>0.54377337567286188</v>
+      </c>
+      <c r="I110" s="17">
+        <f>SQRT(_Mpl_Rd/I109)</f>
+        <v>0.57032215879907633</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111" s="15" t="s">
+        <v>252</v>
+      </c>
+      <c r="B111" s="59">
+        <f>SQRT(B109/B110)</f>
+        <v>0.55326988435906932</v>
+      </c>
+      <c r="C111" s="55">
+        <f t="shared" ref="C111:D111" si="2">SQRT(C109/C110)</f>
+        <v>0.54141174564795125</v>
+      </c>
+      <c r="D111" s="17">
+        <f t="shared" si="2"/>
+        <v>0.57121210467017469</v>
+      </c>
+      <c r="F111" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="G111" s="60">
+        <f>IF(_h/_bfs&lt;=2,0.21,0.34)</f>
+        <v>0.34</v>
+      </c>
+      <c r="H111" s="56">
+        <f>IF(_h/_bfs&lt;=2,0.21,0.34)</f>
+        <v>0.34</v>
+      </c>
+      <c r="I111" s="57">
+        <f>IF(_h/_bfs&lt;=2,0.21,0.34)</f>
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A112" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="B112" s="60">
+        <f>IF(_h/_bfs&lt;=2,0.21,0.34)</f>
+        <v>0.34</v>
+      </c>
+      <c r="C112" s="56">
+        <f>IF(_h/_bfs&lt;=2,0.21,0.34)</f>
+        <v>0.34</v>
+      </c>
+      <c r="D112" s="57">
+        <f>IF(_h/_bfs&lt;=2,0.21,0.34)</f>
+        <v>0.34</v>
+      </c>
+      <c r="F112" s="15" t="s">
+        <v>253</v>
+      </c>
+      <c r="G112" s="59">
+        <f>0.5*(1+G111*(G110-0.2)+G110^2)</f>
+        <v>0.71527785039157066</v>
+      </c>
+      <c r="H112" s="55">
+        <f t="shared" ref="H112:I112" si="3">0.5*(1+H111*(H110-0.2)+H110^2)</f>
+        <v>0.70628621590971619</v>
+      </c>
+      <c r="I112" s="17">
+        <f t="shared" si="3"/>
+        <v>0.72558844940446243</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A113" s="15" t="s">
+        <v>253</v>
+      </c>
+      <c r="B113" s="59">
+        <f>0.5*(1+B112*(B111-0.2)+B111^2)</f>
+        <v>0.71310966281039079</v>
+      </c>
+      <c r="C113" s="55">
+        <f t="shared" ref="C113:D113" si="4">0.5*(1+C112*(C111-0.2)+C111^2)</f>
+        <v>0.70460333592293267</v>
+      </c>
+      <c r="D113" s="17">
+        <f t="shared" si="4"/>
+        <v>0.72624769205479511</v>
+      </c>
+      <c r="F113" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="G113" s="59">
+        <f>1/(G112+SQRT(G112^2-G110^2))</f>
+        <v>0.85841367892050768</v>
+      </c>
+      <c r="H113" s="55">
+        <f t="shared" ref="H113:I113" si="5">1/(H112+SQRT(H112^2-H110^2))</f>
+        <v>0.86429775508559659</v>
+      </c>
+      <c r="I113" s="17">
+        <f t="shared" si="5"/>
+        <v>0.85167689179151895</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A114" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="B114" s="59">
+        <f>1/(B113+SQRT(B113^2-B111^2))</f>
+        <v>0.85983166175255588</v>
+      </c>
+      <c r="C114" s="55">
+        <f t="shared" ref="C114:D114" si="6">1/(C113+SQRT(C113^2-C111^2))</f>
+        <v>0.8654001614839576</v>
+      </c>
+      <c r="D114" s="17">
+        <f t="shared" si="6"/>
+        <v>0.85124646326009779</v>
+      </c>
+      <c r="F114" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="G114" s="60">
+        <f>G113*_Mpl_Rd</f>
+        <v>138.64368948710634</v>
+      </c>
+      <c r="H114" s="56">
+        <f>H113*_Mpl_Rd</f>
+        <v>139.59403551348487</v>
+      </c>
+      <c r="I114" s="57">
+        <f>I113*_Mpl_Rd</f>
+        <v>137.55562082535482</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A115" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="B115" s="60">
+        <f>B114*_Mpl_Rd</f>
+        <v>138.87271003546454</v>
+      </c>
+      <c r="C115" s="56">
+        <f>C114*_Mpl_Rd</f>
+        <v>139.77208683551783</v>
+      </c>
+      <c r="D115" s="57">
+        <f>D114*_Mpl_Rd</f>
+        <v>137.48610166329792</v>
+      </c>
+      <c r="F115" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="G115" s="61">
+        <f>G107/G113</f>
+        <v>0.69357646464639655</v>
+      </c>
+      <c r="H115" s="58">
+        <f>H107/H113</f>
+        <v>0.80161018046641686</v>
+      </c>
+      <c r="I115" s="18">
+        <f>I107/I113</f>
+        <v>0.51659103113074623</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A116" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="B116" s="61">
+        <f>B107/B114</f>
+        <v>0.6924326599188797</v>
+      </c>
+      <c r="C116" s="58">
+        <f t="shared" ref="C116:D116" si="7">C107/C114</f>
+        <v>0.80058903414444005</v>
+      </c>
+      <c r="D116" s="18">
+        <f t="shared" si="7"/>
+        <v>0.51685224281087871</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A102:B102"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="A72:B72"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="A88:B88"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
implémentation cls_ConnecteurArmatures + Test Unitaires
</commit_message>
<xml_diff>
--- a/Manuel Validation/Cas tests références.xlsx
+++ b/Manuel Validation/Cas tests références.xlsx
@@ -262,7 +262,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="371">
   <si>
     <t>h (mm)</t>
   </si>
@@ -1372,6 +1372,9 @@
   </si>
   <si>
     <t>Propriétés plastiques à mi travée (eta)</t>
+  </si>
+  <si>
+    <t>Critere connex</t>
   </si>
 </sst>
 </file>
@@ -1387,7 +1390,7 @@
     <numFmt numFmtId="168" formatCode="0.0000"/>
     <numFmt numFmtId="169" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="170" formatCode="0.000000"/>
-    <numFmt numFmtId="174" formatCode="_-* #,##0.0\ _€_-;\-* #,##0.0\ _€_-;_-* &quot;-&quot;?\ _€_-;_-@_-"/>
+    <numFmt numFmtId="171" formatCode="_-* #,##0.0\ _€_-;\-* #,##0.0\ _€_-;_-* &quot;-&quot;?\ _€_-;_-@_-"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -1925,30 +1928,6 @@
     <xf numFmtId="170" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2041,7 +2020,31 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2337,20 +2340,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="150" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="114"/>
+      <c r="B1" s="151"/>
       <c r="C1"/>
-      <c r="D1" s="113" t="s">
+      <c r="D1" s="150" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="114"/>
+      <c r="E1" s="151"/>
       <c r="F1" s="24"/>
-      <c r="G1" s="113" t="s">
+      <c r="G1" s="150" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="114"/>
+      <c r="H1" s="151"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -2612,10 +2615,10 @@
         <v>0.81361651346682706</v>
       </c>
       <c r="C15"/>
-      <c r="D15" s="113" t="s">
+      <c r="D15" s="150" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="114"/>
+      <c r="E15" s="151"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B16" s="6"/>
@@ -2754,10 +2757,10 @@
       <c r="C29"/>
     </row>
     <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="113" t="s">
+      <c r="A30" s="150" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="114"/>
+      <c r="B30" s="151"/>
       <c r="C30" s="24" t="s">
         <v>53</v>
       </c>
@@ -3025,10 +3028,10 @@
       </c>
     </row>
     <row r="50" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="113" t="s">
+      <c r="A50" s="150" t="s">
         <v>16</v>
       </c>
-      <c r="B50" s="114"/>
+      <c r="B50" s="151"/>
       <c r="D50" s="26" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3065,10 +3068,10 @@
         <f t="shared" si="0"/>
         <v>0.41222226735473377</v>
       </c>
-      <c r="E52" s="115" t="s">
+      <c r="E52" s="152" t="s">
         <v>34</v>
       </c>
-      <c r="F52" s="116"/>
+      <c r="F52" s="153"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -3316,10 +3319,10 @@
       </c>
     </row>
     <row r="68" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="113" t="s">
+      <c r="A68" s="150" t="s">
         <v>79</v>
       </c>
-      <c r="B68" s="114"/>
+      <c r="B68" s="151"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
@@ -3603,10 +3606,10 @@
     </row>
     <row r="95" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="96" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="113" t="s">
+      <c r="A96" s="150" t="s">
         <v>111</v>
       </c>
-      <c r="B96" s="114"/>
+      <c r="B96" s="151"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
@@ -3710,10 +3713,10 @@
     </row>
     <row r="108" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="109" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="113" t="s">
+      <c r="A109" s="150" t="s">
         <v>133</v>
       </c>
-      <c r="B109" s="114"/>
+      <c r="B109" s="151"/>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
@@ -3796,10 +3799,10 @@
     </row>
     <row r="119" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="120" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="113" t="s">
+      <c r="A120" s="150" t="s">
         <v>134</v>
       </c>
-      <c r="B120" s="114"/>
+      <c r="B120" s="151"/>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
@@ -3924,20 +3927,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="150" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="114"/>
+      <c r="B1" s="151"/>
       <c r="C1"/>
-      <c r="D1" s="113" t="s">
+      <c r="D1" s="150" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="114"/>
+      <c r="E1" s="151"/>
       <c r="F1" s="24"/>
-      <c r="G1" s="113" t="s">
+      <c r="G1" s="150" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="114"/>
+      <c r="H1" s="151"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -4172,16 +4175,16 @@
         <f>500/1.15</f>
         <v>434.78260869565219</v>
       </c>
-      <c r="G12" s="113" t="s">
+      <c r="G12" s="150" t="s">
         <v>162</v>
       </c>
-      <c r="H12" s="114"/>
+      <c r="H12" s="151"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="113" t="s">
+      <c r="A13" s="150" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="114"/>
+      <c r="B13" s="151"/>
       <c r="C13"/>
       <c r="D13" t="s">
         <v>125</v>
@@ -4220,10 +4223,10 @@
         <v>200</v>
       </c>
       <c r="C15"/>
-      <c r="D15" s="113" t="s">
+      <c r="D15" s="150" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="114"/>
+      <c r="E15" s="151"/>
       <c r="G15" t="s">
         <v>166</v>
       </c>
@@ -4527,10 +4530,10 @@
       <c r="C30"/>
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="113" t="s">
+      <c r="A31" s="150" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="114"/>
+      <c r="B31" s="151"/>
       <c r="C31" s="24" t="s">
         <v>53</v>
       </c>
@@ -4798,10 +4801,10 @@
       </c>
     </row>
     <row r="51" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="113" t="s">
+      <c r="A51" s="150" t="s">
         <v>16</v>
       </c>
-      <c r="B51" s="114"/>
+      <c r="B51" s="151"/>
       <c r="D51" s="26" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4838,10 +4841,10 @@
         <f t="shared" si="0"/>
         <v>0.41222226735473377</v>
       </c>
-      <c r="E53" s="115" t="s">
+      <c r="E53" s="152" t="s">
         <v>34</v>
       </c>
-      <c r="F53" s="116"/>
+      <c r="F53" s="153"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
@@ -5089,10 +5092,10 @@
       </c>
     </row>
     <row r="69" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="113" t="s">
+      <c r="A69" s="150" t="s">
         <v>79</v>
       </c>
-      <c r="B69" s="114"/>
+      <c r="B69" s="151"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
@@ -5273,10 +5276,10 @@
       <c r="C84" s="36"/>
     </row>
     <row r="85" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="117" t="s">
+      <c r="A85" s="154" t="s">
         <v>188</v>
       </c>
-      <c r="B85" s="118"/>
+      <c r="B85" s="155"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
@@ -5419,10 +5422,10 @@
     </row>
     <row r="100" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="101" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="113" t="s">
+      <c r="A101" s="150" t="s">
         <v>111</v>
       </c>
-      <c r="B101" s="114"/>
+      <c r="B101" s="151"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="7" t="s">
@@ -5562,10 +5565,10 @@
     </row>
     <row r="117" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="118" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="113" t="s">
+      <c r="A118" s="150" t="s">
         <v>133</v>
       </c>
-      <c r="B118" s="114"/>
+      <c r="B118" s="151"/>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
@@ -5684,10 +5687,10 @@
     </row>
     <row r="132" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="133" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A133" s="113" t="s">
+      <c r="A133" s="150" t="s">
         <v>134</v>
       </c>
-      <c r="B133" s="114"/>
+      <c r="B133" s="151"/>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
@@ -5803,10 +5806,10 @@
     </row>
     <row r="146" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="147" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="113" t="s">
+      <c r="A147" s="150" t="s">
         <v>207</v>
       </c>
-      <c r="B147" s="114"/>
+      <c r="B147" s="151"/>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
@@ -5872,6 +5875,11 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="D15:E15"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A51:B51"/>
     <mergeCell ref="G12:H12"/>
@@ -5882,11 +5890,6 @@
     <mergeCell ref="A101:B101"/>
     <mergeCell ref="A118:B118"/>
     <mergeCell ref="A133:B133"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="D15:E15"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E16">
@@ -5925,18 +5928,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="150" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="D1" s="113" t="s">
+      <c r="B1" s="151"/>
+      <c r="D1" s="150" t="s">
         <v>221</v>
       </c>
-      <c r="E1" s="114"/>
-      <c r="G1" s="113" t="s">
+      <c r="E1" s="151"/>
+      <c r="G1" s="150" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="114"/>
+      <c r="H1" s="151"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -6060,10 +6063,10 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="150" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="114"/>
+      <c r="B9" s="151"/>
       <c r="D9" t="s">
         <v>32</v>
       </c>
@@ -6262,10 +6265,10 @@
     </row>
     <row r="28" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="113" t="s">
+      <c r="A29" s="150" t="s">
         <v>16</v>
       </c>
-      <c r="B29" s="114"/>
+      <c r="B29" s="151"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -6284,10 +6287,10 @@
         <f>_Av*100*_fy/(1000*SQRT(3))</f>
         <v>1042.1194079466816</v>
       </c>
-      <c r="D31" s="115" t="s">
+      <c r="D31" s="152" t="s">
         <v>34</v>
       </c>
-      <c r="E31" s="116"/>
+      <c r="E31" s="153"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -6467,10 +6470,10 @@
     </row>
     <row r="46" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="113" t="s">
+      <c r="A47" s="150" t="s">
         <v>133</v>
       </c>
-      <c r="B47" s="114"/>
+      <c r="B47" s="151"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="107" t="s">
@@ -6638,10 +6641,10 @@
     </row>
     <row r="68" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="69" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="113" t="s">
+      <c r="A69" s="150" t="s">
         <v>134</v>
       </c>
-      <c r="B69" s="114"/>
+      <c r="B69" s="151"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
@@ -7020,18 +7023,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="150" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="D1" s="113" t="s">
+      <c r="B1" s="151"/>
+      <c r="D1" s="150" t="s">
         <v>221</v>
       </c>
-      <c r="E1" s="114"/>
-      <c r="G1" s="113" t="s">
+      <c r="E1" s="151"/>
+      <c r="G1" s="150" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="114"/>
+      <c r="H1" s="151"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -7253,10 +7256,10 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="113" t="s">
+      <c r="A13" s="150" t="s">
         <v>256</v>
       </c>
-      <c r="B13" s="114"/>
+      <c r="B13" s="151"/>
       <c r="D13" t="s">
         <v>38</v>
       </c>
@@ -7280,10 +7283,10 @@
         <f>(_bfi-2*_r-_tw)/2</f>
         <v>71.45</v>
       </c>
-      <c r="G14" s="113" t="s">
+      <c r="G14" s="150" t="s">
         <v>162</v>
       </c>
-      <c r="H14" s="114"/>
+      <c r="H14" s="151"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -7542,10 +7545,10 @@
     </row>
     <row r="32" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="113" t="s">
+      <c r="A33" s="150" t="s">
         <v>16</v>
       </c>
-      <c r="B33" s="114"/>
+      <c r="B33" s="151"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
@@ -7564,10 +7567,10 @@
         <f>_Av*100*_fy/(1000*SQRT(3))</f>
         <v>487.74585382155738</v>
       </c>
-      <c r="D35" s="115" t="s">
+      <c r="D35" s="152" t="s">
         <v>34</v>
       </c>
-      <c r="E35" s="116"/>
+      <c r="E35" s="153"/>
       <c r="G35" s="21" t="s">
         <v>44</v>
       </c>
@@ -7677,10 +7680,10 @@
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="J40" s="115" t="s">
+      <c r="J40" s="152" t="s">
         <v>276</v>
       </c>
-      <c r="K40" s="116"/>
+      <c r="K40" s="153"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
@@ -7739,10 +7742,10 @@
         <f>B45-300</f>
         <v>-178.04000000000002</v>
       </c>
-      <c r="J45" s="115" t="s">
+      <c r="J45" s="152" t="s">
         <v>277</v>
       </c>
-      <c r="K45" s="116"/>
+      <c r="K45" s="153"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
@@ -7790,10 +7793,10 @@
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="J49" s="115" t="s">
+      <c r="J49" s="152" t="s">
         <v>278</v>
       </c>
-      <c r="K49" s="116"/>
+      <c r="K49" s="153"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
@@ -7828,10 +7831,10 @@
         <f>IF(B47&gt;0.5,IF(B42&lt;=K41,1,IF(B42&lt;=K42,2,IF(B48&gt;-1,IF(B42&lt;=K50,3,4),IF(B42&lt;=K54,3,4)))),IF(B42&lt;=K46,1,IF(B42&lt;=K47,2,IF(B48&gt;-1,IF(B42&lt;=K50,3,4),IF(B42&lt;=K54,3,4)))))</f>
         <v>2</v>
       </c>
-      <c r="J52" s="115" t="s">
+      <c r="J52" s="152" t="s">
         <v>280</v>
       </c>
-      <c r="K52" s="116"/>
+      <c r="K52" s="153"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -7895,10 +7898,10 @@
       <c r="B62" s="70"/>
     </row>
     <row r="63" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="119" t="s">
+      <c r="A63" s="156" t="s">
         <v>188</v>
       </c>
-      <c r="B63" s="120"/>
+      <c r="B63" s="157"/>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
@@ -8044,10 +8047,10 @@
       <c r="B78" s="70"/>
     </row>
     <row r="79" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="113" t="s">
+      <c r="A79" s="150" t="s">
         <v>79</v>
       </c>
-      <c r="B79" s="114"/>
+      <c r="B79" s="151"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
@@ -8284,16 +8287,16 @@
     </row>
     <row r="95" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="96" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="113" t="s">
+      <c r="A96" s="150" t="s">
         <v>369</v>
       </c>
-      <c r="B96" s="114"/>
+      <c r="B96" s="151"/>
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
         <v>339</v>
       </c>
-      <c r="B97" s="121">
+      <c r="B97" s="113">
         <f>_L/4</f>
         <v>2.5</v>
       </c>
@@ -8302,7 +8305,7 @@
       <c r="A98" s="7" t="s">
         <v>340</v>
       </c>
-      <c r="B98" s="122">
+      <c r="B98" s="114">
         <v>5</v>
       </c>
     </row>
@@ -8310,13 +8313,13 @@
       <c r="A99" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="B99" s="121">
+      <c r="B99" s="113">
         <f>IF(B98&lt;=B97,_beff_appuis+(_beff_mi_travee-_beff_appuis)/B97*B98,_beff_mi_travee)</f>
         <v>2</v>
       </c>
     </row>
     <row r="100" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A100" s="123" t="s">
+      <c r="A100" s="115" t="s">
         <v>341</v>
       </c>
       <c r="B100" s="14">
@@ -8325,7 +8328,7 @@
       </c>
     </row>
     <row r="101" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A101" s="123" t="s">
+      <c r="A101" s="115" t="s">
         <v>342</v>
       </c>
       <c r="B101" s="14">
@@ -8334,7 +8337,7 @@
       </c>
     </row>
     <row r="102" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A102" s="123" t="s">
+      <c r="A102" s="115" t="s">
         <v>343</v>
       </c>
       <c r="B102" s="14">
@@ -8343,8 +8346,8 @@
       </c>
     </row>
     <row r="103" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A103" s="121"/>
-      <c r="B103" s="121"/>
+      <c r="A103" s="113"/>
+      <c r="B103" s="113"/>
     </row>
     <row r="104" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
@@ -8748,16 +8751,16 @@
     </row>
     <row r="115" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="116" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="113" t="s">
+      <c r="A116" s="150" t="s">
         <v>338</v>
       </c>
-      <c r="B116" s="114"/>
+      <c r="B116" s="151"/>
     </row>
     <row r="117" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
         <v>339</v>
       </c>
-      <c r="B117" s="121">
+      <c r="B117" s="113">
         <f>_L/4</f>
         <v>2.5</v>
       </c>
@@ -8766,7 +8769,7 @@
       <c r="A118" s="7" t="s">
         <v>340</v>
       </c>
-      <c r="B118" s="122">
+      <c r="B118" s="114">
         <v>0.5</v>
       </c>
     </row>
@@ -8774,13 +8777,13 @@
       <c r="A119" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="B119" s="121">
+      <c r="B119" s="113">
         <f>IF(B118&lt;=B117,_beff_appuis+(_beff_mi_travee-_beff_appuis)/B117*B118,_beff_mi_travee)</f>
         <v>1.6800000000000002</v>
       </c>
     </row>
     <row r="120" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A120" s="123" t="s">
+      <c r="A120" s="115" t="s">
         <v>341</v>
       </c>
       <c r="B120" s="14">
@@ -8790,7 +8793,7 @@
       <c r="C120" s="24"/>
     </row>
     <row r="121" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A121" s="123" t="s">
+      <c r="A121" s="115" t="s">
         <v>342</v>
       </c>
       <c r="B121" s="14">
@@ -8800,7 +8803,7 @@
       <c r="C121" s="24"/>
     </row>
     <row r="122" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A122" s="123" t="s">
+      <c r="A122" s="115" t="s">
         <v>343</v>
       </c>
       <c r="B122" s="14">
@@ -8810,7 +8813,7 @@
       <c r="C122" s="24"/>
     </row>
     <row r="123" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A123" s="123"/>
+      <c r="A123" s="115"/>
       <c r="B123" s="14"/>
       <c r="C123" s="24"/>
     </row>
@@ -9216,10 +9219,10 @@
     </row>
     <row r="135" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="136" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="113" t="s">
+      <c r="A136" s="150" t="s">
         <v>133</v>
       </c>
-      <c r="B136" s="114"/>
+      <c r="B136" s="151"/>
     </row>
     <row r="137" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
@@ -9430,17 +9433,17 @@
     </row>
     <row r="158" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="159" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A159" s="113" t="s">
+      <c r="A159" s="150" t="s">
         <v>134</v>
       </c>
-      <c r="B159" s="114"/>
+      <c r="B159" s="151"/>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A160" s="121"/>
-      <c r="B160" s="121"/>
+      <c r="A160" s="113"/>
+      <c r="B160" s="113"/>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A161" s="121"/>
+      <c r="A161" s="113"/>
       <c r="B161" s="77" t="s">
         <v>344</v>
       </c>
@@ -9458,10 +9461,10 @@
       </c>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A162" s="132" t="s">
+      <c r="A162" s="124" t="s">
         <v>328</v>
       </c>
-      <c r="B162" s="139"/>
+      <c r="B162" s="131"/>
       <c r="C162" s="66">
         <v>30.8</v>
       </c>
@@ -9471,31 +9474,31 @@
       <c r="E162" s="29">
         <v>29.1</v>
       </c>
-      <c r="F162" s="127"/>
+      <c r="F162" s="119"/>
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="28" t="s">
         <v>365</v>
       </c>
-      <c r="B163" s="155">
+      <c r="B163" s="147">
         <v>5921</v>
       </c>
-      <c r="C163" s="154">
+      <c r="C163" s="146">
         <v>22581</v>
       </c>
-      <c r="D163" s="154">
+      <c r="D163" s="146">
         <v>31404</v>
       </c>
-      <c r="E163" s="156">
+      <c r="E163" s="148">
         <v>22952</v>
       </c>
-      <c r="F163" s="127"/>
+      <c r="F163" s="119"/>
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A164" s="134" t="s">
+      <c r="A164" s="126" t="s">
         <v>366</v>
       </c>
-      <c r="B164" s="152">
+      <c r="B164" s="144">
         <v>-178</v>
       </c>
       <c r="C164" s="82">
@@ -9507,46 +9510,46 @@
       <c r="E164" s="30">
         <v>-23.7</v>
       </c>
-      <c r="F164" s="135"/>
+      <c r="F164" s="127"/>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" s="28" t="s">
         <v>367</v>
       </c>
-      <c r="B165" s="155">
+      <c r="B165" s="147">
         <v>5921</v>
       </c>
-      <c r="C165" s="154">
+      <c r="C165" s="146">
         <v>21530.096266744444</v>
       </c>
-      <c r="D165" s="154">
+      <c r="D165" s="146">
         <v>30234.112325995633</v>
       </c>
-      <c r="E165" s="156">
+      <c r="E165" s="148">
         <v>21539.889165989531</v>
       </c>
-      <c r="F165" s="127"/>
+      <c r="F165" s="119"/>
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A166" s="134" t="s">
+      <c r="A166" s="126" t="s">
         <v>368</v>
       </c>
-      <c r="B166" s="152">
+      <c r="B166" s="144">
         <v>-178</v>
       </c>
       <c r="C166" s="96">
         <v>-34.487492252446586</v>
       </c>
-      <c r="D166" s="153">
+      <c r="D166" s="145">
         <v>30.897637600365364</v>
       </c>
       <c r="E166" s="20">
         <v>-34.40387189041919</v>
       </c>
-      <c r="F166" s="135"/>
+      <c r="F166" s="127"/>
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A167" s="134" t="s">
+      <c r="A167" s="126" t="s">
         <v>351</v>
       </c>
       <c r="B167" s="16" t="s">
@@ -9561,13 +9564,13 @@
       <c r="E167" s="30" t="s">
         <v>353</v>
       </c>
-      <c r="F167" s="135"/>
+      <c r="F167" s="127"/>
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A168" s="150" t="s">
+      <c r="A168" s="142" t="s">
         <v>363</v>
       </c>
-      <c r="B168" s="151">
+      <c r="B168" s="143">
         <f>B139</f>
         <v>31.099709848275001</v>
       </c>
@@ -9585,26 +9588,26 @@
       <c r="F168" s="83"/>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A169" s="133" t="s">
+      <c r="A169" s="125" t="s">
         <v>354</v>
       </c>
-      <c r="B169" s="140">
+      <c r="B169" s="132">
         <f>IF(B167="N",0,$B$140*10^6/(B$163*10^4)*(_td-B$164)/B162)</f>
         <v>0</v>
       </c>
-      <c r="C169" s="125">
+      <c r="C169" s="117">
         <f>IF(C167="N",0,$B$142*10^6/(C$163*10^4)*(_td-C$164)/C162)</f>
         <v>1.0553637496642678</v>
       </c>
-      <c r="D169" s="125">
+      <c r="D169" s="117">
         <f>IF(D167="N",0,$B$144*10^6/(D$163*10^4)*(_td-D$164)/D162)</f>
         <v>9.2213191083356905E-2</v>
       </c>
-      <c r="E169" s="141">
+      <c r="E169" s="133">
         <f>IF(E167="N",0,$B$153*10^6/(E$163*10^4)*(_td-E$164)/E162)</f>
         <v>1.0533792862815441</v>
       </c>
-      <c r="F169" s="128">
+      <c r="F169" s="120">
         <f>1.35*(B169+C169)+1.5*D169+1.35*E169</f>
         <v>2.9851228851518821</v>
       </c>
@@ -9613,26 +9616,26 @@
       </c>
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A170" s="133" t="s">
+      <c r="A170" s="125" t="s">
         <v>355</v>
       </c>
-      <c r="B170" s="140">
+      <c r="B170" s="132">
         <f>$B$140*10^6/(B$163*10^4)*(0-B$164)</f>
         <v>233.73367475903353</v>
       </c>
-      <c r="C170" s="125">
+      <c r="C170" s="117">
         <f>$B$142*10^6/(C$163*10^4)*(0-C$164)</f>
         <v>5.9341924626898717</v>
       </c>
-      <c r="D170" s="124">
+      <c r="D170" s="116">
         <f>$B$144*10^6/(D$163*10^4)*(0-D$164)</f>
         <v>-0.30887784995541961</v>
       </c>
-      <c r="E170" s="142">
+      <c r="E170" s="134">
         <f>$B$153*10^6/(E$163*10^4)*(0-E$164)</f>
         <v>5.0555608376464338</v>
       </c>
-      <c r="F170" s="128">
+      <c r="F170" s="120">
         <f t="shared" ref="F170:F171" si="22">1.35*(B170+C170)+1.5*D170+1.35*E170</f>
         <v>329.91331110521622</v>
       </c>
@@ -9641,26 +9644,26 @@
       </c>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A171" s="134" t="s">
+      <c r="A171" s="126" t="s">
         <v>356</v>
       </c>
-      <c r="B171" s="143">
+      <c r="B171" s="135">
         <f>$B$140*10^6/(B$163*10^4)*(-_h-B$164)</f>
         <v>-160.19948494720276</v>
       </c>
-      <c r="C171" s="137">
+      <c r="C171" s="129">
         <f>$B$142*10^6/(C$163*10^4)*(-_h-C$164)</f>
         <v>-60.493335104734065</v>
       </c>
-      <c r="D171" s="136">
+      <c r="D171" s="128">
         <f>$B$144*10^6/(D$163*10^4)*(-_h-D$164)</f>
         <v>-2.6971086485797984</v>
       </c>
-      <c r="E171" s="144">
+      <c r="E171" s="136">
         <f>$B$153*10^6/(E$163*10^4)*(-_h-E$164)</f>
         <v>-58.938880145219827</v>
       </c>
-      <c r="F171" s="138">
+      <c r="F171" s="130">
         <f t="shared" si="22"/>
         <v>-381.54845823903122</v>
       </c>
@@ -9669,10 +9672,10 @@
       </c>
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A172" s="133" t="s">
+      <c r="A172" s="125" t="s">
         <v>348</v>
       </c>
-      <c r="B172" s="145">
+      <c r="B172" s="137">
         <f>B169/(0.85*_fck_dalle/1.5)</f>
         <v>0</v>
       </c>
@@ -9684,61 +9687,61 @@
         <f>D169/(0.85*_fck_dalle/1.5)</f>
         <v>8.136458036766785E-3</v>
       </c>
-      <c r="E172" s="146">
+      <c r="E172" s="138">
         <f>E169/(0.85*_fck_dalle/1.5)</f>
         <v>9.2945231142489176E-2</v>
       </c>
-      <c r="F172" s="129">
+      <c r="F172" s="121">
         <f>F169/(0.85*_fck_dalle/1.5)</f>
         <v>0.26339319574869546</v>
       </c>
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A173" s="133" t="s">
+      <c r="A173" s="125" t="s">
         <v>349</v>
       </c>
-      <c r="B173" s="147">
+      <c r="B173" s="139">
         <f>B170/(_fy)</f>
         <v>0.55650874942627027</v>
       </c>
-      <c r="C173" s="125">
+      <c r="C173" s="117">
         <f>C170/(_fy)</f>
         <v>1.4129029673071123E-2</v>
       </c>
-      <c r="D173" s="125">
+      <c r="D173" s="117">
         <f>D170/(_fy)</f>
         <v>-7.3542345227480856E-4</v>
       </c>
-      <c r="E173" s="141">
+      <c r="E173" s="133">
         <f>E170/(_fy)</f>
         <v>1.203704961344389E-2</v>
       </c>
-      <c r="F173" s="130">
+      <c r="F173" s="122">
         <f>F170/(_fy)</f>
         <v>0.78550788358384815</v>
       </c>
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A174" s="134" t="s">
+      <c r="A174" s="126" t="s">
         <v>350</v>
       </c>
-      <c r="B174" s="148">
+      <c r="B174" s="140">
         <f>ABS(B171/(_fy))</f>
         <v>0.38142734511238752</v>
       </c>
-      <c r="C174" s="126">
+      <c r="C174" s="118">
         <f>ABS(C171/(_fy))</f>
         <v>0.14403175024936682</v>
       </c>
-      <c r="D174" s="126">
+      <c r="D174" s="118">
         <f>ABS(D171/(_fy))</f>
         <v>6.4216872585233292E-3</v>
       </c>
-      <c r="E174" s="149">
+      <c r="E174" s="141">
         <f>ABS(E171/(_fy))</f>
         <v>0.14033066701242816</v>
       </c>
-      <c r="F174" s="131">
+      <c r="F174" s="123">
         <f>ABS(F171/(_fy))</f>
         <v>0.90844871009293149</v>
       </c>
@@ -9747,19 +9750,19 @@
       <c r="A175" s="7" t="s">
         <v>362</v>
       </c>
-      <c r="B175" s="124">
+      <c r="B175" s="116">
         <f>ABS(IF(B167="N",0,_beff_appuis*1000*(_td-_tj)/B162*(B166-((_td-_tj)/2+_tj))))</f>
         <v>0</v>
       </c>
-      <c r="C175" s="124">
+      <c r="C175" s="116">
         <f>ABS(IF(C167="N",0,_beff_appuis*1000*(_td-_tj)/C162*(C166-((_td-_tj)/2+_tj))))</f>
         <v>568499.95572826616</v>
       </c>
-      <c r="D175" s="124">
+      <c r="D175" s="116">
         <f>ABS(IF(D167="N",0,_beff_appuis*1000*(_td-_tj)/D162*(D166-((_td-_tj)/2+_tj))))</f>
         <v>856207.67223048443</v>
       </c>
-      <c r="E175" s="124">
+      <c r="E175" s="116">
         <f>ABS(IF(E167="N",0,_beff_appuis*1000*(_td-_tj)/E162*(E166-((_td-_tj)/2+_tj))))</f>
         <v>601205.54820322257</v>
       </c>
@@ -9768,19 +9771,19 @@
       <c r="A176" s="7" t="s">
         <v>361</v>
       </c>
-      <c r="B176" s="157">
+      <c r="B176" s="149">
         <f>B168*1000*B175/B165/1000</f>
         <v>0</v>
       </c>
-      <c r="C176" s="157">
+      <c r="C176" s="149">
         <f t="shared" ref="C176:E176" si="23">C168*1000*C175/C165/1000</f>
         <v>528.09792272631466</v>
       </c>
-      <c r="D176" s="157">
+      <c r="D176" s="149">
         <f t="shared" si="23"/>
         <v>14.15962974203657</v>
       </c>
-      <c r="E176" s="157">
+      <c r="E176" s="149">
         <f t="shared" si="23"/>
         <v>0</v>
       </c>
@@ -9789,90 +9792,97 @@
         <v>734.17164029357969</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="7"/>
-      <c r="B177" s="121"/>
-      <c r="C177" s="124"/>
-      <c r="D177" s="124"/>
-      <c r="E177" s="121"/>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A178" s="7"/>
-      <c r="B178" s="121"/>
-    </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A179" t="s">
+      <c r="B177" s="113"/>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
         <v>245</v>
       </c>
-      <c r="B179" s="23">
+      <c r="B178" s="23">
         <f>_Av*100*_fy/(1000*SQRT(3))</f>
         <v>487.74585382155738</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A180" s="123" t="s">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A179" s="115" t="s">
         <v>123</v>
       </c>
-      <c r="B180" s="23">
+      <c r="B179" s="23">
         <v>464.72471483007769</v>
       </c>
-      <c r="C180">
-        <f>B180*B181</f>
+      <c r="C179">
+        <f>B179*B180</f>
         <v>464.72471483007769</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A181" s="123" t="s">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A180" s="115" t="s">
         <v>359</v>
       </c>
+      <c r="B180" s="25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A181" s="115" t="s">
+        <v>364</v>
+      </c>
       <c r="B181" s="25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A182" s="123" t="s">
-        <v>364</v>
-      </c>
-      <c r="B182" s="25">
         <f>_PRd/(_sx/1000)</f>
         <v>341.22561783575122</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B183" s="23"/>
-    </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A184" t="s">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B182" s="23"/>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
         <v>141</v>
       </c>
-      <c r="B184" s="26">
+      <c r="B183" s="26">
         <f>MAX(F172:F174)</f>
         <v>0.90844871009293149</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>142</v>
+      </c>
+      <c r="B184" s="26">
+        <f>B154/B178</f>
+        <v>0.14297324672017361</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>142</v>
+        <v>358</v>
       </c>
       <c r="B185" s="26">
-        <f>B154/B179</f>
-        <v>0.14297324672017361</v>
-      </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+        <f>B155/(B180*B179)</f>
+        <v>0.52140015676004936</v>
+      </c>
+      <c r="C185" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="B186" s="26">
-        <f>B155/(B181*B180)</f>
-        <v>0.52140015676004936</v>
-      </c>
-      <c r="C186" t="s">
-        <v>360</v>
+        <f>F176/B181</f>
+        <v>2.1515724550522255</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="J49:K49"/>
+    <mergeCell ref="J52:K52"/>
+    <mergeCell ref="A136:B136"/>
     <mergeCell ref="A159:B159"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="D1:E1"/>
@@ -9885,11 +9895,6 @@
     <mergeCell ref="A79:B79"/>
     <mergeCell ref="A96:B96"/>
     <mergeCell ref="A116:B116"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="J49:K49"/>
-    <mergeCell ref="J52:K52"/>
-    <mergeCell ref="A136:B136"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Dernier push: Avancement MV + corrections bugs
</commit_message>
<xml_diff>
--- a/Manuel Validation/Cas tests références.xlsx
+++ b/Manuel Validation/Cas tests références.xlsx
@@ -262,7 +262,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="378">
   <si>
     <t>h (mm)</t>
   </si>
@@ -1350,9 +1350,6 @@
     <t>flux cisaillement connecteur (kN/m)</t>
   </si>
   <si>
-    <t>Sh,i (mm3)</t>
-  </si>
-  <si>
     <t>Ved (kN)</t>
   </si>
   <si>
@@ -1375,6 +1372,30 @@
   </si>
   <si>
     <t>Critere connex</t>
+  </si>
+  <si>
+    <t>Sh,0 (mm3)</t>
+  </si>
+  <si>
+    <t>flux cisaillement soudure sup (kN/m)</t>
+  </si>
+  <si>
+    <t>Sh,1 (mm3)</t>
+  </si>
+  <si>
+    <t>Beta w</t>
+  </si>
+  <si>
+    <t>fu (Mpa)</t>
+  </si>
+  <si>
+    <t>aw,sup (mm)</t>
+  </si>
+  <si>
+    <t>aw,inf (mm)</t>
+  </si>
+  <si>
+    <t>Sh,2 (mm3)</t>
   </si>
 </sst>
 </file>
@@ -1798,7 +1819,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2020,9 +2041,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2045,6 +2063,21 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2340,20 +2373,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="150" t="s">
+      <c r="A1" s="149" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="151"/>
+      <c r="B1" s="150"/>
       <c r="C1"/>
-      <c r="D1" s="150" t="s">
+      <c r="D1" s="149" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="151"/>
+      <c r="E1" s="150"/>
       <c r="F1" s="24"/>
-      <c r="G1" s="150" t="s">
+      <c r="G1" s="149" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="151"/>
+      <c r="H1" s="150"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -2615,10 +2648,10 @@
         <v>0.81361651346682706</v>
       </c>
       <c r="C15"/>
-      <c r="D15" s="150" t="s">
+      <c r="D15" s="149" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="151"/>
+      <c r="E15" s="150"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B16" s="6"/>
@@ -2757,10 +2790,10 @@
       <c r="C29"/>
     </row>
     <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="150" t="s">
+      <c r="A30" s="149" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="151"/>
+      <c r="B30" s="150"/>
       <c r="C30" s="24" t="s">
         <v>53</v>
       </c>
@@ -3028,10 +3061,10 @@
       </c>
     </row>
     <row r="50" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="150" t="s">
+      <c r="A50" s="149" t="s">
         <v>16</v>
       </c>
-      <c r="B50" s="151"/>
+      <c r="B50" s="150"/>
       <c r="D50" s="26" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3068,10 +3101,10 @@
         <f t="shared" si="0"/>
         <v>0.41222226735473377</v>
       </c>
-      <c r="E52" s="152" t="s">
+      <c r="E52" s="151" t="s">
         <v>34</v>
       </c>
-      <c r="F52" s="153"/>
+      <c r="F52" s="152"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -3319,10 +3352,10 @@
       </c>
     </row>
     <row r="68" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="150" t="s">
+      <c r="A68" s="149" t="s">
         <v>79</v>
       </c>
-      <c r="B68" s="151"/>
+      <c r="B68" s="150"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
@@ -3606,10 +3639,10 @@
     </row>
     <row r="95" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="96" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="150" t="s">
+      <c r="A96" s="149" t="s">
         <v>111</v>
       </c>
-      <c r="B96" s="151"/>
+      <c r="B96" s="150"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
@@ -3713,10 +3746,10 @@
     </row>
     <row r="108" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="109" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="150" t="s">
+      <c r="A109" s="149" t="s">
         <v>133</v>
       </c>
-      <c r="B109" s="151"/>
+      <c r="B109" s="150"/>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
@@ -3799,10 +3832,10 @@
     </row>
     <row r="119" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="120" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="150" t="s">
+      <c r="A120" s="149" t="s">
         <v>134</v>
       </c>
-      <c r="B120" s="151"/>
+      <c r="B120" s="150"/>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
@@ -3927,20 +3960,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="150" t="s">
+      <c r="A1" s="149" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="151"/>
+      <c r="B1" s="150"/>
       <c r="C1"/>
-      <c r="D1" s="150" t="s">
+      <c r="D1" s="149" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="151"/>
+      <c r="E1" s="150"/>
       <c r="F1" s="24"/>
-      <c r="G1" s="150" t="s">
+      <c r="G1" s="149" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="151"/>
+      <c r="H1" s="150"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -4175,16 +4208,16 @@
         <f>500/1.15</f>
         <v>434.78260869565219</v>
       </c>
-      <c r="G12" s="150" t="s">
+      <c r="G12" s="149" t="s">
         <v>162</v>
       </c>
-      <c r="H12" s="151"/>
+      <c r="H12" s="150"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="150" t="s">
+      <c r="A13" s="149" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="151"/>
+      <c r="B13" s="150"/>
       <c r="C13"/>
       <c r="D13" t="s">
         <v>125</v>
@@ -4223,10 +4256,10 @@
         <v>200</v>
       </c>
       <c r="C15"/>
-      <c r="D15" s="150" t="s">
+      <c r="D15" s="149" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="151"/>
+      <c r="E15" s="150"/>
       <c r="G15" t="s">
         <v>166</v>
       </c>
@@ -4530,10 +4563,10 @@
       <c r="C30"/>
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="150" t="s">
+      <c r="A31" s="149" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="151"/>
+      <c r="B31" s="150"/>
       <c r="C31" s="24" t="s">
         <v>53</v>
       </c>
@@ -4801,10 +4834,10 @@
       </c>
     </row>
     <row r="51" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="150" t="s">
+      <c r="A51" s="149" t="s">
         <v>16</v>
       </c>
-      <c r="B51" s="151"/>
+      <c r="B51" s="150"/>
       <c r="D51" s="26" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4841,10 +4874,10 @@
         <f t="shared" si="0"/>
         <v>0.41222226735473377</v>
       </c>
-      <c r="E53" s="152" t="s">
+      <c r="E53" s="151" t="s">
         <v>34</v>
       </c>
-      <c r="F53" s="153"/>
+      <c r="F53" s="152"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
@@ -5092,10 +5125,10 @@
       </c>
     </row>
     <row r="69" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="150" t="s">
+      <c r="A69" s="149" t="s">
         <v>79</v>
       </c>
-      <c r="B69" s="151"/>
+      <c r="B69" s="150"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
@@ -5276,10 +5309,10 @@
       <c r="C84" s="36"/>
     </row>
     <row r="85" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="154" t="s">
+      <c r="A85" s="153" t="s">
         <v>188</v>
       </c>
-      <c r="B85" s="155"/>
+      <c r="B85" s="154"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
@@ -5422,10 +5455,10 @@
     </row>
     <row r="100" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="101" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="150" t="s">
+      <c r="A101" s="149" t="s">
         <v>111</v>
       </c>
-      <c r="B101" s="151"/>
+      <c r="B101" s="150"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="7" t="s">
@@ -5565,10 +5598,10 @@
     </row>
     <row r="117" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="118" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="150" t="s">
+      <c r="A118" s="149" t="s">
         <v>133</v>
       </c>
-      <c r="B118" s="151"/>
+      <c r="B118" s="150"/>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
@@ -5687,10 +5720,10 @@
     </row>
     <row r="132" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="133" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A133" s="150" t="s">
+      <c r="A133" s="149" t="s">
         <v>134</v>
       </c>
-      <c r="B133" s="151"/>
+      <c r="B133" s="150"/>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
@@ -5806,10 +5839,10 @@
     </row>
     <row r="146" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="147" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="150" t="s">
+      <c r="A147" s="149" t="s">
         <v>207</v>
       </c>
-      <c r="B147" s="151"/>
+      <c r="B147" s="150"/>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
@@ -5875,11 +5908,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="D15:E15"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A51:B51"/>
     <mergeCell ref="G12:H12"/>
@@ -5890,6 +5918,11 @@
     <mergeCell ref="A101:B101"/>
     <mergeCell ref="A118:B118"/>
     <mergeCell ref="A133:B133"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="D15:E15"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E16">
@@ -5928,18 +5961,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="150" t="s">
+      <c r="A1" s="149" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="151"/>
-      <c r="D1" s="150" t="s">
+      <c r="B1" s="150"/>
+      <c r="D1" s="149" t="s">
         <v>221</v>
       </c>
-      <c r="E1" s="151"/>
-      <c r="G1" s="150" t="s">
+      <c r="E1" s="150"/>
+      <c r="G1" s="149" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="151"/>
+      <c r="H1" s="150"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -6063,10 +6096,10 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="150" t="s">
+      <c r="A9" s="149" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="151"/>
+      <c r="B9" s="150"/>
       <c r="D9" t="s">
         <v>32</v>
       </c>
@@ -6265,10 +6298,10 @@
     </row>
     <row r="28" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="150" t="s">
+      <c r="A29" s="149" t="s">
         <v>16</v>
       </c>
-      <c r="B29" s="151"/>
+      <c r="B29" s="150"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -6287,10 +6320,10 @@
         <f>_Av*100*_fy/(1000*SQRT(3))</f>
         <v>1042.1194079466816</v>
       </c>
-      <c r="D31" s="152" t="s">
+      <c r="D31" s="151" t="s">
         <v>34</v>
       </c>
-      <c r="E31" s="153"/>
+      <c r="E31" s="152"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -6470,10 +6503,10 @@
     </row>
     <row r="46" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="150" t="s">
+      <c r="A47" s="149" t="s">
         <v>133</v>
       </c>
-      <c r="B47" s="151"/>
+      <c r="B47" s="150"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="107" t="s">
@@ -6641,10 +6674,10 @@
     </row>
     <row r="68" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="69" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="150" t="s">
+      <c r="A69" s="149" t="s">
         <v>134</v>
       </c>
-      <c r="B69" s="151"/>
+      <c r="B69" s="150"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
@@ -7006,7 +7039,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q186"/>
+  <dimension ref="A1:Q203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
@@ -7023,18 +7056,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="150" t="s">
+      <c r="A1" s="149" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="151"/>
-      <c r="D1" s="150" t="s">
+      <c r="B1" s="150"/>
+      <c r="D1" s="149" t="s">
         <v>221</v>
       </c>
-      <c r="E1" s="151"/>
-      <c r="G1" s="150" t="s">
+      <c r="E1" s="150"/>
+      <c r="G1" s="149" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="151"/>
+      <c r="H1" s="150"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -7256,10 +7289,10 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="150" t="s">
+      <c r="A13" s="149" t="s">
         <v>256</v>
       </c>
-      <c r="B13" s="151"/>
+      <c r="B13" s="150"/>
       <c r="D13" t="s">
         <v>38</v>
       </c>
@@ -7283,10 +7316,10 @@
         <f>(_bfi-2*_r-_tw)/2</f>
         <v>71.45</v>
       </c>
-      <c r="G14" s="150" t="s">
+      <c r="G14" s="149" t="s">
         <v>162</v>
       </c>
-      <c r="H14" s="151"/>
+      <c r="H14" s="150"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -7545,10 +7578,10 @@
     </row>
     <row r="32" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="150" t="s">
+      <c r="A33" s="149" t="s">
         <v>16</v>
       </c>
-      <c r="B33" s="151"/>
+      <c r="B33" s="150"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
@@ -7567,10 +7600,10 @@
         <f>_Av*100*_fy/(1000*SQRT(3))</f>
         <v>487.74585382155738</v>
       </c>
-      <c r="D35" s="152" t="s">
+      <c r="D35" s="151" t="s">
         <v>34</v>
       </c>
-      <c r="E35" s="153"/>
+      <c r="E35" s="152"/>
       <c r="G35" s="21" t="s">
         <v>44</v>
       </c>
@@ -7680,10 +7713,10 @@
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="J40" s="152" t="s">
+      <c r="J40" s="151" t="s">
         <v>276</v>
       </c>
-      <c r="K40" s="153"/>
+      <c r="K40" s="152"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
@@ -7742,10 +7775,10 @@
         <f>B45-300</f>
         <v>-178.04000000000002</v>
       </c>
-      <c r="J45" s="152" t="s">
+      <c r="J45" s="151" t="s">
         <v>277</v>
       </c>
-      <c r="K45" s="153"/>
+      <c r="K45" s="152"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
@@ -7793,10 +7826,10 @@
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="J49" s="152" t="s">
+      <c r="J49" s="151" t="s">
         <v>278</v>
       </c>
-      <c r="K49" s="153"/>
+      <c r="K49" s="152"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
@@ -7831,10 +7864,10 @@
         <f>IF(B47&gt;0.5,IF(B42&lt;=K41,1,IF(B42&lt;=K42,2,IF(B48&gt;-1,IF(B42&lt;=K50,3,4),IF(B42&lt;=K54,3,4)))),IF(B42&lt;=K46,1,IF(B42&lt;=K47,2,IF(B48&gt;-1,IF(B42&lt;=K50,3,4),IF(B42&lt;=K54,3,4)))))</f>
         <v>2</v>
       </c>
-      <c r="J52" s="152" t="s">
+      <c r="J52" s="151" t="s">
         <v>280</v>
       </c>
-      <c r="K52" s="153"/>
+      <c r="K52" s="152"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -7898,10 +7931,10 @@
       <c r="B62" s="70"/>
     </row>
     <row r="63" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="156" t="s">
+      <c r="A63" s="155" t="s">
         <v>188</v>
       </c>
-      <c r="B63" s="157"/>
+      <c r="B63" s="156"/>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
@@ -8047,10 +8080,10 @@
       <c r="B78" s="70"/>
     </row>
     <row r="79" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="150" t="s">
+      <c r="A79" s="149" t="s">
         <v>79</v>
       </c>
-      <c r="B79" s="151"/>
+      <c r="B79" s="150"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
@@ -8287,10 +8320,10 @@
     </row>
     <row r="95" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="96" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="150" t="s">
-        <v>369</v>
-      </c>
-      <c r="B96" s="151"/>
+      <c r="A96" s="149" t="s">
+        <v>368</v>
+      </c>
+      <c r="B96" s="150"/>
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
@@ -8751,10 +8784,10 @@
     </row>
     <row r="115" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="116" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="150" t="s">
+      <c r="A116" s="149" t="s">
         <v>338</v>
       </c>
-      <c r="B116" s="151"/>
+      <c r="B116" s="150"/>
     </row>
     <row r="117" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
@@ -9219,10 +9252,10 @@
     </row>
     <row r="135" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="136" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="150" t="s">
+      <c r="A136" s="149" t="s">
         <v>133</v>
       </c>
-      <c r="B136" s="151"/>
+      <c r="B136" s="150"/>
     </row>
     <row r="137" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
@@ -9433,10 +9466,10 @@
     </row>
     <row r="158" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="159" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A159" s="150" t="s">
+      <c r="A159" s="149" t="s">
         <v>134</v>
       </c>
-      <c r="B159" s="151"/>
+      <c r="B159" s="150"/>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="113"/>
@@ -9478,7 +9511,7 @@
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="28" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B163" s="147">
         <v>5921</v>
@@ -9496,7 +9529,7 @@
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="126" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B164" s="144">
         <v>-178</v>
@@ -9514,7 +9547,7 @@
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" s="28" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B165" s="147">
         <v>5921</v>
@@ -9532,7 +9565,7 @@
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="126" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B166" s="144">
         <v>-178</v>
@@ -9568,7 +9601,7 @@
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="142" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B168" s="143">
         <f>B139</f>
@@ -9747,142 +9780,336 @@
       </c>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A175" s="7" t="s">
-        <v>362</v>
-      </c>
-      <c r="B175" s="116">
+      <c r="A175" s="159" t="s">
+        <v>370</v>
+      </c>
+      <c r="B175" s="157">
         <f>ABS(IF(B167="N",0,_beff_appuis*1000*(_td-_tj)/B162*(B166-((_td-_tj)/2+_tj))))</f>
         <v>0</v>
       </c>
-      <c r="C175" s="116">
+      <c r="C175" s="157">
         <f>ABS(IF(C167="N",0,_beff_appuis*1000*(_td-_tj)/C162*(C166-((_td-_tj)/2+_tj))))</f>
         <v>568499.95572826616</v>
       </c>
-      <c r="D175" s="116">
+      <c r="D175" s="157">
         <f>ABS(IF(D167="N",0,_beff_appuis*1000*(_td-_tj)/D162*(D166-((_td-_tj)/2+_tj))))</f>
         <v>856207.67223048443</v>
       </c>
-      <c r="E175" s="116">
+      <c r="E175" s="157">
         <f>ABS(IF(E167="N",0,_beff_appuis*1000*(_td-_tj)/E162*(E166-((_td-_tj)/2+_tj))))</f>
         <v>601205.54820322257</v>
       </c>
+      <c r="F175" s="29"/>
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A176" s="7" t="s">
+      <c r="A176" s="160" t="s">
         <v>361</v>
       </c>
-      <c r="B176" s="149">
-        <f>B168*1000*B175/B165/1000</f>
+      <c r="B176" s="158">
+        <f>B168*B175/(B165*10^4)*1000</f>
         <v>0</v>
       </c>
-      <c r="C176" s="149">
-        <f t="shared" ref="C176:E176" si="23">C168*1000*C175/C165/1000</f>
-        <v>528.09792272631466</v>
-      </c>
-      <c r="D176" s="149">
-        <f t="shared" si="23"/>
-        <v>14.15962974203657</v>
-      </c>
-      <c r="E176" s="149">
-        <f t="shared" si="23"/>
+      <c r="C176" s="158">
+        <f>C168*C175/(C165*10^4)*1000</f>
+        <v>52.809792272631476</v>
+      </c>
+      <c r="D176" s="158">
+        <f>D168*D175/(D165*10^4)*1000</f>
+        <v>1.4159629742036572</v>
+      </c>
+      <c r="E176" s="158">
+        <f t="shared" ref="E176" si="23">E168*1000*E175/E165/1000</f>
         <v>0</v>
       </c>
-      <c r="F176">
+      <c r="F176" s="20">
         <f>1.35*B176+1.35*C176+1.5*D176+1.35*E176</f>
-        <v>734.17164029357969</v>
-      </c>
-    </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A177" s="7"/>
-      <c r="B177" s="113"/>
-    </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A178" t="s">
+        <v>73.417164029357977</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A177" s="159" t="s">
+        <v>372</v>
+      </c>
+      <c r="B177" s="161">
+        <f>ABS(_hw*_tw*(-_tfs-_hw/2-B166)+_bfi*_tfi*(-_h+_tfi/2-B166))</f>
+        <v>126176.34949999998</v>
+      </c>
+      <c r="C177" s="161">
+        <f>ABS(_hw*_tw*(-_tfs-_hw/2-C166)+_bfi*_tfi*(-_h+_tfi/2-C166))</f>
+        <v>645179.28789348458</v>
+      </c>
+      <c r="D177" s="161">
+        <f>ABS(_hw*_tw*(-_tfs-_hw/2-D166)+_bfi*_tfi*(-_h+_tfi/2-D166))</f>
+        <v>881640.03304708935</v>
+      </c>
+      <c r="E177" s="161">
+        <f>ABS(_hw*_tw*(-_tfs-_hw/2-E166)+_bfi*_tfi*(-_h+_tfi/2-E166))</f>
+        <v>645481.69507933129</v>
+      </c>
+      <c r="F177" s="74"/>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A178" s="160" t="s">
+        <v>371</v>
+      </c>
+      <c r="B178" s="158">
+        <f>B168*B177/(B165*10^4)*1000</f>
+        <v>66.273397384977841</v>
+      </c>
+      <c r="C178" s="158">
+        <f t="shared" ref="C178:E178" si="24">C168*C177/(C165*10^4)*1000</f>
+        <v>59.932782454859115</v>
+      </c>
+      <c r="D178" s="158">
+        <f t="shared" si="24"/>
+        <v>1.4580220241641513</v>
+      </c>
+      <c r="E178" s="158">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="F178" s="20">
+        <f>1.35*B178+1.35*C178+1.5*D178+1.35*E178</f>
+        <v>172.56537582002613</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A179" s="159" t="s">
+        <v>377</v>
+      </c>
+      <c r="B179" s="161">
+        <f>ABS(_bfi*_tfi*(-_h+_tfi/2-B166))</f>
+        <v>187223.24999999997</v>
+      </c>
+      <c r="C179" s="161">
+        <f>ABS(_bfi*_tfi*(-_h+_tfi/2-C166))</f>
+        <v>417560.82493482315</v>
+      </c>
+      <c r="D179" s="161">
+        <f>ABS(_bfi*_tfi*(-_h+_tfi/2-D166))</f>
+        <v>522503.9583485864</v>
+      </c>
+      <c r="E179" s="161">
+        <f>ABS(_bfi*_tfi*(-_h+_tfi/2-E166))</f>
+        <v>417695.03561587719</v>
+      </c>
+      <c r="F179" s="74"/>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A180" s="160" t="s">
+        <v>371</v>
+      </c>
+      <c r="B180" s="158">
+        <f>B168*B179/(B165*10^4)*1000</f>
+        <v>98.33792859062747</v>
+      </c>
+      <c r="C180" s="158">
+        <f t="shared" ref="C180:E180" si="25">C168*C179/(C165*10^4)*1000</f>
+        <v>38.788570172794898</v>
+      </c>
+      <c r="D180" s="158">
+        <f t="shared" si="25"/>
+        <v>0.86409674065299358</v>
+      </c>
+      <c r="E180" s="158">
+        <f t="shared" si="25"/>
+        <v>0</v>
+      </c>
+      <c r="F180" s="20">
+        <f>1.35*B180+1.35*C180+1.5*D180+1.35*E180</f>
+        <v>186.41691844159968</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A181" s="7"/>
+      <c r="B181" s="113"/>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
         <v>245</v>
       </c>
-      <c r="B178" s="23">
+      <c r="B182" s="23">
         <f>_Av*100*_fy/(1000*SQRT(3))</f>
         <v>487.74585382155738</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A179" s="115" t="s">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A183" s="115" t="s">
         <v>123</v>
       </c>
-      <c r="B179" s="23">
+      <c r="B183" s="23">
         <v>464.72471483007769</v>
       </c>
-      <c r="C179">
-        <f>B179*B180</f>
+      <c r="C183">
+        <f>B183*B184</f>
         <v>464.72471483007769</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A180" s="115" t="s">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A184" s="115" t="s">
         <v>359</v>
       </c>
-      <c r="B180" s="25">
+      <c r="B184" s="25">
         <v>1</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A181" s="115" t="s">
-        <v>364</v>
-      </c>
-      <c r="B181" s="25">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A185" s="115" t="s">
+        <v>363</v>
+      </c>
+      <c r="B185" s="3">
         <f>_PRd/(_sx/1000)</f>
         <v>341.22561783575122</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B182" s="23"/>
-    </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A183" t="s">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A186" s="115" t="s">
+        <v>373</v>
+      </c>
+      <c r="B186" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A187" s="115" t="s">
+        <v>374</v>
+      </c>
+      <c r="B187" s="3">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B188" s="23"/>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A189" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="B183" s="26">
+      <c r="B189" s="69">
         <f>MAX(F172:F174)</f>
         <v>0.90844871009293149</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A184" t="s">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A190" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="B184" s="26">
-        <f>B154/B178</f>
+      <c r="B190" s="17">
+        <f>B154/B182</f>
         <v>0.14297324672017361</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A185" t="s">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A191" s="15" t="s">
         <v>358</v>
       </c>
-      <c r="B185" s="26">
-        <f>B155/(B180*B179)</f>
+      <c r="B191" s="17">
+        <f>B155/(B184*B183)</f>
         <v>0.52140015676004936</v>
       </c>
-      <c r="C185" t="s">
+      <c r="C191" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A186" t="s">
-        <v>370</v>
-      </c>
-      <c r="B186" s="26">
-        <f>F176/B181</f>
-        <v>2.1515724550522255</v>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A192" s="15" t="s">
+        <v>369</v>
+      </c>
+      <c r="B192" s="17">
+        <f>F176/B185</f>
+        <v>0.21515724550522256</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A193" s="15" t="s">
+        <v>375</v>
+      </c>
+      <c r="B193" s="17">
+        <f>SQRT(3)/2*F178*B186*1.25/B187</f>
+        <v>0.35924519056190274</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A194" s="16" t="s">
+        <v>376</v>
+      </c>
+      <c r="B194" s="18">
+        <f>SQRT(3)/2*F180*B186*1.25/B187</f>
+        <v>0.38808121890778152</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="196" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A196" s="149" t="s">
+        <v>207</v>
+      </c>
+      <c r="B196" s="150"/>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>209</v>
+      </c>
+      <c r="B197" s="3">
+        <f>_nr*_PRd/(_sx/1000)</f>
+        <v>341.22561783575122</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>208</v>
+      </c>
+      <c r="B198" s="3">
+        <f>B197/(_td-_tj)</f>
+        <v>3.1020510712341021</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>210</v>
+      </c>
+      <c r="B199" s="33">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>212</v>
+      </c>
+      <c r="B200" s="3">
+        <f>0.6*(1-_fck_dalle/250)</f>
+        <v>0.55200000000000005</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>211</v>
+      </c>
+      <c r="B201" s="3">
+        <f>B200*_fck_dalle/1.5*SIN(RADIANS(B199))*COS(RADIANS(B199))</f>
+        <v>2.9771825392998066</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>213</v>
+      </c>
+      <c r="B202" s="3">
+        <f>B198/B201</f>
+        <v>1.0419418461199437</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>214</v>
+      </c>
+      <c r="B203" s="3">
+        <f>B198*(_td-_tj)*TAN(RADIANS(B199))/(500/1.15)*10</f>
+        <v>3.9988521350558321</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="J49:K49"/>
-    <mergeCell ref="J52:K52"/>
-    <mergeCell ref="A136:B136"/>
+  <mergeCells count="18">
+    <mergeCell ref="A196:B196"/>
     <mergeCell ref="A159:B159"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="D1:E1"/>
@@ -9895,6 +10122,11 @@
     <mergeCell ref="A79:B79"/>
     <mergeCell ref="A96:B96"/>
     <mergeCell ref="A116:B116"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="J49:K49"/>
+    <mergeCell ref="J52:K52"/>
+    <mergeCell ref="A136:B136"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>